<commit_message>
chat-sift: batches b20-b29 read; index, extracts and progress updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aq7txTcfpUgzabiqqnXaKj
</commit_message>
<xml_diff>
--- a/chat-sift/output/index.xlsx
+++ b/chat-sift/output/index.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$150</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$247</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H150"/>
+  <dimension ref="A1:H247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5995,8 +5995,3612 @@
         <v>0</v>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-19</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>CCD gain calibration explanation</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-19_1408_CCD-gain-calibration-explanation.md</t>
+        </is>
+      </c>
+      <c r="E151" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G151" s="3" t="inlineStr">
+        <is>
+          <t>Technical investigation of a CCD front-end gain calibration, clamp, op-amp failures and protection, with a failure analysis report, apparently a professional electronics task.</t>
+        </is>
+      </c>
+      <c r="H151" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-20</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>New chat</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-20_0643_New-chat-2.md</t>
+        </is>
+      </c>
+      <c r="E152" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr"/>
+      <c r="G152" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-20</t>
+        </is>
+      </c>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>New chat</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-20_0643_New-chat.md</t>
+        </is>
+      </c>
+      <c r="E153" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr"/>
+      <c r="G153" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-20</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>Investigation report options</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-20_0644_Investigation-report-options.md</t>
+        </is>
+      </c>
+      <c r="E154" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G154" s="3" t="inlineStr">
+        <is>
+          <t>Drafting an engineering failure-analysis report on a CCD front-end and gain-calibration circuit, apparently a professional electronics task.</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-20</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>Imo3 relay configs</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-20_0805_Imo3-relay-configs.md</t>
+        </is>
+      </c>
+      <c r="E155" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G155" s="3" t="inlineStr">
+        <is>
+          <t>Relay variant and wiring question for a gain-calibration circuit, apparently a professional electronics task.</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-20</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>How LTC2757 works</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-20_1749_How-LTC2757-works.md</t>
+        </is>
+      </c>
+      <c r="E156" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G156" s="3" t="inlineStr">
+        <is>
+          <t>Explanation and redraw of an LTC2757 DAC schematic, apparently a professional electronics task.</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>Portable 2-in-1 laptops</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-22_0825_Portable-2-in-1-laptops.md</t>
+        </is>
+      </c>
+      <c r="E157" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F157" s="2" t="inlineStr"/>
+      <c r="G157" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H157" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>OmniBook X vs 5</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-22_0954_OmniBook-X-vs-5.md</t>
+        </is>
+      </c>
+      <c r="E158" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr"/>
+      <c r="G158" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H158" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>Yoga 7 vs Omni X</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-22_1233_Yoga-7-vs-Omni-X.md</t>
+        </is>
+      </c>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F159" s="2" t="inlineStr"/>
+      <c r="G159" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H159" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-23</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>Circuit function explanation</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-23_1857_Circuit-function-explanation.md</t>
+        </is>
+      </c>
+      <c r="E160" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G160" s="3" t="inlineStr">
+        <is>
+          <t>Fault-finding and protection/filter design on an op-amp stage of an electronics board (possibly professional engineering work).</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-26</t>
+        </is>
+      </c>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>Identify slow-blow fuse</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-26_1029_Identify-slow-blow-fuse.md</t>
+        </is>
+      </c>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F161" s="2" t="inlineStr"/>
+      <c r="G161" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H161" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-26</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>Autumn Budget impact 2025</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-26_1744_Autumn-Budget-impact-2025.md</t>
+        </is>
+      </c>
+      <c r="E162" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G162" s="3" t="inlineStr">
+        <is>
+          <t>Effect of the Budget on the owner's salary, and take-home pay if working hours were reduced.</t>
+        </is>
+      </c>
+      <c r="H162" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-27</t>
+        </is>
+      </c>
+      <c r="B163" s="3" t="inlineStr">
+        <is>
+          <t>Why statement is not wrong</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-27_1317_Why-statement-is-not-wrong.md</t>
+        </is>
+      </c>
+      <c r="E163" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr"/>
+      <c r="G163" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-27</t>
+        </is>
+      </c>
+      <c r="B164" s="3" t="inlineStr">
+        <is>
+          <t>Ngai Ombibook meaning</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-27_1704_Ngai-Ombibook-meaning.md</t>
+        </is>
+      </c>
+      <c r="E164" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr"/>
+      <c r="G164" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H164" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-28</t>
+        </is>
+      </c>
+      <c r="B165" s="3" t="inlineStr">
+        <is>
+          <t>Replacement brake pads i9 Max</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-28_1701_Replacement-brake-pads-i9-Max.md</t>
+        </is>
+      </c>
+      <c r="E165" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr"/>
+      <c r="G165" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H165" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-28</t>
+        </is>
+      </c>
+      <c r="B166" s="3" t="inlineStr">
+        <is>
+          <t>Stylus price comparison</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-28_1940_Stylus-price-comparison.md</t>
+        </is>
+      </c>
+      <c r="E166" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr"/>
+      <c r="G166" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H166" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-29</t>
+        </is>
+      </c>
+      <c r="B167" s="3" t="inlineStr">
+        <is>
+          <t>Grouping Sonos speakers effects</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-29_0445_Grouping-Sonos-speakers-effects.md</t>
+        </is>
+      </c>
+      <c r="E167" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr"/>
+      <c r="G167" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H167" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-29</t>
+        </is>
+      </c>
+      <c r="B168" s="3" t="inlineStr">
+        <is>
+          <t>Remove iMac password</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-29_0622_Remove-iMac-password.md</t>
+        </is>
+      </c>
+      <c r="E168" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr"/>
+      <c r="G168" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H168" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-29</t>
+        </is>
+      </c>
+      <c r="B169" s="3" t="inlineStr">
+        <is>
+          <t>Shotgun personality traits</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-29_1255_Shotgun-personality-traits.md</t>
+        </is>
+      </c>
+      <c r="E169" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr"/>
+      <c r="G169" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H169" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-29</t>
+        </is>
+      </c>
+      <c r="B170" s="3" t="inlineStr">
+        <is>
+          <t>Ludacris in Heat film</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-29_1634_Ludacris-in-Heat-film.md</t>
+        </is>
+      </c>
+      <c r="E170" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr"/>
+      <c r="G170" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H170" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B171" s="3" t="inlineStr">
+        <is>
+          <t>Reeves budget misleading claims</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-01_0936_Reeves-budget-misleading-claims.md</t>
+        </is>
+      </c>
+      <c r="E171" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr"/>
+      <c r="G171" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H171" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
+        <is>
+          <t>Extra ground loop transients</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-02_0828_Extra-ground-loop-transients.md</t>
+        </is>
+      </c>
+      <c r="E172" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G172" s="3" t="inlineStr">
+        <is>
+          <t>Ground loops and transients in the context of the CCD amplifier board being worked on (possibly professional engineering work).</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B173" s="3" t="inlineStr">
+        <is>
+          <t>Soft-start options for DC rails</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-02_1211_Soft-start-options-for-DC-rails.md</t>
+        </is>
+      </c>
+      <c r="E173" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G173" s="3" t="inlineStr">
+        <is>
+          <t>Soft-start design for 32V and +/-18V DC rails (possibly professional engineering work).</t>
+        </is>
+      </c>
+      <c r="H173" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>CCTV operators and commission</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-02_1312_CCTV-operators-and-commission.md</t>
+        </is>
+      </c>
+      <c r="E174" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F174" s="2" t="inlineStr"/>
+      <c r="G174" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H174" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B175" s="3" t="inlineStr">
+        <is>
+          <t>Op amp fault explanation</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-03_0831_Op-amp-fault-explanation.md</t>
+        </is>
+      </c>
+      <c r="E175" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G175" s="3" t="inlineStr">
+        <is>
+          <t>Fault-finding an op-amp input fault by comparing a good and a faulty circuit board (possibly professional engineering work).</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>Rachel Reeves update</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-03_1838_Rachel-Reeves-update.md</t>
+        </is>
+      </c>
+      <c r="E176" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr"/>
+      <c r="G176" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B177" s="3" t="inlineStr">
+        <is>
+          <t>Modify pink vest</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-03_2236_Modify-pink-vest.md</t>
+        </is>
+      </c>
+      <c r="E177" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F177" s="2" t="inlineStr"/>
+      <c r="G177" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>Example request clarification</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-04_0759_Example-request-clarification.md</t>
+        </is>
+      </c>
+      <c r="E178" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G178" s="3" t="inlineStr">
+        <is>
+          <t>Rewriting assessment answers that describe workplace communication, work tasks, the engineering lifecycle process and its owner, preferred job type and workplace support needs.</t>
+        </is>
+      </c>
+      <c r="H178" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>Drive dirty meaning</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-04_1742_Drive-dirty-meaning.md</t>
+        </is>
+      </c>
+      <c r="E179" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr"/>
+      <c r="G179" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B180" s="3" t="inlineStr">
+        <is>
+          <t>Sleeping with hoop earrings</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-04_2025_Sleeping-with-hoop-earrings.md</t>
+        </is>
+      </c>
+      <c r="E180" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr"/>
+      <c r="G180" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B181" s="3" t="inlineStr">
+        <is>
+          <t>Rhymes for reckoner</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-04_2156_Rhymes-for-reckoner.md</t>
+        </is>
+      </c>
+      <c r="E181" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr"/>
+      <c r="G181" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B182" s="3" t="inlineStr">
+        <is>
+          <t>Tattoo extension concept</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-04_2228_Tattoo-extension-concept.md</t>
+        </is>
+      </c>
+      <c r="E182" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr"/>
+      <c r="G182" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>Refine concept directions</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-04_2302_Refine-concept-directions.md</t>
+        </is>
+      </c>
+      <c r="E183" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F183" s="2" t="inlineStr"/>
+      <c r="G183" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H183" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B184" s="3" t="inlineStr">
+        <is>
+          <t>Colouring words request</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-04_2333_Colouring-words-request.md</t>
+        </is>
+      </c>
+      <c r="E184" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="inlineStr"/>
+      <c r="G184" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>Forearm tattoo design</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-04_2343_Forearm-tattoo-design.md</t>
+        </is>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F185" s="2" t="inlineStr"/>
+      <c r="G185" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>Forearm tattoo design</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_0005_Forearm-tattoo-design.md</t>
+        </is>
+      </c>
+      <c r="E186" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr"/>
+      <c r="G186" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H186" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B187" s="3" t="inlineStr">
+        <is>
+          <t>Tattoo design concept</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_0105_Tattoo-design-concept.md</t>
+        </is>
+      </c>
+      <c r="E187" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="inlineStr"/>
+      <c r="G187" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B188" s="3" t="inlineStr">
+        <is>
+          <t>Forearm tattoo mock-up</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_0107_Forearm-tattoo-mock-up.md</t>
+        </is>
+      </c>
+      <c r="E188" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr"/>
+      <c r="G188" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H188" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>Tattoo design modification</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_0123_Tattoo-design-modification.md</t>
+        </is>
+      </c>
+      <c r="E189" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="inlineStr"/>
+      <c r="G189" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H189" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B190" s="3" t="inlineStr">
+        <is>
+          <t>Tattoo design feedback</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_0157_Tattoo-design-feedback.md</t>
+        </is>
+      </c>
+      <c r="E190" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr"/>
+      <c r="G190" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B191" s="3" t="inlineStr">
+        <is>
+          <t>Feedback on design</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_0227_Feedback-on-design.md</t>
+        </is>
+      </c>
+      <c r="E191" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="inlineStr"/>
+      <c r="G191" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B192" s="3" t="inlineStr">
+        <is>
+          <t>January sale likelihood</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_0726_January-sale-likelihood.md</t>
+        </is>
+      </c>
+      <c r="E192" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="inlineStr"/>
+      <c r="G192" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B193" s="3" t="inlineStr">
+        <is>
+          <t>Forearm mount questions</t>
+        </is>
+      </c>
+      <c r="C193" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_1206_Forearm-mount-questions.md</t>
+        </is>
+      </c>
+      <c r="E193" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F193" s="2" t="inlineStr"/>
+      <c r="G193" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B194" s="3" t="inlineStr">
+        <is>
+          <t>Extract art from mask</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_1320_Extract-art-from-mask.md</t>
+        </is>
+      </c>
+      <c r="E194" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="inlineStr"/>
+      <c r="G194" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H194" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>Tattoo design request</t>
+        </is>
+      </c>
+      <c r="C195" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_1332_Tattoo-design-request.md</t>
+        </is>
+      </c>
+      <c r="E195" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F195" s="2" t="inlineStr"/>
+      <c r="G195" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H195" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B196" s="3" t="inlineStr">
+        <is>
+          <t>Tattoo design request</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_1400_Tattoo-design-request.md</t>
+        </is>
+      </c>
+      <c r="E196" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F196" s="2" t="inlineStr"/>
+      <c r="G196" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H196" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t>Colour block options</t>
+        </is>
+      </c>
+      <c r="C197" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_1401_Colour-block-options.md</t>
+        </is>
+      </c>
+      <c r="E197" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F197" s="2" t="inlineStr"/>
+      <c r="G197" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H197" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B198" s="3" t="inlineStr">
+        <is>
+          <t>Original reference guide</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_1401_Original-reference-guide.md</t>
+        </is>
+      </c>
+      <c r="E198" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr"/>
+      <c r="G198" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B199" s="3" t="inlineStr">
+        <is>
+          <t>User feedback</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_1443_User-feedback.md</t>
+        </is>
+      </c>
+      <c r="E199" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F199" s="2" t="inlineStr"/>
+      <c r="G199" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H199" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B200" s="3" t="inlineStr">
+        <is>
+          <t>Baseline replication request</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_1504_Baseline-replication-request.md</t>
+        </is>
+      </c>
+      <c r="E200" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="inlineStr"/>
+      <c r="G200" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B201" s="3" t="inlineStr">
+        <is>
+          <t>Add men to design</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-001.json</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_1511_Add-men-to-design.md</t>
+        </is>
+      </c>
+      <c r="E201" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="inlineStr"/>
+      <c r="G201" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H201" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B202" s="3" t="inlineStr">
+        <is>
+          <t>Circuit analysis feedback</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_1808_Circuit-analysis-feedback.md</t>
+        </is>
+      </c>
+      <c r="E202" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G202" s="3" t="inlineStr">
+        <is>
+          <t>Checking a resistor circuit to run a 12 V fan from ±9 V rails; possibly a technical project connected to the owner's job.</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="B203" s="3" t="inlineStr">
+        <is>
+          <t>Texting opener review</t>
+        </is>
+      </c>
+      <c r="C203" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-05_1835_Texting-opener-review.md</t>
+        </is>
+      </c>
+      <c r="E203" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="inlineStr"/>
+      <c r="G203" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H203" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-06</t>
+        </is>
+      </c>
+      <c r="B204" s="3" t="inlineStr">
+        <is>
+          <t>Near Wild Heaven</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-06_0744_Near-Wild-Heaven.md</t>
+        </is>
+      </c>
+      <c r="E204" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr"/>
+      <c r="G204" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H204" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-07</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>Upgrade noisy fan</t>
+        </is>
+      </c>
+      <c r="C205" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-07_0452_Upgrade-noisy-fan.md</t>
+        </is>
+      </c>
+      <c r="E205" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F205" s="2" t="inlineStr"/>
+      <c r="G205" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H205" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-07</t>
+        </is>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>Thermal pad connection LT3091</t>
+        </is>
+      </c>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-07_1620_Thermal-pad-connection-LT3091.md</t>
+        </is>
+      </c>
+      <c r="E206" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G206" s="3" t="inlineStr">
+        <is>
+          <t>PCB layout question about connecting the LT3091 regulator thermal pad; possibly a technical project connected to the owner's job.</t>
+        </is>
+      </c>
+      <c r="H206" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-07</t>
+        </is>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>Tattoo and parental approval</t>
+        </is>
+      </c>
+      <c r="C207" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-07_2044_Tattoo-and-parental-approval.md</t>
+        </is>
+      </c>
+      <c r="E207" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F207" s="2" t="inlineStr"/>
+      <c r="G207" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H207" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-07</t>
+        </is>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>ASD support levels explained</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-07_2106_ASD-support-levels-explained.md</t>
+        </is>
+      </c>
+      <c r="E208" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F208" s="2" t="inlineStr"/>
+      <c r="G208" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H208" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-09</t>
+        </is>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>Coping with unsupportive parents</t>
+        </is>
+      </c>
+      <c r="C209" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-09_1005_Coping-with-unsupportive-parents.md</t>
+        </is>
+      </c>
+      <c r="E209" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F209" s="2" t="inlineStr"/>
+      <c r="G209" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H209" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-09</t>
+        </is>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>Trauma therapy and child baseline</t>
+        </is>
+      </c>
+      <c r="C210" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-09_1508_Trauma-therapy-and-child-baseline.md</t>
+        </is>
+      </c>
+      <c r="E210" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G210" s="3" t="inlineStr">
+        <is>
+          <t>A drafted reply mentions the owner's work as one suggested cause of change.</t>
+        </is>
+      </c>
+      <c r="H210" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-09</t>
+        </is>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>Power supply overcurrent causes</t>
+        </is>
+      </c>
+      <c r="C211" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-09_1652_Power-supply-overcurrent-causes.md</t>
+        </is>
+      </c>
+      <c r="E211" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F211" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G211" s="3" t="inlineStr">
+        <is>
+          <t>Troubleshooting overcurrent and wiring a ±9 V supply on modular bench power supply equipment; possibly job-related test work.</t>
+        </is>
+      </c>
+      <c r="H211" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="B212" s="3" t="inlineStr">
+        <is>
+          <t>Improve my answers</t>
+        </is>
+      </c>
+      <c r="C212" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-10_0341_Improve-my-answers.md</t>
+        </is>
+      </c>
+      <c r="E212" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F212" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G212" s="3" t="inlineStr">
+        <is>
+          <t>Assessment answers referencing workplace behaviour, a former manager, masking at work, current engineering role difficulties with a process owner, a 20-year career and step back from team leadership, and workplace support needs.</t>
+        </is>
+      </c>
+      <c r="H212" s="2" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="B213" s="3" t="inlineStr">
+        <is>
+          <t>Autistic traits identified</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-11_0838_Autistic-traits-identified.md</t>
+        </is>
+      </c>
+      <c r="E213" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F213" s="2" t="inlineStr"/>
+      <c r="G213" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H213" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="B214" s="3" t="inlineStr">
+        <is>
+          <t>Handling team leader conflict</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-11_1643_Handling-team-leader-conflict.md</t>
+        </is>
+      </c>
+      <c r="E214" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F214" s="2" t="inlineStr"/>
+      <c r="G214" s="3" t="inlineStr">
+        <is>
+          <t>Being ignored by the team leader who replaced the owner after they stepped down from the team leader role on medical grounds, and returning to the role.</t>
+        </is>
+      </c>
+      <c r="H214" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-13</t>
+        </is>
+      </c>
+      <c r="B215" s="3" t="inlineStr">
+        <is>
+          <t>Check Office 365 Version</t>
+        </is>
+      </c>
+      <c r="C215" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-13_0615_Check-Office-365-Version.md</t>
+        </is>
+      </c>
+      <c r="E215" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F215" s="2" t="inlineStr"/>
+      <c r="G215" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H215" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-13</t>
+        </is>
+      </c>
+      <c r="B216" s="3" t="inlineStr">
+        <is>
+          <t>RAM upgrade for OptiPlex</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-13_0738_RAM-upgrade-for-OptiPlex.md</t>
+        </is>
+      </c>
+      <c r="E216" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F216" s="2" t="inlineStr"/>
+      <c r="G216" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H216" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-13</t>
+        </is>
+      </c>
+      <c r="B217" s="3" t="inlineStr">
+        <is>
+          <t>Enable Copilot in Outlook</t>
+        </is>
+      </c>
+      <c r="C217" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-13_0837_Enable-Copilot-in-Outlook.md</t>
+        </is>
+      </c>
+      <c r="E217" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F217" s="2" t="inlineStr"/>
+      <c r="G217" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H217" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B218" s="3" t="inlineStr">
+        <is>
+          <t>Redraw house in blueprint style</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14_0630_Redraw-house-in-blueprint-style.md</t>
+        </is>
+      </c>
+      <c r="E218" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F218" s="2" t="inlineStr"/>
+      <c r="G218" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H218" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B219" s="3" t="inlineStr">
+        <is>
+          <t>Recreate symbol</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14_0707_Recreate-symbol.md</t>
+        </is>
+      </c>
+      <c r="E219" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F219" s="2" t="inlineStr"/>
+      <c r="G219" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H219" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B220" s="3" t="inlineStr">
+        <is>
+          <t>Cryptic tree creation</t>
+        </is>
+      </c>
+      <c r="C220" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14_0729_Cryptic-tree-creation.md</t>
+        </is>
+      </c>
+      <c r="E220" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F220" s="2" t="inlineStr"/>
+      <c r="G220" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H220" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B221" s="3" t="inlineStr">
+        <is>
+          <t>Helicopter graphic idea</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14_1510_Helicopter-graphic-idea.md</t>
+        </is>
+      </c>
+      <c r="E221" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F221" s="2" t="inlineStr"/>
+      <c r="G221" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H221" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B222" s="3" t="inlineStr">
+        <is>
+          <t>Merge plan summary</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14_1925_Merge-plan-summary.md</t>
+        </is>
+      </c>
+      <c r="E222" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F222" s="2" t="inlineStr"/>
+      <c r="G222" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H222" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B223" s="3" t="inlineStr">
+        <is>
+          <t>Arrange and merge plan</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14_1952_Arrange-and-merge-plan.md</t>
+        </is>
+      </c>
+      <c r="E223" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F223" s="2" t="inlineStr"/>
+      <c r="G223" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H223" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B224" s="3" t="inlineStr">
+        <is>
+          <t>Replace cross with image</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14_1957_Replace-cross-with-image.md</t>
+        </is>
+      </c>
+      <c r="E224" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F224" s="2" t="inlineStr"/>
+      <c r="G224" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H224" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B225" s="3" t="inlineStr">
+        <is>
+          <t>Childhood details in therapy</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14_2020_Childhood-details-in-therapy.md</t>
+        </is>
+      </c>
+      <c r="E225" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="inlineStr"/>
+      <c r="G225" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H225" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B226" s="3" t="inlineStr">
+        <is>
+          <t>Graphic integration options</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14_2030_Graphic-integration-options.md</t>
+        </is>
+      </c>
+      <c r="E226" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F226" s="2" t="inlineStr"/>
+      <c r="G226" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H226" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B227" s="3" t="inlineStr">
+        <is>
+          <t>Sign design request</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14_2056_Sign-design-request.md</t>
+        </is>
+      </c>
+      <c r="E227" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F227" s="2" t="inlineStr"/>
+      <c r="G227" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H227" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B228" s="3" t="inlineStr">
+        <is>
+          <t>Add sign above cross</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-14_2102_Add-sign-above-cross.md</t>
+        </is>
+      </c>
+      <c r="E228" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F228" s="2" t="inlineStr"/>
+      <c r="G228" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H228" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="B229" s="3" t="inlineStr">
+        <is>
+          <t>Key sight n6743b current</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-15_1028_Key-sight-n6743b-current.md</t>
+        </is>
+      </c>
+      <c r="E229" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F229" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G229" s="3" t="inlineStr">
+        <is>
+          <t>Technical query about the current rating of a Keysight power supply module, possibly for professional lab work.</t>
+        </is>
+      </c>
+      <c r="H229" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-17</t>
+        </is>
+      </c>
+      <c r="B230" s="3" t="inlineStr">
+        <is>
+          <t>Mains load estimation</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-17_1001_Mains-load-estimation.md</t>
+        </is>
+      </c>
+      <c r="E230" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F230" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G230" s="3" t="inlineStr">
+        <is>
+          <t>Technical queries about mains load and module specifications for Keysight power mainframes, possibly for professional lab work.</t>
+        </is>
+      </c>
+      <c r="H230" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-17</t>
+        </is>
+      </c>
+      <c r="B231" s="3" t="inlineStr">
+        <is>
+          <t>Sharing psychological notes</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-17_1911_Sharing-psychological-notes.md</t>
+        </is>
+      </c>
+      <c r="E231" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F231" s="2" t="inlineStr"/>
+      <c r="G231" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H231" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-17</t>
+        </is>
+      </c>
+      <c r="B232" s="3" t="inlineStr">
+        <is>
+          <t>Reasonable adjustments delay</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-17_2157_Reasonable-adjustments-delay.md</t>
+        </is>
+      </c>
+      <c r="E232" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F232" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G232" s="3" t="inlineStr">
+        <is>
+          <t>Reasonable adjustment request, manager relationship, HR, internal role move email, phased return meeting and sickness absence recording.</t>
+        </is>
+      </c>
+      <c r="H232" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B233" s="3" t="inlineStr">
+        <is>
+          <t>Draw trapezoid diagram</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-18_0754_Draw-trapezoid-diagram.md</t>
+        </is>
+      </c>
+      <c r="E233" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F233" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G233" s="3" t="inlineStr">
+        <is>
+          <t>Electronics and hardware design questions (DAC/ADC, PoE, racks, CAD) possibly for professional work.</t>
+        </is>
+      </c>
+      <c r="H233" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B234" s="3" t="inlineStr">
+        <is>
+          <t>Altium AI usage</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-18_0852_Altium-AI-usage.md</t>
+        </is>
+      </c>
+      <c r="E234" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F234" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G234" s="3" t="inlineStr">
+        <is>
+          <t>Questions about EDA tools and AI-assisted circuit design possibly for professional work.</t>
+        </is>
+      </c>
+      <c r="H234" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B235" s="3" t="inlineStr">
+        <is>
+          <t>Balanced rewrite suggestion</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-18_1211_Balanced-rewrite-suggestion.md</t>
+        </is>
+      </c>
+      <c r="E235" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F235" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G235" s="3" t="inlineStr">
+        <is>
+          <t>Drafting a message about role clarity on the Arakkhs work, colleagues and a doctor's note, plus work technical questions and the owner's reading of the manager's intentions.</t>
+        </is>
+      </c>
+      <c r="H235" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B236" s="3" t="inlineStr">
+        <is>
+          <t>Card pull components</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-18_1234_Card-pull-components.md</t>
+        </is>
+      </c>
+      <c r="E236" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F236" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G236" s="3" t="inlineStr">
+        <is>
+          <t>Engineering question about card pull handles for backplane cards.</t>
+        </is>
+      </c>
+      <c r="H236" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B237" s="3" t="inlineStr">
+        <is>
+          <t>Bold text advice</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-18_1324_Bold-text-advice.md</t>
+        </is>
+      </c>
+      <c r="E237" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F237" s="2" t="inlineStr"/>
+      <c r="G237" s="3" t="inlineStr">
+        <is>
+          <t>Formatting advice on a written message to senior colleagues about the owner's role and contribution.</t>
+        </is>
+      </c>
+      <c r="H237" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B238" s="3" t="inlineStr">
+        <is>
+          <t>System name suggestions</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-18_1442_System-name-suggestions.md</t>
+        </is>
+      </c>
+      <c r="E238" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F238" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G238" s="3" t="inlineStr">
+        <is>
+          <t>Naming, scope document and proposal for a burn-in test system project related to the owner's department.</t>
+        </is>
+      </c>
+      <c r="H238" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
+      <c r="B239" s="3" t="inlineStr">
+        <is>
+          <t>Ribbon cable for 5MHz</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-19_0618_Ribbon-cable-for-5MHz.md</t>
+        </is>
+      </c>
+      <c r="E239" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F239" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G239" s="3" t="inlineStr">
+        <is>
+          <t>Engineering questions on LVDS signalling over cable from a Kintex-7 FPGA to an imaging sensor.</t>
+        </is>
+      </c>
+      <c r="H239" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
+      <c r="B240" s="3" t="inlineStr">
+        <is>
+          <t>Tidy and rewrite document</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-19_0702_Tidy-and-rewrite-document.md</t>
+        </is>
+      </c>
+      <c r="E240" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F240" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G240" s="3" t="inlineStr">
+        <is>
+          <t>Brief references to a lack of acknowledgement from the team leader about leave and to taking an afternoon off work.</t>
+        </is>
+      </c>
+      <c r="H240" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
+      <c r="B241" s="3" t="inlineStr">
+        <is>
+          <t>Unanswered messages and politics</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-19_0807_Unanswered-messages-and-politics.md</t>
+        </is>
+      </c>
+      <c r="E241" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F241" s="2" t="inlineStr"/>
+      <c r="G241" s="3" t="inlineStr">
+        <is>
+          <t>No reply from two senior colleagues to the owner's message and workplace politics.</t>
+        </is>
+      </c>
+      <c r="H241" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
+      <c r="B242" s="3" t="inlineStr">
+        <is>
+          <t>Circuit negative current sensing</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-19_1403_Circuit-negative-current-sensing.md</t>
+        </is>
+      </c>
+      <c r="E242" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G242" s="3" t="inlineStr">
+        <is>
+          <t>Technical discussion of a current-sense circuit schematic, apparently a professional electronics design task.</t>
+        </is>
+      </c>
+      <c r="H242" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
+      <c r="B243" s="3" t="inlineStr">
+        <is>
+          <t>Treatment log rewrite</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-19_1714_Treatment-log-rewrite.md</t>
+        </is>
+      </c>
+      <c r="E243" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="inlineStr"/>
+      <c r="G243" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H243" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="B244" s="3" t="inlineStr">
+        <is>
+          <t>ADC channel selection via bus</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20_0350_ADC-channel-selection-via-bus.md</t>
+        </is>
+      </c>
+      <c r="E244" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G244" s="3" t="inlineStr">
+        <is>
+          <t>Technical design, requirements documentation and IP/ownership questions for a legacy burn-in system replacement project (Pixel-Burn) at the owner's employer.</t>
+        </is>
+      </c>
+      <c r="H244" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="B245" s="3" t="inlineStr">
+        <is>
+          <t>Email safety assessment</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20_0746_Email-safety-assessment.md</t>
+        </is>
+      </c>
+      <c r="E245" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F245" s="2" t="inlineStr"/>
+      <c r="G245" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H245" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="B246" s="3" t="inlineStr">
+        <is>
+          <t>Phone voicemail delay</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20_0811_Phone-voicemail-delay.md</t>
+        </is>
+      </c>
+      <c r="E246" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F246" s="2" t="inlineStr"/>
+      <c r="G246" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H246" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="B247" s="3" t="inlineStr">
+        <is>
+          <t>Program details summary</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20_0854_Program-details-summary.md</t>
+        </is>
+      </c>
+      <c r="E247" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F247" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G247" s="3" t="inlineStr">
+        <is>
+          <t>Enquiry about professional training courses for AI, electronics/systems engineering and Microsoft 365 Copilot.</t>
+        </is>
+      </c>
+      <c r="H247" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H150"/>
+  <autoFilter ref="A1:H247"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6020,7 +9624,7 @@
         </is>
       </c>
       <c r="B1" t="n">
-        <v>149</v>
+        <v>246</v>
       </c>
     </row>
     <row r="2">
@@ -6030,7 +9634,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3">
@@ -6040,7 +9644,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
@@ -6050,7 +9654,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>35</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5">
@@ -6060,7 +9664,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>114</v>
+        <v>180</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
chat-sift: batches b30-b39 read; index, extracts and progress updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aq7txTcfpUgzabiqqnXaKj
</commit_message>
<xml_diff>
--- a/chat-sift/output/index.xlsx
+++ b/chat-sift/output/index.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$247</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$320</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H247"/>
+  <dimension ref="A1:H320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9599,8 +9599,2700 @@
         <v>1</v>
       </c>
     </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="B248" s="3" t="inlineStr">
+        <is>
+          <t>DSOX1102A vs EDUX1002G</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20_1034_DSOX1102A-vs-EDUX1002G.md</t>
+        </is>
+      </c>
+      <c r="E248" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G248" s="3" t="inlineStr">
+        <is>
+          <t>Owner states their professional role as an electronics engineer when choosing test equipment.</t>
+        </is>
+      </c>
+      <c r="H248" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="B249" s="3" t="inlineStr">
+        <is>
+          <t>Dunster House assembly costs</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20_1225_Dunster-House-assembly-costs.md</t>
+        </is>
+      </c>
+      <c r="E249" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F249" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G249" s="3" t="inlineStr">
+        <is>
+          <t>Owner mentions being able to verify test equipment calibration at work.</t>
+        </is>
+      </c>
+      <c r="H249" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="B250" s="3" t="inlineStr">
+        <is>
+          <t>Cheapest SDS804XHD offers</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20_1500_Cheapest-SDS804XHD-offers.md</t>
+        </is>
+      </c>
+      <c r="E250" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F250" s="2" t="inlineStr"/>
+      <c r="G250" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H250" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="B251" s="3" t="inlineStr">
+        <is>
+          <t>Sharpen image in Photoshop</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20_1729_Sharpen-image-in-Photoshop.md</t>
+        </is>
+      </c>
+      <c r="E251" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F251" s="2" t="inlineStr"/>
+      <c r="G251" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H251" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="B252" s="3" t="inlineStr">
+        <is>
+          <t>Isolate house reference</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20_1815_Isolate-house-reference.md</t>
+        </is>
+      </c>
+      <c r="E252" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F252" s="2" t="inlineStr"/>
+      <c r="G252" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H252" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="B253" s="3" t="inlineStr">
+        <is>
+          <t>High-resolution OK Computer image</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-20_2008_High-resolution-OK-Computer-image.md</t>
+        </is>
+      </c>
+      <c r="E253" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F253" s="2" t="inlineStr"/>
+      <c r="G253" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H253" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-21</t>
+        </is>
+      </c>
+      <c r="B254" s="3" t="inlineStr">
+        <is>
+          <t>Procreate vs Photoshop benefits</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-21_1105_Procreate-vs-Photoshop-benefits.md</t>
+        </is>
+      </c>
+      <c r="E254" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F254" s="2" t="inlineStr"/>
+      <c r="G254" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H254" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-21</t>
+        </is>
+      </c>
+      <c r="B255" s="3" t="inlineStr">
+        <is>
+          <t>Snap alignment fix</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-21_1404_Snap-alignment-fix.md</t>
+        </is>
+      </c>
+      <c r="E255" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F255" s="2" t="inlineStr"/>
+      <c r="G255" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H255" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-21</t>
+        </is>
+      </c>
+      <c r="B256" s="3" t="inlineStr">
+        <is>
+          <t>AirTasker log cabin help</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-21_1618_AirTasker-log-cabin-help.md</t>
+        </is>
+      </c>
+      <c r="E256" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F256" s="2" t="inlineStr"/>
+      <c r="G256" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H256" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-21</t>
+        </is>
+      </c>
+      <c r="B257" s="3" t="inlineStr">
+        <is>
+          <t>Skin background colours</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-21_1831_Skin-background-colours.md</t>
+        </is>
+      </c>
+      <c r="E257" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F257" s="2" t="inlineStr"/>
+      <c r="G257" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H257" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-21</t>
+        </is>
+      </c>
+      <c r="B258" s="3" t="inlineStr">
+        <is>
+          <t>Blend computer top</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-21_1856_Blend-computer-top.md</t>
+        </is>
+      </c>
+      <c r="E258" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F258" s="2" t="inlineStr"/>
+      <c r="G258" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H258" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-21</t>
+        </is>
+      </c>
+      <c r="B259" s="3" t="inlineStr">
+        <is>
+          <t>Edge softening technique</t>
+        </is>
+      </c>
+      <c r="C259" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-21_1900_Edge-softening-technique.md</t>
+        </is>
+      </c>
+      <c r="E259" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F259" s="2" t="inlineStr"/>
+      <c r="G259" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H259" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="B260" s="3" t="inlineStr">
+        <is>
+          <t>Complete house concept</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-22_1008_Complete-house-concept.md</t>
+        </is>
+      </c>
+      <c r="E260" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F260" s="2" t="inlineStr"/>
+      <c r="G260" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H260" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="B261" s="3" t="inlineStr">
+        <is>
+          <t>Background color details</t>
+        </is>
+      </c>
+      <c r="C261" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-22_1009_Background-color-details.md</t>
+        </is>
+      </c>
+      <c r="E261" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F261" s="2" t="inlineStr"/>
+      <c r="G261" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H261" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="B262" s="3" t="inlineStr">
+        <is>
+          <t>1022 vs Keysight comparison</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-22_1154_1022-vs-Keysight-comparison.md</t>
+        </is>
+      </c>
+      <c r="E262" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F262" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G262" s="3" t="inlineStr">
+        <is>
+          <t>Comparison and availability of waveform generator test equipment.</t>
+        </is>
+      </c>
+      <c r="H262" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="B263" s="3" t="inlineStr">
+        <is>
+          <t>Op amp offset issue</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-22_1627_Op-amp-offset-issue.md</t>
+        </is>
+      </c>
+      <c r="E263" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G263" s="3" t="inlineStr">
+        <is>
+          <t>Fault-finding on a video circuit board (op-amp offset, floating node, start-up bias) and how a proposed fix may be received by others.</t>
+        </is>
+      </c>
+      <c r="H263" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-24</t>
+        </is>
+      </c>
+      <c r="B264" s="3" t="inlineStr">
+        <is>
+          <t>Amusing Dating Response Ideas</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-24_1324_Amusing-Dating-Response-Ideas.md</t>
+        </is>
+      </c>
+      <c r="E264" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F264" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G264" s="3" t="inlineStr">
+        <is>
+          <t>Brief reference to a shared goal of qualifying as a psychotherapist (possible career aspiration).</t>
+        </is>
+      </c>
+      <c r="H264" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-24</t>
+        </is>
+      </c>
+      <c r="B265" s="3" t="inlineStr">
+        <is>
+          <t>Best Stud Wall Videos</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-24_1449_Best-Stud-Wall-Videos.md</t>
+        </is>
+      </c>
+      <c r="E265" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F265" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G265" s="3" t="inlineStr">
+        <is>
+          <t>Concern about job security given as the reason for planning to rent out part of the home.</t>
+        </is>
+      </c>
+      <c r="H265" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-24</t>
+        </is>
+      </c>
+      <c r="B266" s="3" t="inlineStr">
+        <is>
+          <t>Drawing Analysis Explanation</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-24_1831_Drawing-Analysis-Explanation.md</t>
+        </is>
+      </c>
+      <c r="E266" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F266" s="2" t="inlineStr"/>
+      <c r="G266" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H266" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-24</t>
+        </is>
+      </c>
+      <c r="B267" s="3" t="inlineStr">
+        <is>
+          <t>Cutting Cabin Eaves Safely</t>
+        </is>
+      </c>
+      <c r="C267" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-24_2207_Cutting-Cabin-Eaves-Safely.md</t>
+        </is>
+      </c>
+      <c r="E267" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F267" s="2" t="inlineStr"/>
+      <c r="G267" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H267" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-25</t>
+        </is>
+      </c>
+      <c r="B268" s="3" t="inlineStr">
+        <is>
+          <t>Why Women Post Sexy Videos</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-25_0713_Why-Women-Post-Sexy-Videos.md</t>
+        </is>
+      </c>
+      <c r="E268" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F268" s="2" t="inlineStr"/>
+      <c r="G268" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H268" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-25</t>
+        </is>
+      </c>
+      <c r="B269" s="3" t="inlineStr">
+        <is>
+          <t>Pointing and ASD Signs</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-25_1334_Pointing-and-ASD-Signs.md</t>
+        </is>
+      </c>
+      <c r="E269" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F269" s="2" t="inlineStr"/>
+      <c r="G269" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H269" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-25</t>
+        </is>
+      </c>
+      <c r="B270" s="3" t="inlineStr">
+        <is>
+          <t>Quality Log Building Benefits</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-25_1350_Quality-Log-Building-Benefits.md</t>
+        </is>
+      </c>
+      <c r="E270" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F270" s="2" t="inlineStr"/>
+      <c r="G270" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H270" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-25</t>
+        </is>
+      </c>
+      <c r="B271" s="3" t="inlineStr">
+        <is>
+          <t>Schaum Feedback and Control</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-25_1422_Schaum-Feedback-and-Control.md</t>
+        </is>
+      </c>
+      <c r="E271" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F271" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G271" s="3" t="inlineStr">
+        <is>
+          <t>Owner mentions returning to technical work after years as a team leader and wanting to advance job-related skills.</t>
+        </is>
+      </c>
+      <c r="H271" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-25</t>
+        </is>
+      </c>
+      <c r="B272" s="3" t="inlineStr">
+        <is>
+          <t>AoE vs Learning AoE</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-25_1540_AoE-vs-Learning-AoE.md</t>
+        </is>
+      </c>
+      <c r="E272" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F272" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G272" s="3" t="inlineStr">
+        <is>
+          <t>AI relates book choice to the owner's analogue fault-finding work.</t>
+        </is>
+      </c>
+      <c r="H272" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-25</t>
+        </is>
+      </c>
+      <c r="B273" s="3" t="inlineStr">
+        <is>
+          <t>Psychologist Session Mismatch</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-25_1729_Psychologist-Session-Mismatch.md</t>
+        </is>
+      </c>
+      <c r="E273" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F273" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G273" s="3" t="inlineStr">
+        <is>
+          <t>Passing references to a work-donated voucher used for private sessions, leaving work early when unwell, work commitments, and negotiating a four-day working week.</t>
+        </is>
+      </c>
+      <c r="H273" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="B274" s="3" t="inlineStr">
+        <is>
+          <t>Work Folder Optimization Tips</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26_0716_Work-Folder-Optimization-Tips.md</t>
+        </is>
+      </c>
+      <c r="E274" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F274" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G274" s="3" t="inlineStr">
+        <is>
+          <t>Organising a work folder, fault-finding/triage and debug documentation templates, section naming and a weekly work planner, plus related laptop accessories and an employer logo.</t>
+        </is>
+      </c>
+      <c r="H274" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="B275" s="3" t="inlineStr">
+        <is>
+          <t>iPhone 15 Magnetic Cases</t>
+        </is>
+      </c>
+      <c r="C275" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D275" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26_1359_iPhone-15-Magnetic-Cases.md</t>
+        </is>
+      </c>
+      <c r="E275" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F275" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G275" s="3" t="inlineStr">
+        <is>
+          <t>Choosing stylus and screen protector options for occasional work sketching and for a laptop possibly used for work.</t>
+        </is>
+      </c>
+      <c r="H275" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="B276" s="3" t="inlineStr">
+        <is>
+          <t>iPhone 13 Case Compatibility</t>
+        </is>
+      </c>
+      <c r="C276" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D276" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26_1706_iPhone-13-Case-Compatibility.md</t>
+        </is>
+      </c>
+      <c r="E276" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F276" s="2" t="inlineStr"/>
+      <c r="G276" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H276" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="B277" s="3" t="inlineStr">
+        <is>
+          <t>Under Siege 2 Streaming</t>
+        </is>
+      </c>
+      <c r="C277" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D277" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26_1729_Under-Siege-2-Streaming.md</t>
+        </is>
+      </c>
+      <c r="E277" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F277" s="2" t="inlineStr"/>
+      <c r="G277" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H277" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="B278" s="3" t="inlineStr">
+        <is>
+          <t>Childhood Reflection Analysis</t>
+        </is>
+      </c>
+      <c r="C278" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D278" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26_1753_Childhood-Reflection-Analysis.md</t>
+        </is>
+      </c>
+      <c r="E278" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F278" s="2" t="inlineStr"/>
+      <c r="G278" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H278" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="B279" s="3" t="inlineStr">
+        <is>
+          <t>Accidental Message Clarification</t>
+        </is>
+      </c>
+      <c r="C279" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D279" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26_1944_Accidental-Message-Clarification.md</t>
+        </is>
+      </c>
+      <c r="E279" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F279" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G279" s="3" t="inlineStr">
+        <is>
+          <t>Designing a printable weekly work planner with company logo, week number and work-focused sections.</t>
+        </is>
+      </c>
+      <c r="H279" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="B280" s="3" t="inlineStr">
+        <is>
+          <t>Clarification Request</t>
+        </is>
+      </c>
+      <c r="C280" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D280" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26_1944_Clarification-Request.md</t>
+        </is>
+      </c>
+      <c r="E280" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F280" s="2" t="inlineStr"/>
+      <c r="G280" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H280" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="B281" s="3" t="inlineStr">
+        <is>
+          <t>Coffee Opener Suggestions</t>
+        </is>
+      </c>
+      <c r="C281" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D281" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-26_2055_Coffee-Opener-Suggestions.md</t>
+        </is>
+      </c>
+      <c r="E281" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F281" s="2" t="inlineStr"/>
+      <c r="G281" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H281" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-27</t>
+        </is>
+      </c>
+      <c r="B282" s="3" t="inlineStr">
+        <is>
+          <t>Dirty Rotten Scoundrels Twist</t>
+        </is>
+      </c>
+      <c r="C282" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D282" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-27_0717_Dirty-Rotten-Scoundrels-Twist.md</t>
+        </is>
+      </c>
+      <c r="E282" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F282" s="2" t="inlineStr"/>
+      <c r="G282" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H282" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-27</t>
+        </is>
+      </c>
+      <c r="B283" s="3" t="inlineStr">
+        <is>
+          <t>Plastic Surface Preparation</t>
+        </is>
+      </c>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D283" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-27_0922_Plastic-Surface-Preparation.md</t>
+        </is>
+      </c>
+      <c r="E283" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F283" s="2" t="inlineStr"/>
+      <c r="G283" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H283" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-27</t>
+        </is>
+      </c>
+      <c r="B284" s="3" t="inlineStr">
+        <is>
+          <t>Lens Tint Shade Inquiry</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D284" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-27_1058_Lens-Tint-Shade-Inquiry.md</t>
+        </is>
+      </c>
+      <c r="E284" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F284" s="2" t="inlineStr"/>
+      <c r="G284" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H284" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-27</t>
+        </is>
+      </c>
+      <c r="B285" s="3" t="inlineStr">
+        <is>
+          <t>Getting Noticed Playfully</t>
+        </is>
+      </c>
+      <c r="C285" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D285" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-27_1109_Getting-Noticed-Playfully.md</t>
+        </is>
+      </c>
+      <c r="E285" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F285" s="2" t="inlineStr"/>
+      <c r="G285" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H285" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-27</t>
+        </is>
+      </c>
+      <c r="B286" s="3" t="inlineStr">
+        <is>
+          <t>Sheet Metal Crease Survival</t>
+        </is>
+      </c>
+      <c r="C286" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D286" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-27_1303_Sheet-Metal-Crease-Survival.md</t>
+        </is>
+      </c>
+      <c r="E286" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F286" s="2" t="inlineStr"/>
+      <c r="G286" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H286" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-27</t>
+        </is>
+      </c>
+      <c r="B287" s="3" t="inlineStr">
+        <is>
+          <t>Albert Speer's War End</t>
+        </is>
+      </c>
+      <c r="C287" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D287" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-27_1356_Albert-Speer-s-War-End.md</t>
+        </is>
+      </c>
+      <c r="E287" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F287" s="2" t="inlineStr"/>
+      <c r="G287" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H287" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-27</t>
+        </is>
+      </c>
+      <c r="B288" s="3" t="inlineStr">
+        <is>
+          <t>Gerda Christian Biography</t>
+        </is>
+      </c>
+      <c r="C288" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-27_1524_Gerda-Christian-Biography.md</t>
+        </is>
+      </c>
+      <c r="E288" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F288" s="2" t="inlineStr"/>
+      <c r="G288" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H288" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-28</t>
+        </is>
+      </c>
+      <c r="B289" s="3" t="inlineStr">
+        <is>
+          <t>Tesco Sheet</t>
+        </is>
+      </c>
+      <c r="C289" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D289" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-28_0755_Tesco-Sheet.md</t>
+        </is>
+      </c>
+      <c r="E289" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F289" s="2" t="inlineStr"/>
+      <c r="G289" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H289" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-28</t>
+        </is>
+      </c>
+      <c r="B290" s="3" t="inlineStr">
+        <is>
+          <t>Polo vs T-shirt Comparison</t>
+        </is>
+      </c>
+      <c r="C290" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D290" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-28_0847_Polo-vs-T-shirt-Comparison.md</t>
+        </is>
+      </c>
+      <c r="E290" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F290" s="2" t="inlineStr"/>
+      <c r="G290" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H290" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-28</t>
+        </is>
+      </c>
+      <c r="B291" s="3" t="inlineStr">
+        <is>
+          <t>iPhone to PC File Transfer</t>
+        </is>
+      </c>
+      <c r="C291" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D291" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-28_1055_iPhone-to-PC-File-Transfer.md</t>
+        </is>
+      </c>
+      <c r="E291" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F291" s="2" t="inlineStr"/>
+      <c r="G291" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H291" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-28</t>
+        </is>
+      </c>
+      <c r="B292" s="3" t="inlineStr">
+        <is>
+          <t>Bin Collection Schedule CM12TE</t>
+        </is>
+      </c>
+      <c r="C292" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D292" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-28_2032_Bin-Collection-Schedule-CM12TE.md</t>
+        </is>
+      </c>
+      <c r="E292" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F292" s="2" t="inlineStr"/>
+      <c r="G292" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H292" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="B293" s="3" t="inlineStr">
+        <is>
+          <t>No content provided</t>
+        </is>
+      </c>
+      <c r="C293" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D293" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-29_1015_No-content-provided.md</t>
+        </is>
+      </c>
+      <c r="E293" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F293" s="2" t="inlineStr"/>
+      <c r="G293" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H293" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="B294" s="3" t="inlineStr">
+        <is>
+          <t>Revert Number Pad Input</t>
+        </is>
+      </c>
+      <c r="C294" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D294" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-29_1159_Revert-Number-Pad-Input.md</t>
+        </is>
+      </c>
+      <c r="E294" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F294" s="2" t="inlineStr"/>
+      <c r="G294" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H294" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="B295" s="3" t="inlineStr">
+        <is>
+          <t>Raising Presser Foot for Thickness</t>
+        </is>
+      </c>
+      <c r="C295" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D295" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-29_1450_Raising-Presser-Foot-for-Thickness.md</t>
+        </is>
+      </c>
+      <c r="E295" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F295" s="2" t="inlineStr"/>
+      <c r="G295" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H295" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="B296" s="3" t="inlineStr">
+        <is>
+          <t>Best Free Screenshot Annotators</t>
+        </is>
+      </c>
+      <c r="C296" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D296" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-29_1909_Best-Free-Screenshot-Annotators.md</t>
+        </is>
+      </c>
+      <c r="E296" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F296" s="2" t="inlineStr"/>
+      <c r="G296" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H296" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="B297" s="3" t="inlineStr">
+        <is>
+          <t>Scooter Error Code 16</t>
+        </is>
+      </c>
+      <c r="C297" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D297" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-29_2005_Scooter-Error-Code-16.md</t>
+        </is>
+      </c>
+      <c r="E297" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F297" s="2" t="inlineStr"/>
+      <c r="G297" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H297" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="B298" s="3" t="inlineStr">
+        <is>
+          <t>Using ChatGPT as Journal</t>
+        </is>
+      </c>
+      <c r="C298" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D298" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-29_2056_Using-ChatGPT-as-Journal.md</t>
+        </is>
+      </c>
+      <c r="E298" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F298" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G298" s="3" t="inlineStr">
+        <is>
+          <t>Setting up a reflective journal that includes a separate chat for work-related reflections.</t>
+        </is>
+      </c>
+      <c r="H298" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="B299" s="3" t="inlineStr">
+        <is>
+          <t>Empath Loner Explained</t>
+        </is>
+      </c>
+      <c r="C299" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D299" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-29_2221_Empath-Loner-Explained.md</t>
+        </is>
+      </c>
+      <c r="E299" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F299" s="2" t="inlineStr"/>
+      <c r="G299" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H299" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="B300" s="3" t="inlineStr">
+        <is>
+          <t>Shelf Life of Daily Greens</t>
+        </is>
+      </c>
+      <c r="C300" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D300" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-29_2309_Shelf-Life-of-Daily-Greens.md</t>
+        </is>
+      </c>
+      <c r="E300" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F300" s="2" t="inlineStr"/>
+      <c r="G300" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H300" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B301" s="3" t="inlineStr">
+        <is>
+          <t>MPP Stylus Setup Guide</t>
+        </is>
+      </c>
+      <c r="C301" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-002.json</t>
+        </is>
+      </c>
+      <c r="D301" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_0732_MPP-Stylus-Setup-Guide.md</t>
+        </is>
+      </c>
+      <c r="E301" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F301" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G301" s="3" t="inlineStr">
+        <is>
+          <t>Software settings question about viewing technical/engineering drawing PDFs in Acrobat, possibly in a work context.</t>
+        </is>
+      </c>
+      <c r="H301" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B302" s="3" t="inlineStr">
+        <is>
+          <t>Anniversary Expectation Reflection</t>
+        </is>
+      </c>
+      <c r="C302" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D302" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_1536_Anniversary-Expectation-Reflection.md</t>
+        </is>
+      </c>
+      <c r="E302" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F302" s="2" t="inlineStr"/>
+      <c r="G302" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H302" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B303" s="3" t="inlineStr">
+        <is>
+          <t>Family Communication Dynamics</t>
+        </is>
+      </c>
+      <c r="C303" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D303" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_1619_Family-Communication-Dynamics.md</t>
+        </is>
+      </c>
+      <c r="E303" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F303" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G303" s="3" t="inlineStr">
+        <is>
+          <t>Passing references to the owner's work, including whether a diagnosis relates to work and work-related stressors cited as a possible contributor to difficulties.</t>
+        </is>
+      </c>
+      <c r="H303" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B304" s="3" t="inlineStr">
+        <is>
+          <t>Project Reflection Framework</t>
+        </is>
+      </c>
+      <c r="C304" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D304" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_1652_Project-Reflection-Framework.md</t>
+        </is>
+      </c>
+      <c r="E304" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F304" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G304" s="3" t="inlineStr">
+        <is>
+          <t>Passing reference to work-related stressors cited as a possible contributor to the owner's difficulties.</t>
+        </is>
+      </c>
+      <c r="H304" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B305" s="3" t="inlineStr">
+        <is>
+          <t>Clarifying Boundaries and Impact</t>
+        </is>
+      </c>
+      <c r="C305" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D305" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_1709_Clarifying-Boundaries-and-Impact.md</t>
+        </is>
+      </c>
+      <c r="E305" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F305" s="2" t="inlineStr"/>
+      <c r="G305" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H305" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B306" s="3" t="inlineStr">
+        <is>
+          <t>1 - child notes</t>
+        </is>
+      </c>
+      <c r="C306" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D306" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_1831_1-child-notes.md</t>
+        </is>
+      </c>
+      <c r="E306" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F306" s="2" t="inlineStr"/>
+      <c r="G306" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H306" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B307" s="3" t="inlineStr">
+        <is>
+          <t>2a - Bologna</t>
+        </is>
+      </c>
+      <c r="C307" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D307" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_1840_2a-Bologna.md</t>
+        </is>
+      </c>
+      <c r="E307" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F307" s="2" t="inlineStr"/>
+      <c r="G307" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H307" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B308" s="3" t="inlineStr">
+        <is>
+          <t>2b - £80 Incident</t>
+        </is>
+      </c>
+      <c r="C308" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D308" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_1841_2b-80-Incident.md</t>
+        </is>
+      </c>
+      <c r="E308" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F308" s="2" t="inlineStr"/>
+      <c r="G308" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H308" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B309" s="3" t="inlineStr">
+        <is>
+          <t>4 - Christmas incident</t>
+        </is>
+      </c>
+      <c r="C309" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D309" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_1842_4-Christmas-incident.md</t>
+        </is>
+      </c>
+      <c r="E309" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F309" s="2" t="inlineStr"/>
+      <c r="G309" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H309" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B310" s="3" t="inlineStr">
+        <is>
+          <t>2c - Gig Trust Incident</t>
+        </is>
+      </c>
+      <c r="C310" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D310" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_1846_2c-Gig-Trust-Incident.md</t>
+        </is>
+      </c>
+      <c r="E310" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F310" s="2" t="inlineStr"/>
+      <c r="G310" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H310" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B311" s="3" t="inlineStr">
+        <is>
+          <t>5 - Dismissive Medical Journey</t>
+        </is>
+      </c>
+      <c r="C311" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D311" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_1852_5-Dismissive-Medical-Journey.md</t>
+        </is>
+      </c>
+      <c r="E311" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F311" s="2" t="inlineStr"/>
+      <c r="G311" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H311" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B312" s="3" t="inlineStr">
+        <is>
+          <t>Chat Gap Analysis</t>
+        </is>
+      </c>
+      <c r="C312" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D312" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_1853_Chat-Gap-Analysis.md</t>
+        </is>
+      </c>
+      <c r="E312" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F312" s="2" t="inlineStr"/>
+      <c r="G312" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H312" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B313" s="3" t="inlineStr">
+        <is>
+          <t>Next steps after sharing numbers</t>
+        </is>
+      </c>
+      <c r="C313" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D313" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_2026_Next-steps-after-sharing-numbers.md</t>
+        </is>
+      </c>
+      <c r="E313" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F313" s="2" t="inlineStr"/>
+      <c r="G313" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H313" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B314" s="3" t="inlineStr">
+        <is>
+          <t>11 - Dog Care trust</t>
+        </is>
+      </c>
+      <c r="C314" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D314" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_2210_11-Dog-Care-trust.md</t>
+        </is>
+      </c>
+      <c r="E314" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F314" s="2" t="inlineStr"/>
+      <c r="G314" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H314" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B315" s="3" t="inlineStr">
+        <is>
+          <t>12 - sewing machine Trust and Skill Development</t>
+        </is>
+      </c>
+      <c r="C315" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D315" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_2224_12-sewing-machine-Trust-and-Skill-Development.md</t>
+        </is>
+      </c>
+      <c r="E315" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F315" s="2" t="inlineStr"/>
+      <c r="G315" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H315" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B316" s="3" t="inlineStr">
+        <is>
+          <t>Neuron Diversity and Addiction</t>
+        </is>
+      </c>
+      <c r="C316" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D316" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_2234_Neuron-Diversity-and-Addiction.md</t>
+        </is>
+      </c>
+      <c r="E316" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F316" s="2" t="inlineStr"/>
+      <c r="G316" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H316" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B317" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14 - dismissing alcohol consequence </t>
+        </is>
+      </c>
+      <c r="C317" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D317" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_2321_14-dismissing-alcohol-consequence.md</t>
+        </is>
+      </c>
+      <c r="E317" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F317" s="2" t="inlineStr"/>
+      <c r="G317" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H317" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B318" s="3" t="inlineStr">
+        <is>
+          <t>Clinical Psychologist vs Therapist</t>
+        </is>
+      </c>
+      <c r="C318" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D318" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30_2331_Clinical-Psychologist-vs-Therapist.md</t>
+        </is>
+      </c>
+      <c r="E318" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F318" s="2" t="inlineStr"/>
+      <c r="G318" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H318" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B319" s="3" t="inlineStr">
+        <is>
+          <t>17 - psychologist child</t>
+        </is>
+      </c>
+      <c r="C319" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D319" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31_0016_17-psychologist-child.md</t>
+        </is>
+      </c>
+      <c r="E319" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F319" s="2" t="inlineStr"/>
+      <c r="G319" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H319" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B320" s="3" t="inlineStr">
+        <is>
+          <t>ASD Support Levels</t>
+        </is>
+      </c>
+      <c r="C320" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D320" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31_0026_ASD-Support-Levels.md</t>
+        </is>
+      </c>
+      <c r="E320" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F320" s="2" t="inlineStr"/>
+      <c r="G320" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H320" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H247"/>
+  <autoFilter ref="A1:H320"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9624,7 +12316,7 @@
         </is>
       </c>
       <c r="B1" t="n">
-        <v>246</v>
+        <v>319</v>
       </c>
     </row>
     <row r="2">
@@ -9634,7 +12326,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -9644,7 +12336,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4">
@@ -9654,7 +12346,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>66</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5">
@@ -9664,7 +12356,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>180</v>
+        <v>237</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
chat-sift: batches b40-b49 read; index, extracts and progress updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aq7txTcfpUgzabiqqnXaKj
</commit_message>
<xml_diff>
--- a/chat-sift/output/index.xlsx
+++ b/chat-sift/output/index.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$320</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$384</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H320"/>
+  <dimension ref="A1:H384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12291,8 +12291,2352 @@
         <v>0</v>
       </c>
     </row>
+    <row r="321">
+      <c r="A321" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B321" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18 - asd stuff </t>
+        </is>
+      </c>
+      <c r="C321" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D321" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31_0034_18-asd-stuff.md</t>
+        </is>
+      </c>
+      <c r="E321" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F321" s="2" t="inlineStr"/>
+      <c r="G321" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H321" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B322" s="3" t="inlineStr">
+        <is>
+          <t>Simplified Email for GP</t>
+        </is>
+      </c>
+      <c r="C322" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D322" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31_0759_Simplified-Email-for-GP.md</t>
+        </is>
+      </c>
+      <c r="E322" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F322" s="2" t="inlineStr"/>
+      <c r="G322" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H322" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B323" s="3" t="inlineStr">
+        <is>
+          <t>Get Noticed Strategies</t>
+        </is>
+      </c>
+      <c r="C323" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D323" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31_0858_Get-Noticed-Strategies.md</t>
+        </is>
+      </c>
+      <c r="E323" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F323" s="2" t="inlineStr"/>
+      <c r="G323" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H323" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B324" s="3" t="inlineStr">
+        <is>
+          <t>Avoidant Flag in Messaging</t>
+        </is>
+      </c>
+      <c r="C324" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D324" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31_1006_Avoidant-Flag-in-Messaging.md</t>
+        </is>
+      </c>
+      <c r="E324" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F324" s="2" t="inlineStr"/>
+      <c r="G324" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H324" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B325" s="3" t="inlineStr">
+        <is>
+          <t>Legal Process for Drug Offense</t>
+        </is>
+      </c>
+      <c r="C325" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D325" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31_1023_Legal-Process-for-Drug-Offense.md</t>
+        </is>
+      </c>
+      <c r="E325" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F325" s="2" t="inlineStr"/>
+      <c r="G325" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H325" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B326" s="3" t="inlineStr">
+        <is>
+          <t>1.1.1- Legal Process Mapping</t>
+        </is>
+      </c>
+      <c r="C326" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D326" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31_1030_1-1-1-Legal-Process-Mapping.md</t>
+        </is>
+      </c>
+      <c r="E326" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F326" s="2" t="inlineStr"/>
+      <c r="G326" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H326" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B327" s="3" t="inlineStr">
+        <is>
+          <t>2.1.1- Document Upload</t>
+        </is>
+      </c>
+      <c r="C327" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D327" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31_1110_2-1-1-Document-Upload.md</t>
+        </is>
+      </c>
+      <c r="E327" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F327" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G327" s="3" t="inlineStr">
+        <is>
+          <t>Upload of an occupational health report (Medigold Health) and a fit note, acknowledged by the AI.</t>
+        </is>
+      </c>
+      <c r="H327" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B328" s="3" t="inlineStr">
+        <is>
+          <t>Chelmsford New Year's Parkrun</t>
+        </is>
+      </c>
+      <c r="C328" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D328" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31_1334_Chelmsford-New-Year-s-Parkrun.md</t>
+        </is>
+      </c>
+      <c r="E328" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F328" s="2" t="inlineStr"/>
+      <c r="G328" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H328" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B329" s="3" t="inlineStr">
+        <is>
+          <t>[3.1.1]- Chronology Request</t>
+        </is>
+      </c>
+      <c r="C329" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D329" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31_1338_3-1-1-Chronology-Request.md</t>
+        </is>
+      </c>
+      <c r="E329" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F329" s="2" t="inlineStr"/>
+      <c r="G329" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H329" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B330" s="3" t="inlineStr">
+        <is>
+          <t>0.0.0 - Chat Sandbox</t>
+        </is>
+      </c>
+      <c r="C330" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D330" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31_1412_0-0-0-Chat-Sandbox.md</t>
+        </is>
+      </c>
+      <c r="E330" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F330" s="2" t="inlineStr"/>
+      <c r="G330" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H330" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B331" s="3" t="inlineStr">
+        <is>
+          <t>0.1.1 - Receipt Log</t>
+        </is>
+      </c>
+      <c r="C331" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D331" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31_1440_0-1-1-Receipt-Log.md</t>
+        </is>
+      </c>
+      <c r="E331" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F331" s="2" t="inlineStr"/>
+      <c r="G331" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H331" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B332" s="3" t="inlineStr">
+        <is>
+          <t>Self image map</t>
+        </is>
+      </c>
+      <c r="C332" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D332" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31_1847_Self-image-map.md</t>
+        </is>
+      </c>
+      <c r="E332" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F332" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G332" s="3" t="inlineStr">
+        <is>
+          <t>A digitised personal domain map includes a Work section listing employment, productivity, stress, purpose and progression.</t>
+        </is>
+      </c>
+      <c r="H332" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B333" s="3" t="inlineStr">
+        <is>
+          <t>Embracing Solitude and Loneliness</t>
+        </is>
+      </c>
+      <c r="C333" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D333" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-31_2104_Embracing-Solitude-and-Loneliness.md</t>
+        </is>
+      </c>
+      <c r="E333" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F333" s="2" t="inlineStr"/>
+      <c r="G333" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H333" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B334" s="3" t="inlineStr">
+        <is>
+          <t>Solar System Redraw Check</t>
+        </is>
+      </c>
+      <c r="C334" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D334" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01_0619_Solar-System-Redraw-Check.md</t>
+        </is>
+      </c>
+      <c r="E334" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F334" s="2" t="inlineStr"/>
+      <c r="G334" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H334" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B335" s="3" t="inlineStr">
+        <is>
+          <t>Childhood Info Request Process</t>
+        </is>
+      </c>
+      <c r="C335" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D335" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01_0908_Childhood-Info-Request-Process.md</t>
+        </is>
+      </c>
+      <c r="E335" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F335" s="2" t="inlineStr"/>
+      <c r="G335" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H335" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B336" s="3" t="inlineStr">
+        <is>
+          <t>Car Battery Lifespan 2005</t>
+        </is>
+      </c>
+      <c r="C336" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D336" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01_1101_Car-Battery-Lifespan-2005.md</t>
+        </is>
+      </c>
+      <c r="E336" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F336" s="2" t="inlineStr"/>
+      <c r="G336" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H336" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B337" s="3" t="inlineStr">
+        <is>
+          <t>Guilt Over Dog's Needs</t>
+        </is>
+      </c>
+      <c r="C337" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D337" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01_1454_Guilt-Over-Dog-s-Needs.md</t>
+        </is>
+      </c>
+      <c r="E337" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F337" s="2" t="inlineStr"/>
+      <c r="G337" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H337" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B338" s="3" t="inlineStr">
+        <is>
+          <t>Getting Noticed Openers</t>
+        </is>
+      </c>
+      <c r="C338" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D338" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01_1515_Getting-Noticed-Openers.md</t>
+        </is>
+      </c>
+      <c r="E338" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F338" s="2" t="inlineStr"/>
+      <c r="G338" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H338" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B339" s="3" t="inlineStr">
+        <is>
+          <t>Lumps groin headache causes</t>
+        </is>
+      </c>
+      <c r="C339" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D339" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01_1538_Lumps-groin-headache-causes.md</t>
+        </is>
+      </c>
+      <c r="E339" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F339" s="2" t="inlineStr"/>
+      <c r="G339" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H339" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B340" s="3" t="inlineStr">
+        <is>
+          <t>Log Cabin Plan Review</t>
+        </is>
+      </c>
+      <c r="C340" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D340" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01_2026_Log-Cabin-Plan-Review.md</t>
+        </is>
+      </c>
+      <c r="E340" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F340" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G340" s="3" t="inlineStr">
+        <is>
+          <t>Planning and construction design for the owner's 'Daft Badger' log cabin project (possible own venture).</t>
+        </is>
+      </c>
+      <c r="H340" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B341" s="3" t="inlineStr">
+        <is>
+          <t>Project A Overview</t>
+        </is>
+      </c>
+      <c r="C341" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D341" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1245_Project-A-Overview.md</t>
+        </is>
+      </c>
+      <c r="E341" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F341" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G341" s="3" t="inlineStr">
+        <is>
+          <t>An Occupational Health folder is listed within a personal document structure.</t>
+        </is>
+      </c>
+      <c r="H341" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B342" s="3" t="inlineStr">
+        <is>
+          <t>A3 - Documentation Baseline</t>
+        </is>
+      </c>
+      <c r="C342" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D342" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1247_A3-Documentation-Baseline.md</t>
+        </is>
+      </c>
+      <c r="E342" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F342" s="2" t="inlineStr"/>
+      <c r="G342" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H342" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B343" s="3" t="inlineStr">
+        <is>
+          <t>Document Transcription</t>
+        </is>
+      </c>
+      <c r="C343" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D343" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1257_Document-Transcription.md</t>
+        </is>
+      </c>
+      <c r="E343" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F343" s="2" t="inlineStr"/>
+      <c r="G343" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H343" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B344" s="3" t="inlineStr">
+        <is>
+          <t>A4 - Incident &amp; Recall</t>
+        </is>
+      </c>
+      <c r="C344" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D344" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1301_A4-Incident-Recall.md</t>
+        </is>
+      </c>
+      <c r="E344" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F344" s="2" t="inlineStr"/>
+      <c r="G344" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H344" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B345" s="3" t="inlineStr">
+        <is>
+          <t>A1 - GPT History work</t>
+        </is>
+      </c>
+      <c r="C345" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D345" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1303_A1-GPT-History-work.md</t>
+        </is>
+      </c>
+      <c r="E345" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F345" s="2" t="inlineStr"/>
+      <c r="G345" s="3" t="inlineStr">
+        <is>
+          <t>Employment and work-stress context (role, workload, managerial support, project rejection, disclosure at work) within a consolidated reference document.</t>
+        </is>
+      </c>
+      <c r="H345" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B346" s="3" t="inlineStr">
+        <is>
+          <t>A0 - Chat Sandbox</t>
+        </is>
+      </c>
+      <c r="C346" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D346" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1304_A0-Chat-Sandbox.md</t>
+        </is>
+      </c>
+      <c r="E346" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F346" s="2" t="inlineStr"/>
+      <c r="G346" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H346" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B347" s="3" t="inlineStr">
+        <is>
+          <t>A2 - Document Transcription</t>
+        </is>
+      </c>
+      <c r="C347" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D347" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1307_A2-Document-Transcription.md</t>
+        </is>
+      </c>
+      <c r="E347" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F347" s="2" t="inlineStr"/>
+      <c r="G347" s="3" t="inlineStr">
+        <is>
+          <t>Transcription of an occupational health assessment and a GP fit note advising phased return to work with amended duties and workplace adaptations.</t>
+        </is>
+      </c>
+      <c r="H347" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B348" s="3" t="inlineStr">
+        <is>
+          <t>B1 - Case Administration &amp; Records</t>
+        </is>
+      </c>
+      <c r="C348" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D348" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1311_B1-Case-Administration-Records.md</t>
+        </is>
+      </c>
+      <c r="E348" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F348" s="2" t="inlineStr"/>
+      <c r="G348" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H348" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B349" s="3" t="inlineStr">
+        <is>
+          <t>B2 - Evidence &amp; Documentation</t>
+        </is>
+      </c>
+      <c r="C349" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D349" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1311_B2-Evidence-Documentation.md</t>
+        </is>
+      </c>
+      <c r="E349" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F349" s="2" t="inlineStr"/>
+      <c r="G349" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H349" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B350" s="3" t="inlineStr">
+        <is>
+          <t>B3 - Incident Factual Core Layer</t>
+        </is>
+      </c>
+      <c r="C350" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D350" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1312_B3-Incident-Factual-Core-Layer.md</t>
+        </is>
+      </c>
+      <c r="E350" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F350" s="2" t="inlineStr"/>
+      <c r="G350" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H350" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B351" s="3" t="inlineStr">
+        <is>
+          <t>B4 - Context &amp; Mental Health</t>
+        </is>
+      </c>
+      <c r="C351" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D351" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1312_B4-Context-Mental-Health.md</t>
+        </is>
+      </c>
+      <c r="E351" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F351" s="2" t="inlineStr"/>
+      <c r="G351" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H351" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B352" s="3" t="inlineStr">
+        <is>
+          <t>Project B Overview</t>
+        </is>
+      </c>
+      <c r="C352" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D352" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1314_Project-B-Overview.md</t>
+        </is>
+      </c>
+      <c r="E352" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F352" s="2" t="inlineStr"/>
+      <c r="G352" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H352" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B353" s="3" t="inlineStr">
+        <is>
+          <t>B5 - Investigation Interview</t>
+        </is>
+      </c>
+      <c r="C353" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D353" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1315_B5-Investigation-Interview.md</t>
+        </is>
+      </c>
+      <c r="E353" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F353" s="2" t="inlineStr"/>
+      <c r="G353" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H353" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B354" s="3" t="inlineStr">
+        <is>
+          <t>B6 - Charges Court Process</t>
+        </is>
+      </c>
+      <c r="C354" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D354" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1315_B6-Charges-Court-Process.md</t>
+        </is>
+      </c>
+      <c r="E354" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F354" s="2" t="inlineStr"/>
+      <c r="G354" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H354" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B355" s="3" t="inlineStr">
+        <is>
+          <t>B6.1 - First hearing outline &amp; Prep.</t>
+        </is>
+      </c>
+      <c r="C355" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D355" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1351_B6-1-First-hearing-outline-Prep.md</t>
+        </is>
+      </c>
+      <c r="E355" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F355" s="2" t="inlineStr"/>
+      <c r="G355" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H355" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B356" s="3" t="inlineStr">
+        <is>
+          <t>Polo Care Tips</t>
+        </is>
+      </c>
+      <c r="C356" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D356" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1414_Polo-Care-Tips.md</t>
+        </is>
+      </c>
+      <c r="E356" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F356" s="2" t="inlineStr"/>
+      <c r="G356" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H356" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B357" s="3" t="inlineStr">
+        <is>
+          <t>A8 - Court Sandbox</t>
+        </is>
+      </c>
+      <c r="C357" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D357" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1442_A8-Court-Sandbox.md</t>
+        </is>
+      </c>
+      <c r="E357" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F357" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G357" s="3" t="inlineStr">
+        <is>
+          <t>Owner's disclosure of an arrest and court case to their employer, possible employer responses, and career history referenced as sentencing mitigation.</t>
+        </is>
+      </c>
+      <c r="H357" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B358" s="3" t="inlineStr">
+        <is>
+          <t>A5 - Mental Health Circumstances</t>
+        </is>
+      </c>
+      <c r="C358" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D358" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1511_A5-Mental-Health-Circumstances.md</t>
+        </is>
+      </c>
+      <c r="E358" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F358" s="2" t="inlineStr"/>
+      <c r="G358" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H358" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B359" s="3" t="inlineStr">
+        <is>
+          <t>A5.0 - History</t>
+        </is>
+      </c>
+      <c r="C359" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D359" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1512_A5-0-History.md</t>
+        </is>
+      </c>
+      <c r="E359" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F359" s="2" t="inlineStr"/>
+      <c r="G359" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H359" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B360" s="3" t="inlineStr">
+        <is>
+          <t>A5.1 - Resulting Crisis 2025</t>
+        </is>
+      </c>
+      <c r="C360" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D360" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1513_A5-1-Resulting-Crisis-2025.md</t>
+        </is>
+      </c>
+      <c r="E360" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F360" s="2" t="inlineStr"/>
+      <c r="G360" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H360" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B361" s="3" t="inlineStr">
+        <is>
+          <t>A5.2 - MDD</t>
+        </is>
+      </c>
+      <c r="C361" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D361" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1517_A5-2-MDD.md</t>
+        </is>
+      </c>
+      <c r="E361" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F361" s="2" t="inlineStr"/>
+      <c r="G361" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H361" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B362" s="3" t="inlineStr">
+        <is>
+          <t>A5.3 - MDD EPUT</t>
+        </is>
+      </c>
+      <c r="C362" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D362" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1517_A5-3-MDD-EPUT.md</t>
+        </is>
+      </c>
+      <c r="E362" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F362" s="2" t="inlineStr"/>
+      <c r="G362" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H362" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B363" s="3" t="inlineStr">
+        <is>
+          <t>A5.4 - ADHD Context Layer</t>
+        </is>
+      </c>
+      <c r="C363" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D363" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1518_A5-4-ADHD-Context-Layer.md</t>
+        </is>
+      </c>
+      <c r="E363" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F363" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G363" s="3" t="inlineStr">
+        <is>
+          <t>Summary of how ADHD traits affect the owner's work and work feedback.</t>
+        </is>
+      </c>
+      <c r="H363" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B364" s="3" t="inlineStr">
+        <is>
+          <t>A5.5 - Autism Spectrum Disorder</t>
+        </is>
+      </c>
+      <c r="C364" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D364" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1518_A5-5-Autism-Spectrum-Disorder.md</t>
+        </is>
+      </c>
+      <c r="E364" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F364" s="2" t="inlineStr"/>
+      <c r="G364" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H364" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B365" s="3" t="inlineStr">
+        <is>
+          <t>A5.6 - Substance Use Disorder</t>
+        </is>
+      </c>
+      <c r="C365" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D365" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1518_A5-6-Substance-Use-Disorder.md</t>
+        </is>
+      </c>
+      <c r="E365" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F365" s="2" t="inlineStr"/>
+      <c r="G365" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H365" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B366" s="3" t="inlineStr">
+        <is>
+          <t>A5.7 - Occupational Health</t>
+        </is>
+      </c>
+      <c r="C366" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D366" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1519_A5-7-Occupational-Health.md</t>
+        </is>
+      </c>
+      <c r="E366" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F366" s="2" t="inlineStr"/>
+      <c r="G366" s="3" t="inlineStr">
+        <is>
+          <t>Setting up a layer for occupational health assessments, workplace adjustments and return-to-work material.</t>
+        </is>
+      </c>
+      <c r="H366" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B367" s="3" t="inlineStr">
+        <is>
+          <t>A10 - Project Output</t>
+        </is>
+      </c>
+      <c r="C367" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D367" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1522_A10-Project-Output.md</t>
+        </is>
+      </c>
+      <c r="E367" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F367" s="2" t="inlineStr"/>
+      <c r="G367" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H367" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B368" s="3" t="inlineStr">
+        <is>
+          <t>A6 - Voluntary Interview (Input/Output)</t>
+        </is>
+      </c>
+      <c r="C368" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D368" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1534_A6-Voluntary-Interview-Input-Output.md</t>
+        </is>
+      </c>
+      <c r="E368" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F368" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G368" s="3" t="inlineStr">
+        <is>
+          <t>Work stress, a failed work project, managing an engineering team, return to work and an adjusted job role referenced as context.</t>
+        </is>
+      </c>
+      <c r="H368" s="2" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B369" s="3" t="inlineStr">
+        <is>
+          <t>A9 - {Space Saver}</t>
+        </is>
+      </c>
+      <c r="C369" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D369" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1536_A9-Space-Saver.md</t>
+        </is>
+      </c>
+      <c r="E369" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F369" s="2" t="inlineStr"/>
+      <c r="G369" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H369" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B370" s="3" t="inlineStr">
+        <is>
+          <t>Report Structuring Assistance</t>
+        </is>
+      </c>
+      <c r="C370" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D370" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1657_Report-Structuring-Assistance.md</t>
+        </is>
+      </c>
+      <c r="E370" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F370" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G370" s="3" t="inlineStr">
+        <is>
+          <t>Employment role, workload, a rejected work project and non-disclosure of neurodivergence at work referenced as context.</t>
+        </is>
+      </c>
+      <c r="H370" s="2" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B371" s="3" t="inlineStr">
+        <is>
+          <t>Layer A7 Defence Sandbox</t>
+        </is>
+      </c>
+      <c r="C371" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D371" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1737_Layer-A7-Defence-Sandbox.md</t>
+        </is>
+      </c>
+      <c r="E371" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F371" s="2" t="inlineStr"/>
+      <c r="G371" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H371" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B372" s="3" t="inlineStr">
+        <is>
+          <t>Receipt Acknowledgment</t>
+        </is>
+      </c>
+      <c r="C372" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D372" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1739_Receipt-Acknowledgment.md</t>
+        </is>
+      </c>
+      <c r="E372" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F372" s="2" t="inlineStr"/>
+      <c r="G372" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H372" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B373" s="3" t="inlineStr">
+        <is>
+          <t>Legal Report Preparation</t>
+        </is>
+      </c>
+      <c r="C373" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D373" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_1925_Legal-Report-Preparation.md</t>
+        </is>
+      </c>
+      <c r="E373" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F373" s="2" t="inlineStr"/>
+      <c r="G373" s="3" t="inlineStr">
+        <is>
+          <t>Employment and work-stress context (role, workload, managerial support, project rejection, disclosure at work) within a consolidated legal document.</t>
+        </is>
+      </c>
+      <c r="H373" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B374" s="3" t="inlineStr">
+        <is>
+          <t>Hylands Park Incident Summary</t>
+        </is>
+      </c>
+      <c r="C374" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D374" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_2009_Hylands-Park-Incident-Summary.md</t>
+        </is>
+      </c>
+      <c r="E374" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F374" s="2" t="inlineStr"/>
+      <c r="G374" s="3" t="inlineStr">
+        <is>
+          <t>Employment and work-stress context (role, workload, managerial support, project rejection, disclosure at work) within a restructured legal document.</t>
+        </is>
+      </c>
+      <c r="H374" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B375" s="3" t="inlineStr">
+        <is>
+          <t>ASD Childhood Reflection</t>
+        </is>
+      </c>
+      <c r="C375" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D375" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_2041_ASD-Childhood-Reflection.md</t>
+        </is>
+      </c>
+      <c r="E375" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F375" s="2" t="inlineStr"/>
+      <c r="G375" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H375" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B376" s="3" t="inlineStr">
+        <is>
+          <t>Document Analysis Overview</t>
+        </is>
+      </c>
+      <c r="C376" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D376" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03_2202_Document-Analysis-Overview.md</t>
+        </is>
+      </c>
+      <c r="E376" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F376" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G376" s="3" t="inlineStr">
+        <is>
+          <t>Brief references to occupational stress as a contributing factor in a consolidated legal reference document.</t>
+        </is>
+      </c>
+      <c r="H376" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-04</t>
+        </is>
+      </c>
+      <c r="B377" s="3" t="inlineStr">
+        <is>
+          <t>Clinical Diagnostic Documentation</t>
+        </is>
+      </c>
+      <c r="C377" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D377" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-04_0044_Clinical-Diagnostic-Documentation.md</t>
+        </is>
+      </c>
+      <c r="E377" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F377" s="2" t="inlineStr"/>
+      <c r="G377" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H377" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B378" s="3" t="inlineStr">
+        <is>
+          <t>ICB Oversight Request</t>
+        </is>
+      </c>
+      <c r="C378" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D378" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05_0959_ICB-Oversight-Request.md</t>
+        </is>
+      </c>
+      <c r="E378" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F378" s="2" t="inlineStr"/>
+      <c r="G378" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H378" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B379" s="3" t="inlineStr">
+        <is>
+          <t>ASD Assessment Deferral Request</t>
+        </is>
+      </c>
+      <c r="C379" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D379" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05_1315_ASD-Assessment-Deferral-Request.md</t>
+        </is>
+      </c>
+      <c r="E379" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F379" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G379" s="3" t="inlineStr">
+        <is>
+          <t>Return to work cited as one of the pressures in a request to defer an appointment.</t>
+        </is>
+      </c>
+      <c r="H379" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B380" s="3" t="inlineStr">
+        <is>
+          <t>Chip Resistor Value 01B</t>
+        </is>
+      </c>
+      <c r="C380" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D380" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05_1501_Chip-Resistor-Value-01B.md</t>
+        </is>
+      </c>
+      <c r="E380" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F380" s="2" t="inlineStr"/>
+      <c r="G380" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H380" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B381" s="3" t="inlineStr">
+        <is>
+          <t>Log Cabin Price Comparison</t>
+        </is>
+      </c>
+      <c r="C381" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D381" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05_1637_Log-Cabin-Price-Comparison.md</t>
+        </is>
+      </c>
+      <c r="E381" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F381" s="2" t="inlineStr"/>
+      <c r="G381" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H381" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B382" s="3" t="inlineStr">
+        <is>
+          <t>ICB Report Paragraph</t>
+        </is>
+      </c>
+      <c r="C382" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D382" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05_1807_ICB-Report-Paragraph.md</t>
+        </is>
+      </c>
+      <c r="E382" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F382" s="2" t="inlineStr"/>
+      <c r="G382" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H382" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B383" s="3" t="inlineStr">
+        <is>
+          <t>Statement for ICB Review</t>
+        </is>
+      </c>
+      <c r="C383" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D383" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05_1813_Statement-for-ICB-Review.md</t>
+        </is>
+      </c>
+      <c r="E383" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F383" s="2" t="inlineStr"/>
+      <c r="G383" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H383" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B384" s="3" t="inlineStr">
+        <is>
+          <t>Document Tidy Up</t>
+        </is>
+      </c>
+      <c r="C384" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D384" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05_1829_Document-Tidy-Up.md</t>
+        </is>
+      </c>
+      <c r="E384" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F384" s="2" t="inlineStr"/>
+      <c r="G384" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H384" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H320"/>
+  <autoFilter ref="A1:H384"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12316,7 +14660,7 @@
         </is>
       </c>
       <c r="B1" t="n">
-        <v>319</v>
+        <v>383</v>
       </c>
     </row>
     <row r="2">
@@ -12326,7 +14670,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3">
@@ -12336,7 +14680,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>42</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4">
@@ -12346,7 +14690,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>82</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5">
@@ -12356,7 +14700,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>237</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
chat-sift: batches b50-b59 read; index, extracts and progress updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aq7txTcfpUgzabiqqnXaKj
</commit_message>
<xml_diff>
--- a/chat-sift/output/index.xlsx
+++ b/chat-sift/output/index.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$384</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$452</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H384"/>
+  <dimension ref="A1:H452"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14635,8 +14635,2552 @@
         <v>0</v>
       </c>
     </row>
+    <row r="385">
+      <c r="A385" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B385" s="3" t="inlineStr">
+        <is>
+          <t>Read-only Mode Setup</t>
+        </is>
+      </c>
+      <c r="C385" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D385" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05_2012_Read-only-Mode-Setup.md</t>
+        </is>
+      </c>
+      <c r="E385" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F385" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G385" s="3" t="inlineStr">
+        <is>
+          <t>Brief mentions of awaiting a team leader's acknowledgement before travel and taking an afternoon off work for a review appointment.</t>
+        </is>
+      </c>
+      <c r="H385" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B386" s="3" t="inlineStr">
+        <is>
+          <t>Simplified Document Overview</t>
+        </is>
+      </c>
+      <c r="C386" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D386" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05_2106_Simplified-Document-Overview.md</t>
+        </is>
+      </c>
+      <c r="E386" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F386" s="2" t="inlineStr"/>
+      <c r="G386" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H386" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B387" s="3" t="inlineStr">
+        <is>
+          <t>ICB Oversight Request Summary</t>
+        </is>
+      </c>
+      <c r="C387" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D387" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05_2116_ICB-Oversight-Request-Summary.md</t>
+        </is>
+      </c>
+      <c r="E387" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F387" s="2" t="inlineStr"/>
+      <c r="G387" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H387" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B388" s="3" t="inlineStr">
+        <is>
+          <t>ICB Submission Review</t>
+        </is>
+      </c>
+      <c r="C388" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D388" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05_2144_ICB-Submission-Review.md</t>
+        </is>
+      </c>
+      <c r="E388" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F388" s="2" t="inlineStr"/>
+      <c r="G388" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H388" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B389" s="3" t="inlineStr">
+        <is>
+          <t>Cutting Interlocking Spurs</t>
+        </is>
+      </c>
+      <c r="C389" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D389" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05_2220_Cutting-Interlocking-Spurs.md</t>
+        </is>
+      </c>
+      <c r="E389" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F389" s="2" t="inlineStr"/>
+      <c r="G389" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H389" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-06</t>
+        </is>
+      </c>
+      <c r="B390" s="3" t="inlineStr">
+        <is>
+          <t>Psychologist Report Review</t>
+        </is>
+      </c>
+      <c r="C390" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D390" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-06_0822_Psychologist-Report-Review.md</t>
+        </is>
+      </c>
+      <c r="E390" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F390" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G390" s="3" t="inlineStr">
+        <is>
+          <t>Brief passages on how a clinical report addresses occupational functional impact, occupational health and reasonable adjustments.</t>
+        </is>
+      </c>
+      <c r="H390" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-06</t>
+        </is>
+      </c>
+      <c r="B391" s="3" t="inlineStr">
+        <is>
+          <t>Explaining Exhaustion to HR</t>
+        </is>
+      </c>
+      <c r="C391" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D391" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-06_1040_Explaining-Exhaustion-to-HR.md</t>
+        </is>
+      </c>
+      <c r="E391" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F391" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G391" s="3" t="inlineStr">
+        <is>
+          <t>Reasonable adjustment requests to HR and line management on working pattern, HR responses, related documentation, and concerns about HR communication.</t>
+        </is>
+      </c>
+      <c r="H391" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-06</t>
+        </is>
+      </c>
+      <c r="B392" s="3" t="inlineStr">
+        <is>
+          <t>Medicash Proof of Purchase</t>
+        </is>
+      </c>
+      <c r="C392" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D392" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-06_1527_Medicash-Proof-of-Purchase.md</t>
+        </is>
+      </c>
+      <c r="E392" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F392" s="2" t="inlineStr"/>
+      <c r="G392" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H392" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B393" s="3" t="inlineStr">
+        <is>
+          <t>GMC Register Explanation</t>
+        </is>
+      </c>
+      <c r="C393" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D393" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-07_0733_GMC-Register-Explanation.md</t>
+        </is>
+      </c>
+      <c r="E393" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F393" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G393" s="3" t="inlineStr">
+        <is>
+          <t>Obtaining the benefit table for an employer-provided Medicash cash plan scheme, including via HR or the scheme administrator.</t>
+        </is>
+      </c>
+      <c r="H393" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B394" s="3" t="inlineStr">
+        <is>
+          <t>ICB Report Consolidation</t>
+        </is>
+      </c>
+      <c r="C394" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D394" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-07_1023_ICB-Report-Consolidation.md</t>
+        </is>
+      </c>
+      <c r="E394" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F394" s="2" t="inlineStr"/>
+      <c r="G394" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H394" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B395" s="3" t="inlineStr">
+        <is>
+          <t>Flea Bite or Not</t>
+        </is>
+      </c>
+      <c r="C395" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D395" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-07_1823_Flea-Bite-or-Not.md</t>
+        </is>
+      </c>
+      <c r="E395" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F395" s="2" t="inlineStr"/>
+      <c r="G395" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H395" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B396" s="3" t="inlineStr">
+        <is>
+          <t>Highest Poe Level</t>
+        </is>
+      </c>
+      <c r="C396" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D396" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-07_2021_Highest-Poe-Level.md</t>
+        </is>
+      </c>
+      <c r="E396" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F396" s="2" t="inlineStr"/>
+      <c r="G396" s="3" t="inlineStr">
+        <is>
+          <t>Engineering design discussion for a PoE power and control retrofit of the team's existing HTOL test ovens and module electronics.</t>
+        </is>
+      </c>
+      <c r="H396" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-08</t>
+        </is>
+      </c>
+      <c r="B397" s="3" t="inlineStr">
+        <is>
+          <t>NHS Right to Choose Depression</t>
+        </is>
+      </c>
+      <c r="C397" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D397" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-08_1121_NHS-Right-to-Choose-Depression.md</t>
+        </is>
+      </c>
+      <c r="E397" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F397" s="2" t="inlineStr"/>
+      <c r="G397" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H397" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-08</t>
+        </is>
+      </c>
+      <c r="B398" s="3" t="inlineStr">
+        <is>
+          <t>Diode failure vs ADC issue</t>
+        </is>
+      </c>
+      <c r="C398" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D398" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-08_1524_Diode-failure-vs-ADC-issue.md</t>
+        </is>
+      </c>
+      <c r="E398" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F398" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G398" s="3" t="inlineStr">
+        <is>
+          <t>Bench fault-finding on an electronics board (clamp diode, ADC input and x11 gain branch via relay), possibly part of the owner's job.</t>
+        </is>
+      </c>
+      <c r="H398" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-08</t>
+        </is>
+      </c>
+      <c r="B399" s="3" t="inlineStr">
+        <is>
+          <t>Nature and Global Warming</t>
+        </is>
+      </c>
+      <c r="C399" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D399" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-08_1653_Nature-and-Global-Warming.md</t>
+        </is>
+      </c>
+      <c r="E399" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F399" s="2" t="inlineStr"/>
+      <c r="G399" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H399" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-09</t>
+        </is>
+      </c>
+      <c r="B400" s="3" t="inlineStr">
+        <is>
+          <t>Power-on Transients vs Monotonic</t>
+        </is>
+      </c>
+      <c r="C400" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D400" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-09_1358_Power-on-Transients-vs-Monotonic.md</t>
+        </is>
+      </c>
+      <c r="E400" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F400" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G400" s="3" t="inlineStr">
+        <is>
+          <t>Electronics engineering question on power-on transients versus a monotonic power-on edge, possibly related to the owner's job.</t>
+        </is>
+      </c>
+      <c r="H400" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-09</t>
+        </is>
+      </c>
+      <c r="B401" s="3" t="inlineStr">
+        <is>
+          <t>Surviving Toxic Workplaces</t>
+        </is>
+      </c>
+      <c r="C401" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-003.json</t>
+        </is>
+      </c>
+      <c r="D401" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-09_1905_Surviving-Toxic-Workplaces.md</t>
+        </is>
+      </c>
+      <c r="E401" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F401" s="2" t="inlineStr"/>
+      <c r="G401" s="3" t="inlineStr">
+        <is>
+          <t>Coping with a perceived toxic workplace and keeping an evidence trail of being ignored at work.</t>
+        </is>
+      </c>
+      <c r="H401" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-09</t>
+        </is>
+      </c>
+      <c r="B402" s="3" t="inlineStr">
+        <is>
+          <t>Z  - Pre-Project (PP) chat</t>
+        </is>
+      </c>
+      <c r="C402" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D402" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-09_2131_Z-Pre-Project-PP-chat.md</t>
+        </is>
+      </c>
+      <c r="E402" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F402" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G402" s="3" t="inlineStr">
+        <is>
+          <t>Employer response to an Occupational Health report, return to work after sickness absence, reasonable adjustments, working pattern and leave requests, workload tracking, communication with manager and HR, appraisal drafting and a request for regular 1:1s.</t>
+        </is>
+      </c>
+      <c r="H402" s="2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B403" s="3" t="inlineStr">
+        <is>
+          <t>Shark CarpetXpert Model Identification</t>
+        </is>
+      </c>
+      <c r="C403" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D403" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-10_0514_Shark-CarpetXpert-Model-Identification.md</t>
+        </is>
+      </c>
+      <c r="E403" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F403" s="2" t="inlineStr"/>
+      <c r="G403" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H403" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B404" s="3" t="inlineStr">
+        <is>
+          <t>Log Cabin Wall Stack</t>
+        </is>
+      </c>
+      <c r="C404" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D404" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-10_1042_Log-Cabin-Wall-Stack.md</t>
+        </is>
+      </c>
+      <c r="E404" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F404" s="2" t="inlineStr"/>
+      <c r="G404" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H404" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B405" s="3" t="inlineStr">
+        <is>
+          <t>Merge graphics request</t>
+        </is>
+      </c>
+      <c r="C405" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D405" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-10_1419_Merge-graphics-request.md</t>
+        </is>
+      </c>
+      <c r="E405" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F405" s="2" t="inlineStr"/>
+      <c r="G405" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H405" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B406" s="3" t="inlineStr">
+        <is>
+          <t>Project Charter</t>
+        </is>
+      </c>
+      <c r="C406" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D406" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-10_1723_Project-Charter.md</t>
+        </is>
+      </c>
+      <c r="E406" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F406" s="2" t="inlineStr"/>
+      <c r="G406" s="3" t="inlineStr">
+        <is>
+          <t>Setting up a structured project, log and evidence repository for managing role stability at work after a health-related role transition.</t>
+        </is>
+      </c>
+      <c r="H406" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B407" s="3" t="inlineStr">
+        <is>
+          <t>1 - Role Stability Project Control</t>
+        </is>
+      </c>
+      <c r="C407" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D407" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-10_1757_1-Role-Stability-Project-Control.md</t>
+        </is>
+      </c>
+      <c r="E407" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F407" s="2" t="inlineStr"/>
+      <c r="G407" s="3" t="inlineStr">
+        <is>
+          <t>Opening statement for a control chat governing the work role stability project.</t>
+        </is>
+      </c>
+      <c r="H407" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B408" s="3" t="inlineStr">
+        <is>
+          <t>3 - Factual Log Assessment</t>
+        </is>
+      </c>
+      <c r="C408" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D408" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-10_1759_3-Factual-Log-Assessment.md</t>
+        </is>
+      </c>
+      <c r="E408" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F408" s="2" t="inlineStr"/>
+      <c r="G408" s="3" t="inlineStr">
+        <is>
+          <t>Setting up and using a factual log for the work role stability project.</t>
+        </is>
+      </c>
+      <c r="H408" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-11</t>
+        </is>
+      </c>
+      <c r="B409" s="3" t="inlineStr">
+        <is>
+          <t>Facebook Algorithm Explanation</t>
+        </is>
+      </c>
+      <c r="C409" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D409" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-11_1539_Facebook-Algorithm-Explanation.md</t>
+        </is>
+      </c>
+      <c r="E409" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F409" s="2" t="inlineStr"/>
+      <c r="G409" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H409" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-11</t>
+        </is>
+      </c>
+      <c r="B410" s="3" t="inlineStr">
+        <is>
+          <t>Gain Calibration Frequency</t>
+        </is>
+      </c>
+      <c r="C410" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D410" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-11_1654_Gain-Calibration-Frequency.md</t>
+        </is>
+      </c>
+      <c r="E410" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F410" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G410" s="3" t="inlineStr">
+        <is>
+          <t>Electronics engineering questions on gain calibration and RC filter values, likely relating to the owner's engineering role.</t>
+        </is>
+      </c>
+      <c r="H410" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-11</t>
+        </is>
+      </c>
+      <c r="B411" s="3" t="inlineStr">
+        <is>
+          <t>Velcro Placement Advice</t>
+        </is>
+      </c>
+      <c r="C411" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D411" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-11_1803_Velcro-Placement-Advice.md</t>
+        </is>
+      </c>
+      <c r="E411" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F411" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G411" s="3" t="inlineStr">
+        <is>
+          <t>Attaching a notepad to the owner's work folder.</t>
+        </is>
+      </c>
+      <c r="H411" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-11</t>
+        </is>
+      </c>
+      <c r="B412" s="3" t="inlineStr">
+        <is>
+          <t>Lighthouse CON-100G2 Wheel</t>
+        </is>
+      </c>
+      <c r="C412" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D412" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-11_2236_Lighthouse-CON-100G2-Wheel.md</t>
+        </is>
+      </c>
+      <c r="E412" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F412" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G412" s="3" t="inlineStr">
+        <is>
+          <t>Identifying an adjustment wheel on a printer, possibly work equipment.</t>
+        </is>
+      </c>
+      <c r="H412" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B413" s="3" t="inlineStr">
+        <is>
+          <t>LVDS 14m Cable Requirements</t>
+        </is>
+      </c>
+      <c r="C413" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D413" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-12_1820_LVDS-14m-Cable-Requirements.md</t>
+        </is>
+      </c>
+      <c r="E413" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F413" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G413" s="3" t="inlineStr">
+        <is>
+          <t>Engineering design question on driving LVDS over a 14m cable from an FPGA module, likely relating to the owner's engineering role.</t>
+        </is>
+      </c>
+      <c r="H413" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B414" s="3" t="inlineStr">
+        <is>
+          <t>B1 First Hearing Guilty</t>
+        </is>
+      </c>
+      <c r="C414" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D414" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13_0953_B1-First-Hearing-Guilty.md</t>
+        </is>
+      </c>
+      <c r="E414" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F414" s="2" t="inlineStr"/>
+      <c r="G414" s="3" t="inlineStr">
+        <is>
+          <t>Work overload, time off work, phased return and stepping down from team leadership raised as context.</t>
+        </is>
+      </c>
+      <c r="H414" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B415" s="3" t="inlineStr">
+        <is>
+          <t>ADC Output Sampling Issue</t>
+        </is>
+      </c>
+      <c r="C415" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D415" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13_0957_ADC-Output-Sampling-Issue.md</t>
+        </is>
+      </c>
+      <c r="E415" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F415" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G415" s="3" t="inlineStr">
+        <is>
+          <t>Engineering troubleshooting of an ADC output sampling issue, likely relating to the owner's engineering role.</t>
+        </is>
+      </c>
+      <c r="H415" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B416" s="3" t="inlineStr">
+        <is>
+          <t>ADC Histogram Analysis</t>
+        </is>
+      </c>
+      <c r="C416" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D416" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13_0958_ADC-Histogram-Analysis.md</t>
+        </is>
+      </c>
+      <c r="E416" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F416" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G416" s="3" t="inlineStr">
+        <is>
+          <t>Engineering analysis of ADC histogram results across two systems, likely relating to the owner's engineering role.</t>
+        </is>
+      </c>
+      <c r="H416" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B417" s="3" t="inlineStr">
+        <is>
+          <t>CCTV Realisation and Accountability</t>
+        </is>
+      </c>
+      <c r="C417" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D417" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13_1107_CCTV-Realisation-and-Accountability.md</t>
+        </is>
+      </c>
+      <c r="E417" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F417" s="2" t="inlineStr"/>
+      <c r="G417" s="3" t="inlineStr">
+        <is>
+          <t>Work boundaries, time off work, phased return and stepping down from a senior role at work referenced as context.</t>
+        </is>
+      </c>
+      <c r="H417" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B418" s="3" t="inlineStr">
+        <is>
+          <t>Court Day Guidance</t>
+        </is>
+      </c>
+      <c r="C418" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D418" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13_1134_Court-Day-Guidance.md</t>
+        </is>
+      </c>
+      <c r="E418" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F418" s="2" t="inlineStr"/>
+      <c r="G418" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H418" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B419" s="3" t="inlineStr">
+        <is>
+          <t>Missed Station Confusion</t>
+        </is>
+      </c>
+      <c r="C419" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D419" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13_1250_Missed-Station-Confusion.md</t>
+        </is>
+      </c>
+      <c r="E419" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F419" s="2" t="inlineStr"/>
+      <c r="G419" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H419" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B420" s="3" t="inlineStr">
+        <is>
+          <t>Court Appointment Reminder</t>
+        </is>
+      </c>
+      <c r="C420" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D420" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13_1251_Court-Appointment-Reminder.md</t>
+        </is>
+      </c>
+      <c r="E420" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F420" s="2" t="inlineStr"/>
+      <c r="G420" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H420" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B421" s="3" t="inlineStr">
+        <is>
+          <t>Exporting Teams Chats</t>
+        </is>
+      </c>
+      <c r="C421" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D421" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13_1726_Exporting-Teams-Chats.md</t>
+        </is>
+      </c>
+      <c r="E421" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F421" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G421" s="3" t="inlineStr">
+        <is>
+          <t>Exporting Microsoft Teams chats with timestamps and capturing screenshots as a record, including eDiscovery and subject access routes.</t>
+        </is>
+      </c>
+      <c r="H421" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B422" s="3" t="inlineStr">
+        <is>
+          <t>Hotkey for scroll down</t>
+        </is>
+      </c>
+      <c r="C422" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D422" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13_1817_Hotkey-for-scroll-down.md</t>
+        </is>
+      </c>
+      <c r="E422" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F422" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G422" s="3" t="inlineStr">
+        <is>
+          <t>Keyboard shortcuts for scrolling in Microsoft Teams chat.</t>
+        </is>
+      </c>
+      <c r="H422" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B423" s="3" t="inlineStr">
+        <is>
+          <t>Efficient Screenshot Transcription</t>
+        </is>
+      </c>
+      <c r="C423" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D423" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13_1951_Efficient-Screenshot-Transcription.md</t>
+        </is>
+      </c>
+      <c r="E423" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F423" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G423" s="3" t="inlineStr">
+        <is>
+          <t>Workflow for transcribing a large number of screenshots, possibly of workplace messages.</t>
+        </is>
+      </c>
+      <c r="H423" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B424" s="3" t="inlineStr">
+        <is>
+          <t>Office 365 Work Toggle</t>
+        </is>
+      </c>
+      <c r="C424" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D424" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13_2122_Office-365-Work-Toggle.md</t>
+        </is>
+      </c>
+      <c r="E424" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F424" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G424" s="3" t="inlineStr">
+        <is>
+          <t>Meaning of the Work account toggle in Office 365 and employer visibility of documents.</t>
+        </is>
+      </c>
+      <c r="H424" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B425" s="3" t="inlineStr">
+        <is>
+          <t>Test Electronics Checklist</t>
+        </is>
+      </c>
+      <c r="C425" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D425" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13_2142_Test-Electronics-Checklist.md</t>
+        </is>
+      </c>
+      <c r="E425" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F425" s="2" t="inlineStr"/>
+      <c r="G425" s="3" t="inlineStr">
+        <is>
+          <t>Developing a system requirements checklist, library part checklist and SRR pre-gate documentation for imaging sensor test electronics.</t>
+        </is>
+      </c>
+      <c r="H425" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B426" s="3" t="inlineStr">
+        <is>
+          <t>Library Part Checklist Excel</t>
+        </is>
+      </c>
+      <c r="C426" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D426" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13_2214_Library-Part-Checklist-Excel.md</t>
+        </is>
+      </c>
+      <c r="E426" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F426" s="2" t="inlineStr"/>
+      <c r="G426" s="3" t="inlineStr">
+        <is>
+          <t>Converting a library part checklist for electronics design into an Excel spreadsheet.</t>
+        </is>
+      </c>
+      <c r="H426" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B427" s="3" t="inlineStr">
+        <is>
+          <t>Electronics MRR Lifecycle Gate</t>
+        </is>
+      </c>
+      <c r="C427" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D427" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13_2216_Electronics-MRR-Lifecycle-Gate.md</t>
+        </is>
+      </c>
+      <c r="E427" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F427" s="2" t="inlineStr"/>
+      <c r="G427" s="3" t="inlineStr">
+        <is>
+          <t>Defining an electronics manufacturing readiness review (MRR) lifecycle gate checklist.</t>
+        </is>
+      </c>
+      <c r="H427" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B428" s="3" t="inlineStr">
+        <is>
+          <t>Exceeding Expectations and Stress</t>
+        </is>
+      </c>
+      <c r="C428" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D428" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-13_2245_Exceeding-Expectations-and-Stress.md</t>
+        </is>
+      </c>
+      <c r="E428" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F428" s="2" t="inlineStr"/>
+      <c r="G428" s="3" t="inlineStr">
+        <is>
+          <t>Appraisal ratings, expectations, a prior needs-improvement rating linked to an email, and the effect of workload on mental health.</t>
+        </is>
+      </c>
+      <c r="H428" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B429" s="3" t="inlineStr">
+        <is>
+          <t>Multiplexing Gain Cal Output</t>
+        </is>
+      </c>
+      <c r="C429" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D429" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14_0048_Multiplexing-Gain-Cal-Output.md</t>
+        </is>
+      </c>
+      <c r="E429" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F429" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G429" s="3" t="inlineStr">
+        <is>
+          <t>Technical design question on multiplexing a gain calibration output across video chains and channel selection circuitry.</t>
+        </is>
+      </c>
+      <c r="H429" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B430" s="3" t="inlineStr">
+        <is>
+          <t>Altium Report +5V Components</t>
+        </is>
+      </c>
+      <c r="C430" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D430" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14_0102_Altium-Report-5V-Components.md</t>
+        </is>
+      </c>
+      <c r="E430" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F430" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G430" s="3" t="inlineStr">
+        <is>
+          <t>Technical question on generating an Altium Designer report of components on a supply rail.</t>
+        </is>
+      </c>
+      <c r="H430" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B431" s="3" t="inlineStr">
+        <is>
+          <t>Single-ended to LVDS Conversion</t>
+        </is>
+      </c>
+      <c r="C431" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D431" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14_1205_Single-ended-to-LVDS-Conversion.md</t>
+        </is>
+      </c>
+      <c r="E431" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F431" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G431" s="3" t="inlineStr">
+        <is>
+          <t>Technical question on driving an LVDS signal from a single-ended input.</t>
+        </is>
+      </c>
+      <c r="H431" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B432" s="3" t="inlineStr">
+        <is>
+          <t>Parent's Emotional Response Analysis</t>
+        </is>
+      </c>
+      <c r="C432" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D432" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14_1305_Parent-s-Emotional-Response-Analysis.md</t>
+        </is>
+      </c>
+      <c r="E432" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F432" s="2" t="inlineStr"/>
+      <c r="G432" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H432" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B433" s="3" t="inlineStr">
+        <is>
+          <t>Appraisal Chat Guidance</t>
+        </is>
+      </c>
+      <c r="C433" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D433" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14_1453_Appraisal-Chat-Guidance.md</t>
+        </is>
+      </c>
+      <c r="E433" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F433" s="2" t="inlineStr"/>
+      <c r="G433" s="3" t="inlineStr">
+        <is>
+          <t>Drafting appraisal self-assessment statements and grades for work objectives.</t>
+        </is>
+      </c>
+      <c r="H433" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B434" s="3" t="inlineStr">
+        <is>
+          <t>Nails complaint summary</t>
+        </is>
+      </c>
+      <c r="C434" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D434" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14_1458_Nails-complaint-summary.md</t>
+        </is>
+      </c>
+      <c r="E434" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F434" s="2" t="inlineStr"/>
+      <c r="G434" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H434" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B435" s="3" t="inlineStr">
+        <is>
+          <t>New chat</t>
+        </is>
+      </c>
+      <c r="C435" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D435" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-15_0847_New-chat.md</t>
+        </is>
+      </c>
+      <c r="E435" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F435" s="2" t="inlineStr"/>
+      <c r="G435" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H435" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B436" s="3" t="inlineStr">
+        <is>
+          <t>Test Retake Clarification</t>
+        </is>
+      </c>
+      <c r="C436" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D436" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-15_1610_Test-Retake-Clarification.md</t>
+        </is>
+      </c>
+      <c r="E436" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F436" s="2" t="inlineStr"/>
+      <c r="G436" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H436" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B437" s="3" t="inlineStr">
+        <is>
+          <t>Objective Review Revision</t>
+        </is>
+      </c>
+      <c r="C437" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D437" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-15_1835_Objective-Review-Revision.md</t>
+        </is>
+      </c>
+      <c r="E437" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F437" s="2" t="inlineStr"/>
+      <c r="G437" s="3" t="inlineStr">
+        <is>
+          <t>Wording an appraisal objective review for a not-achieved delivery objective and a communication competency statement.</t>
+        </is>
+      </c>
+      <c r="H437" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B438" s="3" t="inlineStr">
+        <is>
+          <t>Appraisal Risk Management</t>
+        </is>
+      </c>
+      <c r="C438" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D438" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-15_1843_Appraisal-Risk-Management.md</t>
+        </is>
+      </c>
+      <c r="E438" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F438" s="2" t="inlineStr"/>
+      <c r="G438" s="3" t="inlineStr">
+        <is>
+          <t>Approach to an upcoming appraisal and costs and returns of a constructive dismissal claim.</t>
+        </is>
+      </c>
+      <c r="H438" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B439" s="3" t="inlineStr">
+        <is>
+          <t>Final Review Summary</t>
+        </is>
+      </c>
+      <c r="C439" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D439" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-15_2047_Final-Review-Summary.md</t>
+        </is>
+      </c>
+      <c r="E439" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F439" s="2" t="inlineStr"/>
+      <c r="G439" s="3" t="inlineStr">
+        <is>
+          <t>Final rewrite of performance review objectives, document references and competency summaries.</t>
+        </is>
+      </c>
+      <c r="H439" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B440" s="3" t="inlineStr">
+        <is>
+          <t>Friction in Design Documentation</t>
+        </is>
+      </c>
+      <c r="C440" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D440" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-15_2126_Friction-in-Design-Documentation.md</t>
+        </is>
+      </c>
+      <c r="E440" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F440" s="2" t="inlineStr"/>
+      <c r="G440" s="3" t="inlineStr">
+        <is>
+          <t>Analysis of where friction arose in a work design documentation review milestone.</t>
+        </is>
+      </c>
+      <c r="H440" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B441" s="3" t="inlineStr">
+        <is>
+          <t>Remove Zeros in Excel</t>
+        </is>
+      </c>
+      <c r="C441" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D441" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16_0140_Remove-Zeros-in-Excel.md</t>
+        </is>
+      </c>
+      <c r="E441" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F441" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G441" s="3" t="inlineStr">
+        <is>
+          <t>Excel help for a requirements compliance checklist spreadsheet.</t>
+        </is>
+      </c>
+      <c r="H441" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B442" s="3" t="inlineStr">
+        <is>
+          <t>Library Checklist Examples</t>
+        </is>
+      </c>
+      <c r="C442" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D442" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16_0306_Library-Checklist-Examples.md</t>
+        </is>
+      </c>
+      <c r="E442" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F442" s="2" t="inlineStr"/>
+      <c r="G442" s="3" t="inlineStr">
+        <is>
+          <t>Screenshot evidence and worked example for a PCB component library checklist.</t>
+        </is>
+      </c>
+      <c r="H442" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B443" s="3" t="inlineStr">
+        <is>
+          <t>Excel Conditional Formatting</t>
+        </is>
+      </c>
+      <c r="C443" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D443" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16_0318_Excel-Conditional-Formatting.md</t>
+        </is>
+      </c>
+      <c r="E443" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F443" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G443" s="3" t="inlineStr">
+        <is>
+          <t>Excel conditional formatting help, possibly for a work checklist.</t>
+        </is>
+      </c>
+      <c r="H443" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B444" s="3" t="inlineStr">
+        <is>
+          <t>Excel OR Formula Explained</t>
+        </is>
+      </c>
+      <c r="C444" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D444" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16_0339_Excel-OR-Formula-Explained.md</t>
+        </is>
+      </c>
+      <c r="E444" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F444" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G444" s="3" t="inlineStr">
+        <is>
+          <t>Excel OR formula help, possibly for a work checklist.</t>
+        </is>
+      </c>
+      <c r="H444" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B445" s="3" t="inlineStr">
+        <is>
+          <t>Sampling Rate Explanation</t>
+        </is>
+      </c>
+      <c r="C445" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D445" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16_0721_Sampling-Rate-Explanation.md</t>
+        </is>
+      </c>
+      <c r="E445" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F445" s="2" t="inlineStr"/>
+      <c r="G445" s="3" t="inlineStr">
+        <is>
+          <t>Drafting requirement rationale text and column headings for a technical requirements matrix for a CCD FEE test system.</t>
+        </is>
+      </c>
+      <c r="H445" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B446" s="3" t="inlineStr">
+        <is>
+          <t>Interest rate drop explanation</t>
+        </is>
+      </c>
+      <c r="C446" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D446" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-18_1147_Interest-rate-drop-explanation.md</t>
+        </is>
+      </c>
+      <c r="E446" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F446" s="2" t="inlineStr"/>
+      <c r="G446" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H446" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B447" s="3" t="inlineStr">
+        <is>
+          <t>Positive Treatment Response Help</t>
+        </is>
+      </c>
+      <c r="C447" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D447" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-18_1259_Positive-Treatment-Response-Help.md</t>
+        </is>
+      </c>
+      <c r="E447" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F447" s="2" t="inlineStr"/>
+      <c r="G447" s="3" t="inlineStr">
+        <is>
+          <t>Describing progress against a work-related goal (task focus, time management, delivery) in a treatment review.</t>
+        </is>
+      </c>
+      <c r="H447" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B448" s="3" t="inlineStr">
+        <is>
+          <t>Concatenate Cells in Excel</t>
+        </is>
+      </c>
+      <c r="C448" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D448" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-18_2211_Concatenate-Cells-in-Excel.md</t>
+        </is>
+      </c>
+      <c r="E448" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F448" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G448" s="3" t="inlineStr">
+        <is>
+          <t>Excel formula question that may relate to a work spreadsheet.</t>
+        </is>
+      </c>
+      <c r="H448" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B449" s="3" t="inlineStr">
+        <is>
+          <t>Guitar course in February</t>
+        </is>
+      </c>
+      <c r="C449" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D449" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-19_1314_Guitar-course-in-February.md</t>
+        </is>
+      </c>
+      <c r="E449" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F449" s="2" t="inlineStr"/>
+      <c r="G449" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H449" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B450" s="3" t="inlineStr">
+        <is>
+          <t>Email drafting assistance</t>
+        </is>
+      </c>
+      <c r="C450" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D450" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-19_1823_Email-drafting-assistance.md</t>
+        </is>
+      </c>
+      <c r="E450" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F450" s="2" t="inlineStr"/>
+      <c r="G450" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H450" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B451" s="3" t="inlineStr">
+        <is>
+          <t>LVDS Interface Options</t>
+        </is>
+      </c>
+      <c r="C451" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D451" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20_0931_LVDS-Interface-Options.md</t>
+        </is>
+      </c>
+      <c r="E451" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F451" s="2" t="inlineStr"/>
+      <c r="G451" s="3" t="inlineStr">
+        <is>
+          <t>Engineering design discussion of a long-distance LVDS/CoaXPress interface for a work project and proposing it internally.</t>
+        </is>
+      </c>
+      <c r="H451" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B452" s="3" t="inlineStr">
+        <is>
+          <t>Navigating Work Challenges</t>
+        </is>
+      </c>
+      <c r="C452" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D452" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20_1029_Navigating-Work-Challenges.md</t>
+        </is>
+      </c>
+      <c r="E452" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F452" s="2" t="inlineStr"/>
+      <c r="G452" s="3" t="inlineStr">
+        <is>
+          <t>Setting up a framework to document and navigate a difficult period at work.</t>
+        </is>
+      </c>
+      <c r="H452" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H384"/>
+  <autoFilter ref="A1:H452"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14660,7 +17204,7 @@
         </is>
       </c>
       <c r="B1" t="n">
-        <v>383</v>
+        <v>451</v>
       </c>
     </row>
     <row r="2">
@@ -14670,7 +17214,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>42</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3">
@@ -14680,7 +17224,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4">
@@ -14690,7 +17234,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>97</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5">
@@ -14700,7 +17244,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>286</v>
+        <v>309</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
chat-sift: batches b60-b69 read; index, extracts and progress updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aq7txTcfpUgzabiqqnXaKj
</commit_message>
<xml_diff>
--- a/chat-sift/output/index.xlsx
+++ b/chat-sift/output/index.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$452</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$520</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H452"/>
+  <dimension ref="A1:H520"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17179,8 +17179,2524 @@
         <v>1</v>
       </c>
     </row>
+    <row r="453">
+      <c r="A453" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B453" s="3" t="inlineStr">
+        <is>
+          <t>4 - Appraisal</t>
+        </is>
+      </c>
+      <c r="C453" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D453" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20_1032_4-Appraisal.md</t>
+        </is>
+      </c>
+      <c r="E453" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F453" s="2" t="inlineStr"/>
+      <c r="G453" s="3" t="inlineStr">
+        <is>
+          <t>Appraisal strategy and challenge of a communication competency rating, OH report handling by HR, phased return, and constructive dismissal contingency.</t>
+        </is>
+      </c>
+      <c r="H453" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B454" s="3" t="inlineStr">
+        <is>
+          <t>2a - George (My new line manager - Reports to Ryan)</t>
+        </is>
+      </c>
+      <c r="C454" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D454" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20_1037_2a-George-My-new-line-manager-Reports-to-Ryan.md</t>
+        </is>
+      </c>
+      <c r="E454" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F454" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G454" s="3" t="inlineStr">
+        <is>
+          <t>Appraisal record section label referring to line manager George.</t>
+        </is>
+      </c>
+      <c r="H454" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B455" s="3" t="inlineStr">
+        <is>
+          <t>2b - Ryan (Old Manager when i was a team leader)</t>
+        </is>
+      </c>
+      <c r="C455" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D455" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20_1037_2b-Ryan-Old-Manager-when-i-was-a-team-leader.md</t>
+        </is>
+      </c>
+      <c r="E455" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F455" s="2" t="inlineStr"/>
+      <c r="G455" s="3" t="inlineStr">
+        <is>
+          <t>Appraisal framing in relation to former manager Ryan.</t>
+        </is>
+      </c>
+      <c r="H455" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B456" s="3" t="inlineStr">
+        <is>
+          <t>2c - Amanda (HR)</t>
+        </is>
+      </c>
+      <c r="C456" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D456" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20_1037_2c-Amanda-HR.md</t>
+        </is>
+      </c>
+      <c r="E456" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F456" s="2" t="inlineStr"/>
+      <c r="G456" s="3" t="inlineStr">
+        <is>
+          <t>Appraisal section drafting on engagement with HR contact Amanda.</t>
+        </is>
+      </c>
+      <c r="H456" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B457" s="3" t="inlineStr">
+        <is>
+          <t>People Interaction Write-up</t>
+        </is>
+      </c>
+      <c r="C457" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D457" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20_1037_People-Interaction-Write-up.md</t>
+        </is>
+      </c>
+      <c r="E457" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F457" s="2" t="inlineStr"/>
+      <c r="G457" s="3" t="inlineStr">
+        <is>
+          <t>Appraisal write-up for the people interaction section.</t>
+        </is>
+      </c>
+      <c r="H457" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B458" s="3" t="inlineStr">
+        <is>
+          <t>1 - Log</t>
+        </is>
+      </c>
+      <c r="C458" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D458" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20_1040_1-Log.md</t>
+        </is>
+      </c>
+      <c r="E458" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F458" s="2" t="inlineStr"/>
+      <c r="G458" s="3" t="inlineStr">
+        <is>
+          <t>Log entry on appraisal positioning and record-keeping.</t>
+        </is>
+      </c>
+      <c r="H458" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B459" s="3" t="inlineStr">
+        <is>
+          <t>3 - Communication Traffic</t>
+        </is>
+      </c>
+      <c r="C459" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D459" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20_1040_3-Communication-Traffic.md</t>
+        </is>
+      </c>
+      <c r="E459" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F459" s="2" t="inlineStr"/>
+      <c r="G459" s="3" t="inlineStr">
+        <is>
+          <t>Appraisal write-up for the communication section.</t>
+        </is>
+      </c>
+      <c r="H459" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B460" s="3" t="inlineStr">
+        <is>
+          <t>3a - George</t>
+        </is>
+      </c>
+      <c r="C460" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D460" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20_1040_3a-George.md</t>
+        </is>
+      </c>
+      <c r="E460" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F460" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G460" s="3" t="inlineStr">
+        <is>
+          <t>Appraisal record section label referring to line manager George.</t>
+        </is>
+      </c>
+      <c r="H460" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B461" s="3" t="inlineStr">
+        <is>
+          <t>3b - Ryan Analysis</t>
+        </is>
+      </c>
+      <c r="C461" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D461" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20_1040_3b-Ryan-Analysis.md</t>
+        </is>
+      </c>
+      <c r="E461" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F461" s="2" t="inlineStr"/>
+      <c r="G461" s="3" t="inlineStr">
+        <is>
+          <t>Appraisal analysis of former manager Ryan's role in the review period.</t>
+        </is>
+      </c>
+      <c r="H461" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B462" s="3" t="inlineStr">
+        <is>
+          <t>3c - Amanda</t>
+        </is>
+      </c>
+      <c r="C462" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D462" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20_1041_3c-Amanda.md</t>
+        </is>
+      </c>
+      <c r="E462" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F462" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G462" s="3" t="inlineStr">
+        <is>
+          <t>Appraisal record section concerning HR contact Amanda.</t>
+        </is>
+      </c>
+      <c r="H462" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B463" s="3" t="inlineStr">
+        <is>
+          <t>6 - Observations and Analysis</t>
+        </is>
+      </c>
+      <c r="C463" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D463" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20_1043_6-Observations-and-Analysis.md</t>
+        </is>
+      </c>
+      <c r="E463" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F463" s="2" t="inlineStr"/>
+      <c r="G463" s="3" t="inlineStr">
+        <is>
+          <t>Appraisal observations and analysis section covering performance, workload and health context.</t>
+        </is>
+      </c>
+      <c r="H463" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B464" s="3" t="inlineStr">
+        <is>
+          <t>5 - Medical and OH Review</t>
+        </is>
+      </c>
+      <c r="C464" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D464" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20_1046_5-Medical-and-OH-Review.md</t>
+        </is>
+      </c>
+      <c r="E464" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F464" s="2" t="inlineStr"/>
+      <c r="G464" s="3" t="inlineStr">
+        <is>
+          <t>Appraisal section on sickness absence, occupational health and return to work.</t>
+        </is>
+      </c>
+      <c r="H464" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B465" s="3" t="inlineStr">
+        <is>
+          <t>68b Resistor Query</t>
+        </is>
+      </c>
+      <c r="C465" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D465" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20_1933_68b-Resistor-Query.md</t>
+        </is>
+      </c>
+      <c r="E465" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F465" s="2" t="inlineStr"/>
+      <c r="G465" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H465" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B466" s="3" t="inlineStr">
+        <is>
+          <t>Concrete Base and Timber Moisture</t>
+        </is>
+      </c>
+      <c r="C466" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D466" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-20_2149_Concrete-Base-and-Timber-Moisture.md</t>
+        </is>
+      </c>
+      <c r="E466" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F466" s="2" t="inlineStr"/>
+      <c r="G466" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H466" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B467" s="3" t="inlineStr">
+        <is>
+          <t>Cheap Log Cabin Elevation</t>
+        </is>
+      </c>
+      <c r="C467" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D467" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-21_1226_Cheap-Log-Cabin-Elevation.md</t>
+        </is>
+      </c>
+      <c r="E467" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F467" s="2" t="inlineStr"/>
+      <c r="G467" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H467" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B468" s="3" t="inlineStr">
+        <is>
+          <t>Find Component by Designator</t>
+        </is>
+      </c>
+      <c r="C468" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D468" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-21_1520_Find-Component-by-Designator.md</t>
+        </is>
+      </c>
+      <c r="E468" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F468" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G468" s="3" t="inlineStr">
+        <is>
+          <t>Question about locating a component by designator in Altium Designer PCB software, possibly for professional work.</t>
+        </is>
+      </c>
+      <c r="H468" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B469" s="3" t="inlineStr">
+        <is>
+          <t>SIP Wall Installation Tips</t>
+        </is>
+      </c>
+      <c r="C469" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D469" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-21_2046_SIP-Wall-Installation-Tips.md</t>
+        </is>
+      </c>
+      <c r="E469" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F469" s="2" t="inlineStr"/>
+      <c r="G469" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H469" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B470" s="3" t="inlineStr">
+        <is>
+          <t>Neutron Radiation and Electronics</t>
+        </is>
+      </c>
+      <c r="C470" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D470" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-21_2209_Neutron-Radiation-and-Electronics.md</t>
+        </is>
+      </c>
+      <c r="E470" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F470" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G470" s="3" t="inlineStr">
+        <is>
+          <t>Technical design of LVDS links, test electronics and acquisition for neutron irradiation testing of a sensor test head.</t>
+        </is>
+      </c>
+      <c r="H470" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B471" s="3" t="inlineStr">
+        <is>
+          <t>Colon Usage Correction</t>
+        </is>
+      </c>
+      <c r="C471" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D471" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-22_1756_Colon-Usage-Correction.md</t>
+        </is>
+      </c>
+      <c r="E471" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F471" s="2" t="inlineStr"/>
+      <c r="G471" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H471" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B472" s="3" t="inlineStr">
+        <is>
+          <t>JustPark refund policy</t>
+        </is>
+      </c>
+      <c r="C472" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D472" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-22_2007_JustPark-refund-policy.md</t>
+        </is>
+      </c>
+      <c r="E472" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F472" s="2" t="inlineStr"/>
+      <c r="G472" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H472" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B473" s="3" t="inlineStr">
+        <is>
+          <t>AD9978BCPZ Overview</t>
+        </is>
+      </c>
+      <c r="C473" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D473" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-23_1045_AD9978BCPZ-Overview.md</t>
+        </is>
+      </c>
+      <c r="E473" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F473" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G473" s="3" t="inlineStr">
+        <is>
+          <t>Technical query on an imaging analog front-end IC and equivalent parts for an electronics design.</t>
+        </is>
+      </c>
+      <c r="H473" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B474" s="3" t="inlineStr">
+        <is>
+          <t>Productivity vs Time and Cost</t>
+        </is>
+      </c>
+      <c r="C474" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D474" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-23_1457_Productivity-vs-Time-and-Cost.md</t>
+        </is>
+      </c>
+      <c r="E474" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F474" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G474" s="3" t="inlineStr">
+        <is>
+          <t>Discussion of pay and hours relative to higher productivity, self-regulating effort at work, and a weekly work pattern.</t>
+        </is>
+      </c>
+      <c r="H474" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B475" s="3" t="inlineStr">
+        <is>
+          <t>AutoCAD default dimension size</t>
+        </is>
+      </c>
+      <c r="C475" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D475" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-23_1846_AutoCAD-default-dimension-size.md</t>
+        </is>
+      </c>
+      <c r="E475" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F475" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G475" s="3" t="inlineStr">
+        <is>
+          <t>AutoCAD dimension style and hatching settings questions; work context unclear.</t>
+        </is>
+      </c>
+      <c r="H475" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B476" s="3" t="inlineStr">
+        <is>
+          <t>Airing Wood After Rain</t>
+        </is>
+      </c>
+      <c r="C476" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D476" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-24_0925_Airing-Wood-After-Rain.md</t>
+        </is>
+      </c>
+      <c r="E476" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F476" s="2" t="inlineStr"/>
+      <c r="G476" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H476" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B477" s="3" t="inlineStr">
+        <is>
+          <t>Dopamine ICSS Experiment</t>
+        </is>
+      </c>
+      <c r="C477" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D477" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-24_1927_Dopamine-ICSS-Experiment.md</t>
+        </is>
+      </c>
+      <c r="E477" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F477" s="2" t="inlineStr"/>
+      <c r="G477" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H477" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B478" s="3" t="inlineStr">
+        <is>
+          <t>Toggle NC Sony WF-C710N</t>
+        </is>
+      </c>
+      <c r="C478" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D478" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-25_0943_Toggle-NC-Sony-WF-C710N.md</t>
+        </is>
+      </c>
+      <c r="E478" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F478" s="2" t="inlineStr"/>
+      <c r="G478" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H478" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B479" s="3" t="inlineStr">
+        <is>
+          <t>Date Dilemma Advice</t>
+        </is>
+      </c>
+      <c r="C479" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D479" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-25_1043_Date-Dilemma-Advice.md</t>
+        </is>
+      </c>
+      <c r="E479" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F479" s="2" t="inlineStr"/>
+      <c r="G479" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H479" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B480" s="3" t="inlineStr">
+        <is>
+          <t>Dogs and Raw Pork</t>
+        </is>
+      </c>
+      <c r="C480" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D480" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-25_1205_Dogs-and-Raw-Pork.md</t>
+        </is>
+      </c>
+      <c r="E480" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F480" s="2" t="inlineStr"/>
+      <c r="G480" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H480" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B481" s="3" t="inlineStr">
+        <is>
+          <t>Separate Cabins for Acoustics</t>
+        </is>
+      </c>
+      <c r="C481" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D481" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-25_1728_Separate-Cabins-for-Acoustics.md</t>
+        </is>
+      </c>
+      <c r="E481" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F481" s="2" t="inlineStr"/>
+      <c r="G481" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H481" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B482" s="3" t="inlineStr">
+        <is>
+          <t>TV License Cancellation Issues</t>
+        </is>
+      </c>
+      <c r="C482" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D482" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-26_1230_TV-License-Cancellation-Issues.md</t>
+        </is>
+      </c>
+      <c r="E482" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F482" s="2" t="inlineStr"/>
+      <c r="G482" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H482" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B483" s="3" t="inlineStr">
+        <is>
+          <t>Smith vs Oracle</t>
+        </is>
+      </c>
+      <c r="C483" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D483" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-26_1901_Smith-vs-Oracle.md</t>
+        </is>
+      </c>
+      <c r="E483" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F483" s="2" t="inlineStr"/>
+      <c r="G483" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H483" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B484" s="3" t="inlineStr">
+        <is>
+          <t>Earbud Repair Limitations</t>
+        </is>
+      </c>
+      <c r="C484" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D484" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-26_2136_Earbud-Repair-Limitations.md</t>
+        </is>
+      </c>
+      <c r="E484" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F484" s="2" t="inlineStr"/>
+      <c r="G484" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H484" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B485" s="3" t="inlineStr">
+        <is>
+          <t>Cheapest Building Materials London</t>
+        </is>
+      </c>
+      <c r="C485" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D485" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-27_1858_Cheapest-Building-Materials-London.md</t>
+        </is>
+      </c>
+      <c r="E485" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F485" s="2" t="inlineStr"/>
+      <c r="G485" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H485" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B486" s="3" t="inlineStr">
+        <is>
+          <t>Window Replacement Advice</t>
+        </is>
+      </c>
+      <c r="C486" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D486" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-27_1914_Window-Replacement-Advice.md</t>
+        </is>
+      </c>
+      <c r="E486" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F486" s="2" t="inlineStr"/>
+      <c r="G486" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H486" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B487" s="3" t="inlineStr">
+        <is>
+          <t>Tyvek Roll Size Inquiry</t>
+        </is>
+      </c>
+      <c r="C487" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D487" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-27_1954_Tyvek-Roll-Size-Inquiry.md</t>
+        </is>
+      </c>
+      <c r="E487" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F487" s="2" t="inlineStr"/>
+      <c r="G487" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H487" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B488" s="3" t="inlineStr">
+        <is>
+          <t>Suspension or Resignation?</t>
+        </is>
+      </c>
+      <c r="C488" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D488" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-27_2051_Suspension-or-Resignation.md</t>
+        </is>
+      </c>
+      <c r="E488" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F488" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G488" s="3" t="inlineStr">
+        <is>
+          <t>Colleague's walk-off, performance process and exit; blame directed at owner, defence documentation, HR meetings, sickness recording, reasonable adjustments, flexible working, appraisal, project reallocation and a reported data-security issue.</t>
+        </is>
+      </c>
+      <c r="H488" s="2" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B489" s="3" t="inlineStr">
+        <is>
+          <t>Soldering Temp for THT</t>
+        </is>
+      </c>
+      <c r="C489" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D489" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-28_1653_Soldering-Temp-for-THT.md</t>
+        </is>
+      </c>
+      <c r="E489" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F489" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G489" s="3" t="inlineStr">
+        <is>
+          <t>Through-hole soldering temperature and flux question, possibly related to electronics engineering work.</t>
+        </is>
+      </c>
+      <c r="H489" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B490" s="3" t="inlineStr">
+        <is>
+          <t>Video Background Distortion Fixes</t>
+        </is>
+      </c>
+      <c r="C490" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D490" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-28_1733_Video-Background-Distortion-Fixes.md</t>
+        </is>
+      </c>
+      <c r="E490" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F490" s="2" t="inlineStr"/>
+      <c r="G490" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H490" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B491" s="3" t="inlineStr">
+        <is>
+          <t>Response Options for Message Count</t>
+        </is>
+      </c>
+      <c r="C491" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D491" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29_0537_Response-Options-for-Message-Count.md</t>
+        </is>
+      </c>
+      <c r="E491" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F491" s="2" t="inlineStr"/>
+      <c r="G491" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H491" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B492" s="3" t="inlineStr">
+        <is>
+          <t>Smart response options</t>
+        </is>
+      </c>
+      <c r="C492" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D492" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29_1001_Smart-response-options.md</t>
+        </is>
+      </c>
+      <c r="E492" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F492" s="2" t="inlineStr"/>
+      <c r="G492" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H492" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B493" s="3" t="inlineStr">
+        <is>
+          <t>Bonus Redistribution Explained</t>
+        </is>
+      </c>
+      <c r="C493" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D493" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29_1449_Bonus-Redistribution-Explained.md</t>
+        </is>
+      </c>
+      <c r="E493" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F493" s="2" t="inlineStr"/>
+      <c r="G493" s="3" t="inlineStr">
+        <is>
+          <t>Owner's annual work bonus amount relative to the stated percentage and a colleague's exclusion due to a performance plan.</t>
+        </is>
+      </c>
+      <c r="H493" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B494" s="3" t="inlineStr">
+        <is>
+          <t>Make links visible CADSTAR</t>
+        </is>
+      </c>
+      <c r="C494" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D494" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-29_1822_Make-links-visible-CADSTAR.md</t>
+        </is>
+      </c>
+      <c r="E494" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F494" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G494" s="3" t="inlineStr">
+        <is>
+          <t>Question on displaying connectivity links in CADSTAR PCB design software, possibly for engineering work.</t>
+        </is>
+      </c>
+      <c r="H494" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B495" s="3" t="inlineStr">
+        <is>
+          <t>Triple Glazed Upgrade Feasibility</t>
+        </is>
+      </c>
+      <c r="C495" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D495" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-30_1306_Triple-Glazed-Upgrade-Feasibility.md</t>
+        </is>
+      </c>
+      <c r="E495" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F495" s="2" t="inlineStr"/>
+      <c r="G495" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H495" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B496" s="3" t="inlineStr">
+        <is>
+          <t>BorrowMyDoggy Premium Requirements</t>
+        </is>
+      </c>
+      <c r="C496" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D496" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31_0904_BorrowMyDoggy-Premium-Requirements.md</t>
+        </is>
+      </c>
+      <c r="E496" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F496" s="2" t="inlineStr"/>
+      <c r="G496" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H496" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B497" s="3" t="inlineStr">
+        <is>
+          <t>DJ Controller GarageBand Setup</t>
+        </is>
+      </c>
+      <c r="C497" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D497" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31_1108_DJ-Controller-GarageBand-Setup.md</t>
+        </is>
+      </c>
+      <c r="E497" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F497" s="2" t="inlineStr"/>
+      <c r="G497" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H497" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B498" s="3" t="inlineStr">
+        <is>
+          <t>Self-awareness and Stillness</t>
+        </is>
+      </c>
+      <c r="C498" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D498" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31_1133_Self-awareness-and-Stillness.md</t>
+        </is>
+      </c>
+      <c r="E498" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F498" s="2" t="inlineStr"/>
+      <c r="G498" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H498" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B499" s="3" t="inlineStr">
+        <is>
+          <t>Song Learning vs Progression</t>
+        </is>
+      </c>
+      <c r="C499" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D499" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31_1211_Song-Learning-vs-Progression.md</t>
+        </is>
+      </c>
+      <c r="E499" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F499" s="2" t="inlineStr"/>
+      <c r="G499" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H499" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B500" s="3" t="inlineStr">
+        <is>
+          <t>Best Books for ESE</t>
+        </is>
+      </c>
+      <c r="C500" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D500" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31_1311_Best-Books-for-ESE.md</t>
+        </is>
+      </c>
+      <c r="E500" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F500" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G500" s="3" t="inlineStr">
+        <is>
+          <t>Book recommendations for electronic systems engineering and systems engineering, relevant to the owner's profession.</t>
+        </is>
+      </c>
+      <c r="H500" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B501" s="3" t="inlineStr">
+        <is>
+          <t>E-bike recommendations for versatility</t>
+        </is>
+      </c>
+      <c r="C501" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-004.json</t>
+        </is>
+      </c>
+      <c r="D501" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31_1459_E-bike-recommendations-for-versatility.md</t>
+        </is>
+      </c>
+      <c r="E501" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F501" s="2" t="inlineStr"/>
+      <c r="G501" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H501" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B502" s="3" t="inlineStr">
+        <is>
+          <t>Dragon Anywhere License</t>
+        </is>
+      </c>
+      <c r="C502" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D502" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31_1930_Dragon-Anywhere-License.md</t>
+        </is>
+      </c>
+      <c r="E502" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F502" s="2" t="inlineStr"/>
+      <c r="G502" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H502" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B503" s="3" t="inlineStr">
+        <is>
+          <t>Elvanse Break Effectiveness</t>
+        </is>
+      </c>
+      <c r="C503" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D503" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31_2218_Elvanse-Break-Effectiveness.md</t>
+        </is>
+      </c>
+      <c r="E503" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F503" s="2" t="inlineStr"/>
+      <c r="G503" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H503" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B504" s="3" t="inlineStr">
+        <is>
+          <t>Quitting smoking and ASD</t>
+        </is>
+      </c>
+      <c r="C504" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D504" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01_1128_Quitting-smoking-and-ASD.md</t>
+        </is>
+      </c>
+      <c r="E504" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F504" s="2" t="inlineStr"/>
+      <c r="G504" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H504" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B505" s="3" t="inlineStr">
+        <is>
+          <t>Electronic Design Welcome</t>
+        </is>
+      </c>
+      <c r="C505" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D505" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01_1244_Electronic-Design-Welcome.md</t>
+        </is>
+      </c>
+      <c r="E505" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F505" s="2" t="inlineStr"/>
+      <c r="G505" s="3" t="inlineStr">
+        <is>
+          <t>Designing electronics-themed welcome back signs for a returning colleague.</t>
+        </is>
+      </c>
+      <c r="H505" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B506" s="3" t="inlineStr">
+        <is>
+          <t>Design Consistency Request</t>
+        </is>
+      </c>
+      <c r="C506" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D506" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01_1304_Design-Consistency-Request.md</t>
+        </is>
+      </c>
+      <c r="E506" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F506" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G506" s="3" t="inlineStr">
+        <is>
+          <t>Image edit request apparently continuing the welcome back sign design for a colleague.</t>
+        </is>
+      </c>
+      <c r="H506" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B507" s="3" t="inlineStr">
+        <is>
+          <t>Introduction Rewrite Request</t>
+        </is>
+      </c>
+      <c r="C507" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D507" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01_2204_Introduction-Rewrite-Request.md</t>
+        </is>
+      </c>
+      <c r="E507" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F507" s="2" t="inlineStr"/>
+      <c r="G507" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H507" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="B508" s="3" t="inlineStr">
+        <is>
+          <t>ADHD360 Shared Care Refusal</t>
+        </is>
+      </c>
+      <c r="C508" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D508" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01_2304_ADHD360-Shared-Care-Refusal.md</t>
+        </is>
+      </c>
+      <c r="E508" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F508" s="2" t="inlineStr"/>
+      <c r="G508" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H508" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B509" s="3" t="inlineStr">
+        <is>
+          <t>Screenshot transcription request</t>
+        </is>
+      </c>
+      <c r="C509" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D509" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02_1510_Screenshot-transcription-request.md</t>
+        </is>
+      </c>
+      <c r="E509" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F509" s="2" t="inlineStr"/>
+      <c r="G509" s="3" t="inlineStr">
+        <is>
+          <t>Transcription and evidence log of a workplace Teams chat with a colleague about CS125 burn-in, test modules and task ownership.</t>
+        </is>
+      </c>
+      <c r="H509" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B510" s="3" t="inlineStr">
+        <is>
+          <t>Requirements Validation for Reused Hardware</t>
+        </is>
+      </c>
+      <c r="C510" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D510" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02_1623_Requirements-Validation-for-Reused-Hardware.md</t>
+        </is>
+      </c>
+      <c r="E510" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F510" s="2" t="inlineStr"/>
+      <c r="G510" s="3" t="inlineStr">
+        <is>
+          <t>Engineering question on validating requirements for reused hardware and delta design documentation.</t>
+        </is>
+      </c>
+      <c r="H510" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B511" s="3" t="inlineStr">
+        <is>
+          <t>ADOS-2 Clinical Summary</t>
+        </is>
+      </c>
+      <c r="C511" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D511" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02_1816_ADOS-2-Clinical-Summary.md</t>
+        </is>
+      </c>
+      <c r="E511" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F511" s="2" t="inlineStr"/>
+      <c r="G511" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H511" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03</t>
+        </is>
+      </c>
+      <c r="B512" s="3" t="inlineStr">
+        <is>
+          <t>Debut Payments Explained</t>
+        </is>
+      </c>
+      <c r="C512" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D512" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-03_1143_Debut-Payments-Explained.md</t>
+        </is>
+      </c>
+      <c r="E512" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F512" s="2" t="inlineStr"/>
+      <c r="G512" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H512" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B513" s="3" t="inlineStr">
+        <is>
+          <t>Document Comparison Review</t>
+        </is>
+      </c>
+      <c r="C513" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D513" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-04_1318_Document-Comparison-Review.md</t>
+        </is>
+      </c>
+      <c r="E513" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F513" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G513" s="3" t="inlineStr">
+        <is>
+          <t>Describes how the owner organises their work (workload categorisation, workspace, folders, tools) as examples within a personal document.</t>
+        </is>
+      </c>
+      <c r="H513" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B514" s="3" t="inlineStr">
+        <is>
+          <t>What is an abstract</t>
+        </is>
+      </c>
+      <c r="C514" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D514" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-04_1329_What-is-an-abstract.md</t>
+        </is>
+      </c>
+      <c r="E514" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F514" s="2" t="inlineStr"/>
+      <c r="G514" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H514" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B515" s="3" t="inlineStr">
+        <is>
+          <t>New chat</t>
+        </is>
+      </c>
+      <c r="C515" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D515" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-05_0157_New-chat.md</t>
+        </is>
+      </c>
+      <c r="E515" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F515" s="2" t="inlineStr"/>
+      <c r="G515" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H515" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B516" s="3" t="inlineStr">
+        <is>
+          <t>New chat</t>
+        </is>
+      </c>
+      <c r="C516" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D516" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-05_0211_New-chat.md</t>
+        </is>
+      </c>
+      <c r="E516" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F516" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G516" s="3" t="inlineStr">
+        <is>
+          <t>Technical engineering question about high-speed LVDS cabling for radiation environments.</t>
+        </is>
+      </c>
+      <c r="H516" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B517" s="3" t="inlineStr">
+        <is>
+          <t>New chat</t>
+        </is>
+      </c>
+      <c r="C517" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D517" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-05_0840_New-chat.md</t>
+        </is>
+      </c>
+      <c r="E517" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F517" s="2" t="inlineStr"/>
+      <c r="G517" s="3" t="inlineStr">
+        <is>
+          <t>Whether a design should pass Critical Design Review when modifications are not captured in an up-issued design.</t>
+        </is>
+      </c>
+      <c r="H517" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-05</t>
+        </is>
+      </c>
+      <c r="B518" s="3" t="inlineStr">
+        <is>
+          <t>Teams usage with ADHD</t>
+        </is>
+      </c>
+      <c r="C518" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D518" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-05_2035_Teams-usage-with-ADHD.md</t>
+        </is>
+      </c>
+      <c r="E518" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F518" s="2" t="inlineStr"/>
+      <c r="G518" s="3" t="inlineStr">
+        <is>
+          <t>Requirement to use Teams onsite, reasonable adjustments for ADHD/ASD, and setting communication boundaries with work.</t>
+        </is>
+      </c>
+      <c r="H518" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="B519" s="3" t="inlineStr">
+        <is>
+          <t>Process vs Engineering Flow</t>
+        </is>
+      </c>
+      <c r="C519" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D519" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-06_1346_Process-vs-Engineering-Flow.md</t>
+        </is>
+      </c>
+      <c r="E519" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F519" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G519" s="3" t="inlineStr">
+        <is>
+          <t>Question about process-oriented managers managing engineering professionals and workflows.</t>
+        </is>
+      </c>
+      <c r="H519" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="B520" s="3" t="inlineStr">
+        <is>
+          <t>Autism Assessment Cancellation Reaction</t>
+        </is>
+      </c>
+      <c r="C520" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D520" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-07_1606_Autism-Assessment-Cancellation-Reaction.md</t>
+        </is>
+      </c>
+      <c r="E520" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F520" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G520" s="3" t="inlineStr">
+        <is>
+          <t>Discusses wrongful accusations and a formal investigation at work following a colleague performance feedback request, restricted workspace access, return to work after sickness absence, and the effect on the owner's mental health.</t>
+        </is>
+      </c>
+      <c r="H520" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H452"/>
+  <autoFilter ref="A1:H520"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17204,7 +19720,7 @@
         </is>
       </c>
       <c r="B1" t="n">
-        <v>451</v>
+        <v>519</v>
       </c>
     </row>
     <row r="2">
@@ -17214,7 +19730,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>79</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3">
@@ -17224,7 +19740,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4">
@@ -17234,7 +19750,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>142</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5">
@@ -17244,7 +19760,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>309</v>
+        <v>345</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
chat-sift: batches b70-b79 read; index, extracts and progress updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aq7txTcfpUgzabiqqnXaKj
</commit_message>
<xml_diff>
--- a/chat-sift/output/index.xlsx
+++ b/chat-sift/output/index.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$520</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$637</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H520"/>
+  <dimension ref="A1:H637"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19695,8 +19695,4368 @@
         <v>4</v>
       </c>
     </row>
+    <row r="521">
+      <c r="A521" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B521" s="3" t="inlineStr">
+        <is>
+          <t>ASD Assessment Alternative Evidence</t>
+        </is>
+      </c>
+      <c r="C521" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D521" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0514_ASD-Assessment-Alternative-Evidence.md</t>
+        </is>
+      </c>
+      <c r="E521" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F521" s="2" t="inlineStr"/>
+      <c r="G521" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H521" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B522" s="3" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="C522" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D522" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0607_0-0.md</t>
+        </is>
+      </c>
+      <c r="E522" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F522" s="2" t="inlineStr"/>
+      <c r="G522" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H522" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B523" s="3" t="inlineStr">
+        <is>
+          <t>Layer 1.1 Report</t>
+        </is>
+      </c>
+      <c r="C523" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D523" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0609_Layer-1-1-Report.md</t>
+        </is>
+      </c>
+      <c r="E523" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F523" s="2" t="inlineStr"/>
+      <c r="G523" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H523" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B524" s="3" t="inlineStr">
+        <is>
+          <t>Layer 1.0 Year Report</t>
+        </is>
+      </c>
+      <c r="C524" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D524" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0610_Layer-1-0-Year-Report.md</t>
+        </is>
+      </c>
+      <c r="E524" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F524" s="2" t="inlineStr"/>
+      <c r="G524" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H524" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B525" s="3" t="inlineStr">
+        <is>
+          <t>Year 2 Report Summary</t>
+        </is>
+      </c>
+      <c r="C525" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D525" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0611_Year-2-Report-Summary.md</t>
+        </is>
+      </c>
+      <c r="E525" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F525" s="2" t="inlineStr"/>
+      <c r="G525" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H525" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B526" s="3" t="inlineStr">
+        <is>
+          <t>Layer 1.4 Report Summary</t>
+        </is>
+      </c>
+      <c r="C526" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D526" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0612_Layer-1-4-Report-Summary.md</t>
+        </is>
+      </c>
+      <c r="E526" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F526" s="2" t="inlineStr"/>
+      <c r="G526" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H526" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B527" s="3" t="inlineStr">
+        <is>
+          <t>Primary School Report</t>
+        </is>
+      </c>
+      <c r="C527" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D527" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0612_Primary-School-Report.md</t>
+        </is>
+      </c>
+      <c r="E527" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F527" s="2" t="inlineStr"/>
+      <c r="G527" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H527" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B528" s="3" t="inlineStr">
+        <is>
+          <t>New chat</t>
+        </is>
+      </c>
+      <c r="C528" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D528" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0613_New-chat.md</t>
+        </is>
+      </c>
+      <c r="E528" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F528" s="2" t="inlineStr"/>
+      <c r="G528" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H528" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B529" s="3" t="inlineStr">
+        <is>
+          <t>Layer 1.7 Confirmation</t>
+        </is>
+      </c>
+      <c r="C529" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D529" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0614_Layer-1-7-Confirmation.md</t>
+        </is>
+      </c>
+      <c r="E529" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F529" s="2" t="inlineStr"/>
+      <c r="G529" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H529" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B530" s="3" t="inlineStr">
+        <is>
+          <t>New chat</t>
+        </is>
+      </c>
+      <c r="C530" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D530" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0614_New-chat.md</t>
+        </is>
+      </c>
+      <c r="E530" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F530" s="2" t="inlineStr"/>
+      <c r="G530" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H530" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B531" s="3" t="inlineStr">
+        <is>
+          <t>Layer 1.8 Report Summary</t>
+        </is>
+      </c>
+      <c r="C531" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D531" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0617_Layer-1-8-Report-Summary.md</t>
+        </is>
+      </c>
+      <c r="E531" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F531" s="2" t="inlineStr"/>
+      <c r="G531" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H531" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B532" s="3" t="inlineStr">
+        <is>
+          <t>Layer 1.9 Analysis</t>
+        </is>
+      </c>
+      <c r="C532" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D532" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0617_Layer-1-9-Analysis.md</t>
+        </is>
+      </c>
+      <c r="E532" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F532" s="2" t="inlineStr"/>
+      <c r="G532" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H532" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B533" s="3" t="inlineStr">
+        <is>
+          <t>Layer 1.10 Confirmation</t>
+        </is>
+      </c>
+      <c r="C533" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D533" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0618_Layer-1-10-Confirmation.md</t>
+        </is>
+      </c>
+      <c r="E533" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F533" s="2" t="inlineStr"/>
+      <c r="G533" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H533" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B534" s="3" t="inlineStr">
+        <is>
+          <t>Layer 1.11 Review</t>
+        </is>
+      </c>
+      <c r="C534" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D534" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0619_Layer-1-11-Review.md</t>
+        </is>
+      </c>
+      <c r="E534" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F534" s="2" t="inlineStr"/>
+      <c r="G534" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H534" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B535" s="3" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="C535" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D535" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0621_2-0.md</t>
+        </is>
+      </c>
+      <c r="E535" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F535" s="2" t="inlineStr"/>
+      <c r="G535" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H535" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B536" s="3" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="C536" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D536" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0624_2-1.md</t>
+        </is>
+      </c>
+      <c r="E536" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F536" s="2" t="inlineStr"/>
+      <c r="G536" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H536" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B537" s="3" t="inlineStr">
+        <is>
+          <t>Evidence Extraction Example</t>
+        </is>
+      </c>
+      <c r="C537" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D537" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0626_Evidence-Extraction-Example.md</t>
+        </is>
+      </c>
+      <c r="E537" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F537" s="2" t="inlineStr"/>
+      <c r="G537" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H537" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B538" s="3" t="inlineStr">
+        <is>
+          <t>Evidence Extraction Layer 2.3</t>
+        </is>
+      </c>
+      <c r="C538" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D538" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0627_Evidence-Extraction-Layer-2-3.md</t>
+        </is>
+      </c>
+      <c r="E538" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F538" s="2" t="inlineStr"/>
+      <c r="G538" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H538" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B539" s="3" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="C539" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D539" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0628_2-5.md</t>
+        </is>
+      </c>
+      <c r="E539" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F539" s="2" t="inlineStr"/>
+      <c r="G539" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H539" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B540" s="3" t="inlineStr">
+        <is>
+          <t>Evidence Extraction Layer 2.4</t>
+        </is>
+      </c>
+      <c r="C540" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D540" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0628_Evidence-Extraction-Layer-2-4.md</t>
+        </is>
+      </c>
+      <c r="E540" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F540" s="2" t="inlineStr"/>
+      <c r="G540" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H540" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B541" s="3" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="C541" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D541" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0629_2-6.md</t>
+        </is>
+      </c>
+      <c r="E541" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F541" s="2" t="inlineStr"/>
+      <c r="G541" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H541" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B542" s="3" t="inlineStr">
+        <is>
+          <t>Evidence Extraction Layer 2.7</t>
+        </is>
+      </c>
+      <c r="C542" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D542" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0630_Evidence-Extraction-Layer-2-7.md</t>
+        </is>
+      </c>
+      <c r="E542" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F542" s="2" t="inlineStr"/>
+      <c r="G542" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H542" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B543" s="3" t="inlineStr">
+        <is>
+          <t>Evidence Extraction Layer 2.8</t>
+        </is>
+      </c>
+      <c r="C543" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D543" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0630_Evidence-Extraction-Layer-2-8.md</t>
+        </is>
+      </c>
+      <c r="E543" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F543" s="2" t="inlineStr"/>
+      <c r="G543" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H543" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B544" s="3" t="inlineStr">
+        <is>
+          <t>Evidence Extraction Layer 2.9</t>
+        </is>
+      </c>
+      <c r="C544" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D544" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0631_Evidence-Extraction-Layer-2-9.md</t>
+        </is>
+      </c>
+      <c r="E544" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F544" s="2" t="inlineStr"/>
+      <c r="G544" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H544" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B545" s="3" t="inlineStr">
+        <is>
+          <t>Verbatim Evidence Extraction</t>
+        </is>
+      </c>
+      <c r="C545" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D545" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0631_Verbatim-Evidence-Extraction.md</t>
+        </is>
+      </c>
+      <c r="E545" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F545" s="2" t="inlineStr"/>
+      <c r="G545" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H545" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B546" s="3" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="C546" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D546" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0632_2-11.md</t>
+        </is>
+      </c>
+      <c r="E546" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F546" s="2" t="inlineStr"/>
+      <c r="G546" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H546" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B547" s="3" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="C547" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D547" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0650_3-0.md</t>
+        </is>
+      </c>
+      <c r="E547" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F547" s="2" t="inlineStr"/>
+      <c r="G547" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H547" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B548" s="3" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="C548" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D548" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0652_3-1.md</t>
+        </is>
+      </c>
+      <c r="E548" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F548" s="2" t="inlineStr"/>
+      <c r="G548" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H548" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B549" s="3" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="C549" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D549" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0653_3-2.md</t>
+        </is>
+      </c>
+      <c r="E549" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F549" s="2" t="inlineStr"/>
+      <c r="G549" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H549" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B550" s="3" t="inlineStr">
+        <is>
+          <t>Layer 3.3 Synthesis</t>
+        </is>
+      </c>
+      <c r="C550" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D550" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0714_Layer-3-3-Synthesis.md</t>
+        </is>
+      </c>
+      <c r="E550" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F550" s="2" t="inlineStr"/>
+      <c r="G550" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H550" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B551" s="3" t="inlineStr">
+        <is>
+          <t>Pattern Synthesis Guidelines</t>
+        </is>
+      </c>
+      <c r="C551" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D551" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0715_Pattern-Synthesis-Guidelines.md</t>
+        </is>
+      </c>
+      <c r="E551" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F551" s="2" t="inlineStr"/>
+      <c r="G551" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H551" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B552" s="3" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="C552" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D552" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0716_3-5.md</t>
+        </is>
+      </c>
+      <c r="E552" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F552" s="2" t="inlineStr"/>
+      <c r="G552" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H552" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B553" s="3" t="inlineStr">
+        <is>
+          <t>3.6</t>
+        </is>
+      </c>
+      <c r="C553" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D553" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0723_3-6.md</t>
+        </is>
+      </c>
+      <c r="E553" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F553" s="2" t="inlineStr"/>
+      <c r="G553" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H553" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B554" s="3" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="C554" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D554" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0724_3-7.md</t>
+        </is>
+      </c>
+      <c r="E554" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F554" s="2" t="inlineStr"/>
+      <c r="G554" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H554" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B555" s="3" t="inlineStr">
+        <is>
+          <t>3.8</t>
+        </is>
+      </c>
+      <c r="C555" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D555" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0725_3-8.md</t>
+        </is>
+      </c>
+      <c r="E555" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F555" s="2" t="inlineStr"/>
+      <c r="G555" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H555" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B556" s="3" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
+      </c>
+      <c r="C556" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D556" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0725_3-9.md</t>
+        </is>
+      </c>
+      <c r="E556" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F556" s="2" t="inlineStr"/>
+      <c r="G556" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H556" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B557" s="3" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="C557" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D557" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0726_3-10.md</t>
+        </is>
+      </c>
+      <c r="E557" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F557" s="2" t="inlineStr"/>
+      <c r="G557" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H557" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B558" s="3" t="inlineStr">
+        <is>
+          <t>3.11</t>
+        </is>
+      </c>
+      <c r="C558" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D558" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0726_3-11.md</t>
+        </is>
+      </c>
+      <c r="E558" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F558" s="2" t="inlineStr"/>
+      <c r="G558" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H558" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B559" s="3" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="C559" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D559" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0736_4-0.md</t>
+        </is>
+      </c>
+      <c r="E559" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F559" s="2" t="inlineStr"/>
+      <c r="G559" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H559" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B560" s="3" t="inlineStr">
+        <is>
+          <t>Layer 5.0 Info Dump</t>
+        </is>
+      </c>
+      <c r="C560" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D560" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0747_Layer-5-0-Info-Dump.md</t>
+        </is>
+      </c>
+      <c r="E560" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F560" s="2" t="inlineStr"/>
+      <c r="G560" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H560" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B561" s="3" t="inlineStr">
+        <is>
+          <t>Transcript of Year 7 Report</t>
+        </is>
+      </c>
+      <c r="C561" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D561" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0802_Transcript-of-Year-7-Report.md</t>
+        </is>
+      </c>
+      <c r="E561" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F561" s="2" t="inlineStr"/>
+      <c r="G561" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H561" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B562" s="3" t="inlineStr">
+        <is>
+          <t>Full Transcription Request</t>
+        </is>
+      </c>
+      <c r="C562" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D562" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0805_Full-Transcription-Request.md</t>
+        </is>
+      </c>
+      <c r="E562" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F562" s="2" t="inlineStr"/>
+      <c r="G562" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H562" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B563" s="3" t="inlineStr">
+        <is>
+          <t>Full Transcript Request</t>
+        </is>
+      </c>
+      <c r="C563" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D563" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0806_Full-Transcript-Request.md</t>
+        </is>
+      </c>
+      <c r="E563" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F563" s="2" t="inlineStr"/>
+      <c r="G563" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H563" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B564" s="3" t="inlineStr">
+        <is>
+          <t>Full Transcription Request</t>
+        </is>
+      </c>
+      <c r="C564" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D564" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0806_Full-Transcription-Request.md</t>
+        </is>
+      </c>
+      <c r="E564" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F564" s="2" t="inlineStr"/>
+      <c r="G564" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H564" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B565" s="3" t="inlineStr">
+        <is>
+          <t>Full Transcription Request</t>
+        </is>
+      </c>
+      <c r="C565" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D565" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0807_Full-Transcription-Request.md</t>
+        </is>
+      </c>
+      <c r="E565" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F565" s="2" t="inlineStr"/>
+      <c r="G565" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H565" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B566" s="3" t="inlineStr">
+        <is>
+          <t>Report transcription</t>
+        </is>
+      </c>
+      <c r="C566" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D566" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0819_Report-transcription.md</t>
+        </is>
+      </c>
+      <c r="E566" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F566" s="2" t="inlineStr"/>
+      <c r="G566" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H566" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B567" s="3" t="inlineStr">
+        <is>
+          <t>Year R Report Summary</t>
+        </is>
+      </c>
+      <c r="C567" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D567" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0819_Year-R-Report-Summary.md</t>
+        </is>
+      </c>
+      <c r="E567" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F567" s="2" t="inlineStr"/>
+      <c r="G567" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H567" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B568" s="3" t="inlineStr">
+        <is>
+          <t>Transcription of Report</t>
+        </is>
+      </c>
+      <c r="C568" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D568" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0820_Transcription-of-Report.md</t>
+        </is>
+      </c>
+      <c r="E568" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F568" s="2" t="inlineStr"/>
+      <c r="G568" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H568" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B569" s="3" t="inlineStr">
+        <is>
+          <t>Transcript of Report</t>
+        </is>
+      </c>
+      <c r="C569" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D569" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0821_Transcript-of-Report.md</t>
+        </is>
+      </c>
+      <c r="E569" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F569" s="2" t="inlineStr"/>
+      <c r="G569" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H569" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B570" s="3" t="inlineStr">
+        <is>
+          <t>Transcription of Report</t>
+        </is>
+      </c>
+      <c r="C570" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D570" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0821_Transcription-of-Report.md</t>
+        </is>
+      </c>
+      <c r="E570" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F570" s="2" t="inlineStr"/>
+      <c r="G570" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H570" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B571" s="3" t="inlineStr">
+        <is>
+          <t>Transcription of Report</t>
+        </is>
+      </c>
+      <c r="C571" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D571" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0822_Transcription-of-Report.md</t>
+        </is>
+      </c>
+      <c r="E571" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F571" s="2" t="inlineStr"/>
+      <c r="G571" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H571" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B572" s="3" t="inlineStr">
+        <is>
+          <t>Transcript Request</t>
+        </is>
+      </c>
+      <c r="C572" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D572" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_0826_Transcript-Request.md</t>
+        </is>
+      </c>
+      <c r="E572" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F572" s="2" t="inlineStr"/>
+      <c r="G572" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H572" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08</t>
+        </is>
+      </c>
+      <c r="B573" s="3" t="inlineStr">
+        <is>
+          <t>Managerial Time Enforcement Debate</t>
+        </is>
+      </c>
+      <c r="C573" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D573" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-08_1226_Managerial-Time-Enforcement-Debate.md</t>
+        </is>
+      </c>
+      <c r="E573" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F573" s="2" t="inlineStr"/>
+      <c r="G573" s="3" t="inlineStr">
+        <is>
+          <t>New manager enforcing fixed start and finish times, team dynamics, removal of team lead duties after stress-related absence, and a personal work operating framework.</t>
+        </is>
+      </c>
+      <c r="H573" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B574" s="3" t="inlineStr">
+        <is>
+          <t>Flexible Working Justification</t>
+        </is>
+      </c>
+      <c r="C574" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D574" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09_1339_Flexible-Working-Justification.md</t>
+        </is>
+      </c>
+      <c r="E574" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F574" s="2" t="inlineStr"/>
+      <c r="G574" s="3" t="inlineStr">
+        <is>
+          <t>Drafting a flexible working request (compressed hours, partial home working) referencing the Occupational Health report and disability question on the form.</t>
+        </is>
+      </c>
+      <c r="H574" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B575" s="3" t="inlineStr">
+        <is>
+          <t>Cable Distance with LVDS</t>
+        </is>
+      </c>
+      <c r="C575" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D575" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09_1857_Cable-Distance-with-LVDS.md</t>
+        </is>
+      </c>
+      <c r="E575" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F575" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G575" s="3" t="inlineStr">
+        <is>
+          <t>Technical question on LVDS line driver cable distance, likely related to engineering work.</t>
+        </is>
+      </c>
+      <c r="H575" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B576" s="3" t="inlineStr">
+        <is>
+          <t>Defined Responsibility Envelope</t>
+        </is>
+      </c>
+      <c r="C576" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D576" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09_2210_Defined-Responsibility-Envelope.md</t>
+        </is>
+      </c>
+      <c r="E576" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F576" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G576" s="3" t="inlineStr">
+        <is>
+          <t>Refining a personal rule set on limiting responsibilities to assigned work scope.</t>
+        </is>
+      </c>
+      <c r="H576" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B577" s="3" t="inlineStr">
+        <is>
+          <t>Operating Model Redesign</t>
+        </is>
+      </c>
+      <c r="C577" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D577" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09_2210_Operating-Model-Redesign.md</t>
+        </is>
+      </c>
+      <c r="E577" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F577" s="2" t="inlineStr"/>
+      <c r="G577" s="3" t="inlineStr">
+        <is>
+          <t>Refining a project charter for a professional operating model following work overload and role reallocation.</t>
+        </is>
+      </c>
+      <c r="H577" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B578" s="3" t="inlineStr">
+        <is>
+          <t>Clean Excellence Standard</t>
+        </is>
+      </c>
+      <c r="C578" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D578" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09_2211_Clean-Excellence-Standard.md</t>
+        </is>
+      </c>
+      <c r="E578" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F578" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G578" s="3" t="inlineStr">
+        <is>
+          <t>Refining a personal standard for work output and communication.</t>
+        </is>
+      </c>
+      <c r="H578" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B579" s="3" t="inlineStr">
+        <is>
+          <t>Emotional Neutrality Protocol</t>
+        </is>
+      </c>
+      <c r="C579" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D579" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09_2212_Emotional-Neutrality-Protocol.md</t>
+        </is>
+      </c>
+      <c r="E579" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F579" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G579" s="3" t="inlineStr">
+        <is>
+          <t>Refining a personal protocol for responding to leadership process and micro-control.</t>
+        </is>
+      </c>
+      <c r="H579" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B580" s="3" t="inlineStr">
+        <is>
+          <t>Strategic Identity Refinement</t>
+        </is>
+      </c>
+      <c r="C580" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D580" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09_2212_Strategic-Identity-Refinement.md</t>
+        </is>
+      </c>
+      <c r="E580" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F580" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G580" s="3" t="inlineStr">
+        <is>
+          <t>Refining a personal statement of professional identity as a technical operator.</t>
+        </is>
+      </c>
+      <c r="H580" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B581" s="3" t="inlineStr">
+        <is>
+          <t>Sustainability Guardrails</t>
+        </is>
+      </c>
+      <c r="C581" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D581" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09_2213_Sustainability-Guardrails.md</t>
+        </is>
+      </c>
+      <c r="E581" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F581" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G581" s="3" t="inlineStr">
+        <is>
+          <t>Refining personal guardrails for managing stress and workload exposure.</t>
+        </is>
+      </c>
+      <c r="H581" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B582" s="3" t="inlineStr">
+        <is>
+          <t>Dopamine and Autism Traits</t>
+        </is>
+      </c>
+      <c r="C582" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D582" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09_2214_Dopamine-and-Autism-Traits.md</t>
+        </is>
+      </c>
+      <c r="E582" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F582" s="2" t="inlineStr"/>
+      <c r="G582" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H582" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B583" s="3" t="inlineStr">
+        <is>
+          <t>Fiido D3 Max Speed</t>
+        </is>
+      </c>
+      <c r="C583" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D583" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09_2345_Fiido-D3-Max-Speed.md</t>
+        </is>
+      </c>
+      <c r="E583" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F583" s="2" t="inlineStr"/>
+      <c r="G583" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H583" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="B584" s="3" t="inlineStr">
+        <is>
+          <t>Baking Electronics in Vacuum</t>
+        </is>
+      </c>
+      <c r="C584" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D584" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10_1216_Baking-Electronics-in-Vacuum.md</t>
+        </is>
+      </c>
+      <c r="E584" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F584" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G584" s="3" t="inlineStr">
+        <is>
+          <t>Technical question on baking out electronics in a vacuum chamber, likely related to engineering work.</t>
+        </is>
+      </c>
+      <c r="H584" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="B585" s="3" t="inlineStr">
+        <is>
+          <t>Summarize into statement</t>
+        </is>
+      </c>
+      <c r="C585" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D585" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10_2026_Summarize-into-statement.md</t>
+        </is>
+      </c>
+      <c r="E585" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F585" s="2" t="inlineStr"/>
+      <c r="G585" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H585" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="B586" s="3" t="inlineStr">
+        <is>
+          <t>MCX connector size</t>
+        </is>
+      </c>
+      <c r="C586" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D586" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10_2042_MCX-connector-size.md</t>
+        </is>
+      </c>
+      <c r="E586" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F586" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G586" s="3" t="inlineStr">
+        <is>
+          <t>Technical questions on connectors and differential signalling standards, likely related to engineering work.</t>
+        </is>
+      </c>
+      <c r="H586" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="B587" s="3" t="inlineStr">
+        <is>
+          <t>DIN 41612 Pin Count</t>
+        </is>
+      </c>
+      <c r="C587" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D587" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10_2122_DIN-41612-Pin-Count.md</t>
+        </is>
+      </c>
+      <c r="E587" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F587" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G587" s="3" t="inlineStr">
+        <is>
+          <t>Technical questions on backplane connectors and board interconnect design, likely related to engineering work.</t>
+        </is>
+      </c>
+      <c r="H587" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="B588" s="3" t="inlineStr">
+        <is>
+          <t>Multiplexing IO Techniques</t>
+        </is>
+      </c>
+      <c r="C588" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D588" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10_2214_Multiplexing-IO-Techniques.md</t>
+        </is>
+      </c>
+      <c r="E588" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F588" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G588" s="3" t="inlineStr">
+        <is>
+          <t>Technical questions on multiplexing measurement channels, current sense amplifiers and LDO regulators, likely related to engineering work.</t>
+        </is>
+      </c>
+      <c r="H588" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="B589" s="3" t="inlineStr">
+        <is>
+          <t>Ribbon Cable for 50MHz</t>
+        </is>
+      </c>
+      <c r="C589" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D589" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-10_2323_Ribbon-Cable-for-50MHz.md</t>
+        </is>
+      </c>
+      <c r="E589" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F589" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G589" s="3" t="inlineStr">
+        <is>
+          <t>Technical questions on high-temperature cabling for 50 MHz signals, likely related to engineering work.</t>
+        </is>
+      </c>
+      <c r="H589" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="B590" s="3" t="inlineStr">
+        <is>
+          <t>Connector Width Details</t>
+        </is>
+      </c>
+      <c r="C590" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D590" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11_0021_Connector-Width-Details.md</t>
+        </is>
+      </c>
+      <c r="E590" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F590" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G590" s="3" t="inlineStr">
+        <is>
+          <t>Technical question on connector dimensions, likely related to engineering work.</t>
+        </is>
+      </c>
+      <c r="H590" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="B591" s="3" t="inlineStr">
+        <is>
+          <t>DAC Location Best Practices</t>
+        </is>
+      </c>
+      <c r="C591" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D591" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11_0127_DAC-Location-Best-Practices.md</t>
+        </is>
+      </c>
+      <c r="E591" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F591" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G591" s="3" t="inlineStr">
+        <is>
+          <t>Technical circuit design questions on DAC/ADC, LDO and buck regulator selection and thermal management, likely related to engineering work.</t>
+        </is>
+      </c>
+      <c r="H591" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="B592" s="3" t="inlineStr">
+        <is>
+          <t>Mezzanine Connector Recommendations</t>
+        </is>
+      </c>
+      <c r="C592" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D592" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11_0246_Mezzanine-Connector-Recommendations.md</t>
+        </is>
+      </c>
+      <c r="E592" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F592" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G592" s="3" t="inlineStr">
+        <is>
+          <t>Electronics engineering query on mezzanine connector selection, possibly for the owner's hardware engineering work.</t>
+        </is>
+      </c>
+      <c r="H592" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="B593" s="3" t="inlineStr">
+        <is>
+          <t>Document Transcription</t>
+        </is>
+      </c>
+      <c r="C593" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D593" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11_1028_Document-Transcription.md</t>
+        </is>
+      </c>
+      <c r="E593" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F593" s="2" t="inlineStr"/>
+      <c r="G593" s="3" t="inlineStr">
+        <is>
+          <t>Transcription of the owner's occupational health report addressed to the employer.</t>
+        </is>
+      </c>
+      <c r="H593" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="B594" s="3" t="inlineStr">
+        <is>
+          <t>System Requirements Handbook</t>
+        </is>
+      </c>
+      <c r="C594" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D594" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11_1033_System-Requirements-Handbook.md</t>
+        </is>
+      </c>
+      <c r="E594" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F594" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G594" s="3" t="inlineStr">
+        <is>
+          <t>Producing a system requirements handbook and SRS templates for electronics engineering work.</t>
+        </is>
+      </c>
+      <c r="H594" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="B595" s="3" t="inlineStr">
+        <is>
+          <t>Scooter i9 Max Fitment</t>
+        </is>
+      </c>
+      <c r="C595" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D595" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11_1206_Scooter-i9-Max-Fitment.md</t>
+        </is>
+      </c>
+      <c r="E595" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F595" s="2" t="inlineStr"/>
+      <c r="G595" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H595" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="B596" s="3" t="inlineStr">
+        <is>
+          <t>Compact Apple Pencil Loop</t>
+        </is>
+      </c>
+      <c r="C596" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D596" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11_1210_Compact-Apple-Pencil-Loop.md</t>
+        </is>
+      </c>
+      <c r="E596" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F596" s="2" t="inlineStr"/>
+      <c r="G596" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H596" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="B597" s="3" t="inlineStr">
+        <is>
+          <t>Handbook Consolidation Review</t>
+        </is>
+      </c>
+      <c r="C597" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D597" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11_1406_Handbook-Consolidation-Review.md</t>
+        </is>
+      </c>
+      <c r="E597" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F597" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G597" s="3" t="inlineStr">
+        <is>
+          <t>Consolidating and expanding an electronic systems requirements engineering handbook/standard, linked to a burn-in system programme.</t>
+        </is>
+      </c>
+      <c r="H597" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="B598" s="3" t="inlineStr">
+        <is>
+          <t>Latin for Fluency and Flux</t>
+        </is>
+      </c>
+      <c r="C598" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D598" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-11_1541_Latin-for-Fluency-and-Flux.md</t>
+        </is>
+      </c>
+      <c r="E598" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F598" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G598" s="3" t="inlineStr">
+        <is>
+          <t>Latin terms for physics concepts, possibly for naming a technical or engineering project.</t>
+        </is>
+      </c>
+      <c r="H598" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="B599" s="3" t="inlineStr">
+        <is>
+          <t>35km to mph</t>
+        </is>
+      </c>
+      <c r="C599" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D599" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-12_1221_35km-to-mph.md</t>
+        </is>
+      </c>
+      <c r="E599" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F599" s="2" t="inlineStr"/>
+      <c r="G599" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H599" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="B600" s="3" t="inlineStr">
+        <is>
+          <t>Improving Professional Communication</t>
+        </is>
+      </c>
+      <c r="C600" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D600" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-12_1413_Improving-Professional-Communication.md</t>
+        </is>
+      </c>
+      <c r="E600" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F600" s="2" t="inlineStr"/>
+      <c r="G600" s="3" t="inlineStr">
+        <is>
+          <t>Drafting emails to HR about handling of the occupational health report, closing an informal Teams chat with the line manager, and appraisal feedback on communication.</t>
+        </is>
+      </c>
+      <c r="H600" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="B601" s="3" t="inlineStr">
+        <is>
+          <t>RTV 3140 Flex-Rigid Use</t>
+        </is>
+      </c>
+      <c r="C601" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-005.json</t>
+        </is>
+      </c>
+      <c r="D601" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-12_1555_RTV-3140-Flex-Rigid-Use.md</t>
+        </is>
+      </c>
+      <c r="E601" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F601" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G601" s="3" t="inlineStr">
+        <is>
+          <t>Engineering query on using RTV 3140 as a flex-rigid transition, possibly for hardware engineering work.</t>
+        </is>
+      </c>
+      <c r="H601" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="B602" s="3" t="inlineStr">
+        <is>
+          <t>Occupational Health Report Analysis</t>
+        </is>
+      </c>
+      <c r="C602" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D602" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-13_0131_Occupational-Health-Report-Analysis.md</t>
+        </is>
+      </c>
+      <c r="E602" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F602" s="2" t="inlineStr"/>
+      <c r="G602" s="3" t="inlineStr">
+        <is>
+          <t>Analysis of the occupational health report, appraisal, phased return review meetings with HR and managers, working patterns and reasonable adjustments, and sources of external employment advice.</t>
+        </is>
+      </c>
+      <c r="H602" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="B603" s="3" t="inlineStr">
+        <is>
+          <t>Temp Rated Coax Options</t>
+        </is>
+      </c>
+      <c r="C603" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D603" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-13_0908_Temp-Rated-Coax-Options.md</t>
+        </is>
+      </c>
+      <c r="E603" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F603" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G603" s="3" t="inlineStr">
+        <is>
+          <t>Sourcing 125 degC rated coax cable assemblies, likely for engineering work.</t>
+        </is>
+      </c>
+      <c r="H603" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="B604" s="3" t="inlineStr">
+        <is>
+          <t>Radiation Grade Coax</t>
+        </is>
+      </c>
+      <c r="C604" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D604" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-13_1520_Radiation-Grade-Coax.md</t>
+        </is>
+      </c>
+      <c r="E604" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F604" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G604" s="3" t="inlineStr">
+        <is>
+          <t>Selecting radiation-tolerant coax and twisted-pair cabling, likely for engineering work.</t>
+        </is>
+      </c>
+      <c r="H604" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="B605" s="3" t="inlineStr">
+        <is>
+          <t>Digital Pots in Video</t>
+        </is>
+      </c>
+      <c r="C605" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D605" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-13_1836_Digital-Pots-in-Video.md</t>
+        </is>
+      </c>
+      <c r="E605" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F605" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G605" s="3" t="inlineStr">
+        <is>
+          <t>Circuit design for video amplifier gain and CCD clock edge-rate control, likely for engineering work.</t>
+        </is>
+      </c>
+      <c r="H605" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="B606" s="3" t="inlineStr">
+        <is>
+          <t>Boiler Grunt Causes</t>
+        </is>
+      </c>
+      <c r="C606" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D606" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-13_2227_Boiler-Grunt-Causes.md</t>
+        </is>
+      </c>
+      <c r="E606" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F606" s="2" t="inlineStr"/>
+      <c r="G606" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H606" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-14</t>
+        </is>
+      </c>
+      <c r="B607" s="3" t="inlineStr">
+        <is>
+          <t>Voltage Classification for Reset Restore</t>
+        </is>
+      </c>
+      <c r="C607" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D607" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-14_2158_Voltage-Classification-for-Reset-Restore.md</t>
+        </is>
+      </c>
+      <c r="E607" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F607" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G607" s="3" t="inlineStr">
+        <is>
+          <t>CCD voltage domain classification using the team's usual naming convention, likely for engineering work.</t>
+        </is>
+      </c>
+      <c r="H607" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-14</t>
+        </is>
+      </c>
+      <c r="B608" s="3" t="inlineStr">
+        <is>
+          <t>Slew Rate Control in Rameses</t>
+        </is>
+      </c>
+      <c r="C608" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D608" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-14_2240_Slew-Rate-Control-in-Rameses.md</t>
+        </is>
+      </c>
+      <c r="E608" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F608" s="2" t="inlineStr"/>
+      <c r="G608" s="3" t="inlineStr">
+        <is>
+          <t>Engineering design work on CCD clock driver slew-rate control, headboard/active head test hardware, design review and requirements reporting.</t>
+        </is>
+      </c>
+      <c r="H608" s="2" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="B609" s="3" t="inlineStr">
+        <is>
+          <t>2-Channel LVDS Alternatives</t>
+        </is>
+      </c>
+      <c r="C609" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D609" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-17_2135_2-Channel-LVDS-Alternatives.md</t>
+        </is>
+      </c>
+      <c r="E609" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F609" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G609" s="3" t="inlineStr">
+        <is>
+          <t>Selecting dual and quad LVDS receiver ICs and packages for an electronics design project.</t>
+        </is>
+      </c>
+      <c r="H609" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="B610" s="3" t="inlineStr">
+        <is>
+          <t>Extract Local Library CADSTAR</t>
+        </is>
+      </c>
+      <c r="C610" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D610" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19_1713_Extract-Local-Library-CADSTAR.md</t>
+        </is>
+      </c>
+      <c r="E610" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F610" s="2" t="inlineStr"/>
+      <c r="G610" s="3" t="inlineStr">
+        <is>
+          <t>Migrating a job's component libraries and schematic from CADSTAR to Altium and rebuilding footprints.</t>
+        </is>
+      </c>
+      <c r="H610" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="B611" s="3" t="inlineStr">
+        <is>
+          <t>Best From the Basement Sets</t>
+        </is>
+      </c>
+      <c r="C611" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D611" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19_1844_Best-From-the-Basement-Sets.md</t>
+        </is>
+      </c>
+      <c r="E611" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F611" s="2" t="inlineStr"/>
+      <c r="G611" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H611" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="B612" s="3" t="inlineStr">
+        <is>
+          <t>Fiido D3 Pro Clamp Adjustment</t>
+        </is>
+      </c>
+      <c r="C612" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D612" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19_1913_Fiido-D3-Pro-Clamp-Adjustment.md</t>
+        </is>
+      </c>
+      <c r="E612" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F612" s="2" t="inlineStr"/>
+      <c r="G612" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H612" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="B613" s="3" t="inlineStr">
+        <is>
+          <t>PowerPoint Crash Recovery Tips</t>
+        </is>
+      </c>
+      <c r="C613" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D613" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19_1958_PowerPoint-Crash-Recovery-Tips.md</t>
+        </is>
+      </c>
+      <c r="E613" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F613" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G613" s="3" t="inlineStr">
+        <is>
+          <t>Recovering PowerPoint work lost in a crash; possibly work material.</t>
+        </is>
+      </c>
+      <c r="H613" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="B614" s="3" t="inlineStr">
+        <is>
+          <t>Consolidating Altium Libraries</t>
+        </is>
+      </c>
+      <c r="C614" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D614" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19_2036_Consolidating-Altium-Libraries.md</t>
+        </is>
+      </c>
+      <c r="E614" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F614" s="2" t="inlineStr"/>
+      <c r="G614" s="3" t="inlineStr">
+        <is>
+          <t>Consolidating and migrating PCB design libraries and CADSTAR designs into Altium, including reuse blocks, footprints, 3D models and component sourcing for a work board project.</t>
+        </is>
+      </c>
+      <c r="H614" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B615" s="3" t="inlineStr">
+        <is>
+          <t>HDMI to USB-C Pinout</t>
+        </is>
+      </c>
+      <c r="C615" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D615" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20_0143_HDMI-to-USB-C-Pinout.md</t>
+        </is>
+      </c>
+      <c r="E615" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F615" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G615" s="3" t="inlineStr">
+        <is>
+          <t>Technical engineering question on USB-C to HDMI signal mapping and circuit risks, possibly for professional hardware design work.</t>
+        </is>
+      </c>
+      <c r="H615" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B616" s="3" t="inlineStr">
+        <is>
+          <t>4:1 Video Mux Design</t>
+        </is>
+      </c>
+      <c r="C616" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D616" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20_0207_4-1-Video-Mux-Design.md</t>
+        </is>
+      </c>
+      <c r="E616" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F616" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G616" s="3" t="inlineStr">
+        <is>
+          <t>Engineering design discussion of an analogue mux and op-amp GainCal signal chain and PCB components, possibly for professional hardware work.</t>
+        </is>
+      </c>
+      <c r="H616" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B617" s="3" t="inlineStr">
+        <is>
+          <t>D3 Throttle Debug Code</t>
+        </is>
+      </c>
+      <c r="C617" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D617" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20_0742_D3-Throttle-Debug-Code.md</t>
+        </is>
+      </c>
+      <c r="E617" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F617" s="2" t="inlineStr"/>
+      <c r="G617" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H617" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B618" s="3" t="inlineStr">
+        <is>
+          <t>Explaining ChatGPT's Knowledge</t>
+        </is>
+      </c>
+      <c r="C618" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D618" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20_1532_Explaining-ChatGPT-s-Knowledge.md</t>
+        </is>
+      </c>
+      <c r="E618" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F618" s="2" t="inlineStr"/>
+      <c r="G618" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H618" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B619" s="3" t="inlineStr">
+        <is>
+          <t>Pension Decision Making Guide</t>
+        </is>
+      </c>
+      <c r="C619" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D619" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20_1621_Pension-Decision-Making-Guide.md</t>
+        </is>
+      </c>
+      <c r="E619" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F619" s="2" t="inlineStr"/>
+      <c r="G619" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H619" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B620" s="3" t="inlineStr">
+        <is>
+          <t>MCX vs UMC Differences</t>
+        </is>
+      </c>
+      <c r="C620" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D620" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20_1645_MCX-vs-UMC-Differences.md</t>
+        </is>
+      </c>
+      <c r="E620" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F620" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G620" s="3" t="inlineStr">
+        <is>
+          <t>Technical question on RF connector choice and a monitor tap resistor in a circuit, possibly for professional hardware design work.</t>
+        </is>
+      </c>
+      <c r="H620" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B621" s="3" t="inlineStr">
+        <is>
+          <t>LVDS SPI over Ribbon Cable</t>
+        </is>
+      </c>
+      <c r="C621" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D621" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20_1829_LVDS-SPI-over-Ribbon-Cable.md</t>
+        </is>
+      </c>
+      <c r="E621" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F621" s="2" t="inlineStr"/>
+      <c r="G621" s="3" t="inlineStr">
+        <is>
+          <t>Engineering design discussion of an LVDS link into a thermal chamber for an internal customer requirement.</t>
+        </is>
+      </c>
+      <c r="H621" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-21</t>
+        </is>
+      </c>
+      <c r="B622" s="3" t="inlineStr">
+        <is>
+          <t>Fiido D3 Speed Limit</t>
+        </is>
+      </c>
+      <c r="C622" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D622" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-21_1152_Fiido-D3-Speed-Limit.md</t>
+        </is>
+      </c>
+      <c r="E622" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F622" s="2" t="inlineStr"/>
+      <c r="G622" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H622" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-21</t>
+        </is>
+      </c>
+      <c r="B623" s="3" t="inlineStr">
+        <is>
+          <t>Document Comparison</t>
+        </is>
+      </c>
+      <c r="C623" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D623" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-21_1330_Document-Comparison.md</t>
+        </is>
+      </c>
+      <c r="E623" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F623" s="2" t="inlineStr"/>
+      <c r="G623" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H623" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-21</t>
+        </is>
+      </c>
+      <c r="B624" s="3" t="inlineStr">
+        <is>
+          <t>External cabin wall structure</t>
+        </is>
+      </c>
+      <c r="C624" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D624" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-21_1939_External-cabin-wall-structure.md</t>
+        </is>
+      </c>
+      <c r="E624" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F624" s="2" t="inlineStr"/>
+      <c r="G624" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H624" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-21</t>
+        </is>
+      </c>
+      <c r="B625" s="3" t="inlineStr">
+        <is>
+          <t>Dating App Response Timing</t>
+        </is>
+      </c>
+      <c r="C625" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D625" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-21_2234_Dating-App-Response-Timing.md</t>
+        </is>
+      </c>
+      <c r="E625" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F625" s="2" t="inlineStr"/>
+      <c r="G625" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H625" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
+        </is>
+      </c>
+      <c r="B626" s="3" t="inlineStr">
+        <is>
+          <t>Data Centre Job Skills</t>
+        </is>
+      </c>
+      <c r="C626" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D626" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-22_1131_Data-Centre-Job-Skills.md</t>
+        </is>
+      </c>
+      <c r="E626" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F626" s="2" t="inlineStr"/>
+      <c r="G626" s="3" t="inlineStr">
+        <is>
+          <t>Career question on data-centre job roles and skills development for employment.</t>
+        </is>
+      </c>
+      <c r="H626" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
+        </is>
+      </c>
+      <c r="B627" s="3" t="inlineStr">
+        <is>
+          <t>Firing Employees Challenges</t>
+        </is>
+      </c>
+      <c r="C627" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D627" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-22_1242_Firing-Employees-Challenges.md</t>
+        </is>
+      </c>
+      <c r="E627" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F627" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G627" s="3" t="inlineStr">
+        <is>
+          <t>General question on why dismissing employees is difficult under employment law.</t>
+        </is>
+      </c>
+      <c r="H627" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
+        </is>
+      </c>
+      <c r="B628" s="3" t="inlineStr">
+        <is>
+          <t>Dell Display Manager Function</t>
+        </is>
+      </c>
+      <c r="C628" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D628" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-22_1935_Dell-Display-Manager-Function.md</t>
+        </is>
+      </c>
+      <c r="E628" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F628" s="2" t="inlineStr"/>
+      <c r="G628" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H628" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="B629" s="3" t="inlineStr">
+        <is>
+          <t>Altium CircuitStudio Overview</t>
+        </is>
+      </c>
+      <c r="C629" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D629" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23_1025_Altium-CircuitStudio-Overview.md</t>
+        </is>
+      </c>
+      <c r="E629" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F629" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G629" s="3" t="inlineStr">
+        <is>
+          <t>Questions about Altium PCB design tool licensing under an enterprise subscription, possibly for professional work.</t>
+        </is>
+      </c>
+      <c r="H629" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="B630" s="3" t="inlineStr">
+        <is>
+          <t>Moving Pin Numbers Altium</t>
+        </is>
+      </c>
+      <c r="C630" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D630" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23_1638_Moving-Pin-Numbers-Altium.md</t>
+        </is>
+      </c>
+      <c r="E630" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F630" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G630" s="3" t="inlineStr">
+        <is>
+          <t>Technical question on editing pin designators in Altium, possibly for professional design work.</t>
+        </is>
+      </c>
+      <c r="H630" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B631" s="3" t="inlineStr">
+        <is>
+          <t>ASD Assessment Narrative</t>
+        </is>
+      </c>
+      <c r="C631" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D631" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-24_0902_ASD-Assessment-Narrative.md</t>
+        </is>
+      </c>
+      <c r="E631" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F631" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G631" s="3" t="inlineStr">
+        <is>
+          <t>Summary of supporting documents includes work functioning, work performance concerns and an Occupational Health assessment; a later evidence table references a change of work role.</t>
+        </is>
+      </c>
+      <c r="H631" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B632" s="3" t="inlineStr">
+        <is>
+          <t>Autism Assessment Reflection</t>
+        </is>
+      </c>
+      <c r="C632" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D632" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-24_1641_Autism-Assessment-Reflection.md</t>
+        </is>
+      </c>
+      <c r="E632" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F632" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G632" s="3" t="inlineStr">
+        <is>
+          <t>Brief reference to being asked to describe their job and answering at length.</t>
+        </is>
+      </c>
+      <c r="H632" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="B633" s="3" t="inlineStr">
+        <is>
+          <t>Schematic PCB Sync Issue</t>
+        </is>
+      </c>
+      <c r="C633" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D633" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-25_1646_Schematic-PCB-Sync-Issue.md</t>
+        </is>
+      </c>
+      <c r="E633" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F633" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G633" s="3" t="inlineStr">
+        <is>
+          <t>Altium schematic/PCB synchronisation and annotation issues in a PCB design project.</t>
+        </is>
+      </c>
+      <c r="H633" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="B634" s="3" t="inlineStr">
+        <is>
+          <t>DG412 Single Gate Equivalent</t>
+        </is>
+      </c>
+      <c r="C634" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D634" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-25_2338_DG412-Single-Gate-Equivalent.md</t>
+        </is>
+      </c>
+      <c r="E634" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F634" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G634" s="3" t="inlineStr">
+        <is>
+          <t>Component selection and decoupling for an analog switch in a circuit design.</t>
+        </is>
+      </c>
+      <c r="H634" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="B635" s="3" t="inlineStr">
+        <is>
+          <t>Reuse Block Troubleshooting</t>
+        </is>
+      </c>
+      <c r="C635" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D635" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-26_1535_Reuse-Block-Troubleshooting.md</t>
+        </is>
+      </c>
+      <c r="E635" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F635" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G635" s="3" t="inlineStr">
+        <is>
+          <t>Altium reuse blocks, library management and schematic-to-PCB updates across design jobs.</t>
+        </is>
+      </c>
+      <c r="H635" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="B636" s="3" t="inlineStr">
+        <is>
+          <t>Layers</t>
+        </is>
+      </c>
+      <c r="C636" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D636" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27_1030_Layers.md</t>
+        </is>
+      </c>
+      <c r="E636" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F636" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G636" s="3" t="inlineStr">
+        <is>
+          <t>Altium multi-channel design, room replication and PCB stackup thickness for a 12-layer board.</t>
+        </is>
+      </c>
+      <c r="H636" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="B637" s="3" t="inlineStr">
+        <is>
+          <t>Missing connections in Altium</t>
+        </is>
+      </c>
+      <c r="C637" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D637" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27_1531_Missing-connections-in-Altium.md</t>
+        </is>
+      </c>
+      <c r="E637" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F637" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G637" s="3" t="inlineStr">
+        <is>
+          <t>Altium PCB layout tasks including ECO updates, rooms, layout replication and decoupling.</t>
+        </is>
+      </c>
+      <c r="H637" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H520"/>
+  <autoFilter ref="A1:H637"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19720,7 +24080,7 @@
         </is>
       </c>
       <c r="B1" t="n">
-        <v>519</v>
+        <v>636</v>
       </c>
     </row>
     <row r="2">
@@ -19730,7 +24090,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>109</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3">
@@ -19740,7 +24100,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4">
@@ -19750,7 +24110,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>174</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5">
@@ -19760,7 +24120,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>345</v>
+        <v>414</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
chat-sift: batches b80-b89 read; index, extracts and progress updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aq7txTcfpUgzabiqqnXaKj
</commit_message>
<xml_diff>
--- a/chat-sift/output/index.xlsx
+++ b/chat-sift/output/index.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$637</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$720</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H637"/>
+  <dimension ref="A1:H720"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24055,8 +24055,3156 @@
         <v>1</v>
       </c>
     </row>
+    <row r="638">
+      <c r="A638" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="B638" s="3" t="inlineStr">
+        <is>
+          <t>Symbol Meaning in Altium</t>
+        </is>
+      </c>
+      <c r="C638" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D638" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27_2116_Symbol-Meaning-in-Altium.md</t>
+        </is>
+      </c>
+      <c r="E638" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F638" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G638" s="3" t="inlineStr">
+        <is>
+          <t>PCB design work in Altium: room replication, component renumbering and schematic grid issues.</t>
+        </is>
+      </c>
+      <c r="H638" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="B639" s="3" t="inlineStr">
+        <is>
+          <t>Turn off net highlights</t>
+        </is>
+      </c>
+      <c r="C639" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D639" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-01_1756_Turn-off-net-highlights.md</t>
+        </is>
+      </c>
+      <c r="E639" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F639" s="2" t="inlineStr"/>
+      <c r="G639" s="3" t="inlineStr">
+        <is>
+          <t>Schematic and library work in Altium, including company grid standards, BOM attributes and connector reference conventions.</t>
+        </is>
+      </c>
+      <c r="H639" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B640" s="3" t="inlineStr">
+        <is>
+          <t>TQFP Meaning Explained</t>
+        </is>
+      </c>
+      <c r="C640" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D640" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-02_1921_TQFP-Meaning-Explained.md</t>
+        </is>
+      </c>
+      <c r="E640" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F640" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G640" s="3" t="inlineStr">
+        <is>
+          <t>Electronics design questions on component packages and LVDS signalling distance and cabling.</t>
+        </is>
+      </c>
+      <c r="H640" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="B641" s="3" t="inlineStr">
+        <is>
+          <t>74HC595 Data Clock Delay</t>
+        </is>
+      </c>
+      <c r="C641" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D641" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-03_0201_74HC595-Data-Clock-Delay.md</t>
+        </is>
+      </c>
+      <c r="E641" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F641" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G641" s="3" t="inlineStr">
+        <is>
+          <t>Electronics design question on driving a shift register from a single line and simulating it in Multisim.</t>
+        </is>
+      </c>
+      <c r="H641" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="B642" s="3" t="inlineStr">
+        <is>
+          <t>Polygon Cleanup in Altium</t>
+        </is>
+      </c>
+      <c r="C642" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D642" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-03_1544_Polygon-Cleanup-in-Altium.md</t>
+        </is>
+      </c>
+      <c r="E642" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F642" s="2" t="inlineStr"/>
+      <c r="G642" s="3" t="inlineStr">
+        <is>
+          <t>Taking over a PCB design in Altium: polygon cleanup, component link and ECO problems, LVDS part selection and remote access.</t>
+        </is>
+      </c>
+      <c r="H642" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="B643" s="3" t="inlineStr">
+        <is>
+          <t>Importing DXF in Altium</t>
+        </is>
+      </c>
+      <c r="C643" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D643" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-03_1804_Importing-DXF-in-Altium.md</t>
+        </is>
+      </c>
+      <c r="E643" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F643" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G643" s="3" t="inlineStr">
+        <is>
+          <t>Altium PCB work: importing a DXF board outline and graphics settings on a remotely accessed workstation.</t>
+        </is>
+      </c>
+      <c r="H643" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="B644" s="3" t="inlineStr">
+        <is>
+          <t>Unclear Explanation</t>
+        </is>
+      </c>
+      <c r="C644" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D644" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04_1009_Unclear-Explanation.md</t>
+        </is>
+      </c>
+      <c r="E644" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F644" s="2" t="inlineStr"/>
+      <c r="G644" s="3" t="inlineStr">
+        <is>
+          <t>Setting up Altium multi-channel design on a real project and merging it with a legacy design.</t>
+        </is>
+      </c>
+      <c r="H644" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="B645" s="3" t="inlineStr">
+        <is>
+          <t>OS Current Measurement</t>
+        </is>
+      </c>
+      <c r="C645" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D645" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04_1651_OS-Current-Measurement.md</t>
+        </is>
+      </c>
+      <c r="E645" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F645" s="2" t="inlineStr"/>
+      <c r="G645" s="3" t="inlineStr">
+        <is>
+          <t>Engineering design discussion for a work requirement on measuring and monitoring CCD OS current and voltage on a test board.</t>
+        </is>
+      </c>
+      <c r="H645" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="B646" s="3" t="inlineStr">
+        <is>
+          <t>Hardware Test Ideas</t>
+        </is>
+      </c>
+      <c r="C646" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D646" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04_1903_Hardware-Test-Ideas.md</t>
+        </is>
+      </c>
+      <c r="E646" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F646" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G646" s="3" t="inlineStr">
+        <is>
+          <t>Hardware design discussion on built-in test features for a shift-register gain-selection circuit on a board.</t>
+        </is>
+      </c>
+      <c r="H646" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="B647" s="3" t="inlineStr">
+        <is>
+          <t>PCB Test Plan</t>
+        </is>
+      </c>
+      <c r="C647" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D647" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04_2132_PCB-Test-Plan.md</t>
+        </is>
+      </c>
+      <c r="E647" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F647" s="2" t="inlineStr"/>
+      <c r="G647" s="3" t="inlineStr">
+        <is>
+          <t>Drafting a PCB test plan against a requirements document for a CCD test-camera board.</t>
+        </is>
+      </c>
+      <c r="H647" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="B648" s="3" t="inlineStr">
+        <is>
+          <t>Net rename in Altium</t>
+        </is>
+      </c>
+      <c r="C648" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D648" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-05_1854_Net-rename-in-Altium.md</t>
+        </is>
+      </c>
+      <c r="E648" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F648" s="2" t="inlineStr"/>
+      <c r="G648" s="3" t="inlineStr">
+        <is>
+          <t>Altium schematic/PCB design issues on a board project (net rename, version history, track width).</t>
+        </is>
+      </c>
+      <c r="H648" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="B649" s="3" t="inlineStr">
+        <is>
+          <t>Cat Hair Loss Causes</t>
+        </is>
+      </c>
+      <c r="C649" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D649" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-05_1934_Cat-Hair-Loss-Causes.md</t>
+        </is>
+      </c>
+      <c r="E649" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F649" s="2" t="inlineStr"/>
+      <c r="G649" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H649" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B650" s="3" t="inlineStr">
+        <is>
+          <t>Perplexity AI Usage</t>
+        </is>
+      </c>
+      <c r="C650" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D650" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-06_0943_Perplexity-AI-Usage.md</t>
+        </is>
+      </c>
+      <c r="E650" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F650" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G650" s="3" t="inlineStr">
+        <is>
+          <t>Whether an AI search tool is safe for sensitive information in the owner's engineering work context.</t>
+        </is>
+      </c>
+      <c r="H650" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B651" s="3" t="inlineStr">
+        <is>
+          <t>CDR Report Rewrite</t>
+        </is>
+      </c>
+      <c r="C651" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D651" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-06_0950_CDR-Report-Rewrite.md</t>
+        </is>
+      </c>
+      <c r="E651" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F651" s="2" t="inlineStr"/>
+      <c r="G651" s="3" t="inlineStr">
+        <is>
+          <t>Restructuring a CDR design report for a CCD test camera headboard project.</t>
+        </is>
+      </c>
+      <c r="H651" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B652" s="3" t="inlineStr">
+        <is>
+          <t>Fiido Unlock with Apple Watch</t>
+        </is>
+      </c>
+      <c r="C652" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D652" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-06_1044_Fiido-Unlock-with-Apple-Watch.md</t>
+        </is>
+      </c>
+      <c r="E652" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F652" s="2" t="inlineStr"/>
+      <c r="G652" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H652" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="B653" s="3" t="inlineStr">
+        <is>
+          <t>Diagram Style Recognition</t>
+        </is>
+      </c>
+      <c r="C653" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D653" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-06_1318_Diagram-Style-Recognition.md</t>
+        </is>
+      </c>
+      <c r="E653" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F653" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G653" s="3" t="inlineStr">
+        <is>
+          <t>Identifying the tool used to produce engineering design-review diagrams.</t>
+        </is>
+      </c>
+      <c r="H653" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="B654" s="3" t="inlineStr">
+        <is>
+          <t>Creating Altium Manual Sources</t>
+        </is>
+      </c>
+      <c r="C654" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D654" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-07_1040_Creating-Altium-Manual-Sources.md</t>
+        </is>
+      </c>
+      <c r="E654" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F654" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G654" s="3" t="inlineStr">
+        <is>
+          <t>Gathering sources for an Altium design software manual.</t>
+        </is>
+      </c>
+      <c r="H654" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="B655" s="3" t="inlineStr">
+        <is>
+          <t>Multichannel Signal Naming</t>
+        </is>
+      </c>
+      <c r="C655" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D655" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-07_2150_Multichannel-Signal-Naming.md</t>
+        </is>
+      </c>
+      <c r="E655" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F655" s="2" t="inlineStr"/>
+      <c r="G655" s="3" t="inlineStr">
+        <is>
+          <t>Altium schematic multichannel clock naming and hierarchy compile errors for the CCD38x interface design.</t>
+        </is>
+      </c>
+      <c r="H655" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+      <c r="B656" s="3" t="inlineStr">
+        <is>
+          <t>JLab Mouse Configuration</t>
+        </is>
+      </c>
+      <c r="C656" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D656" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-08_1830_JLab-Mouse-Configuration.md</t>
+        </is>
+      </c>
+      <c r="E656" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F656" s="2" t="inlineStr"/>
+      <c r="G656" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H656" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B657" s="3" t="inlineStr">
+        <is>
+          <t>Net Name Issue</t>
+        </is>
+      </c>
+      <c r="C657" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D657" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-09_0032_Net-Name-Issue.md</t>
+        </is>
+      </c>
+      <c r="E657" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F657" s="2" t="inlineStr"/>
+      <c r="G657" s="3" t="inlineStr">
+        <is>
+          <t>Altium schematic net naming query on a CCD bias net.</t>
+        </is>
+      </c>
+      <c r="H657" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B658" s="3" t="inlineStr">
+        <is>
+          <t>Clock Net Naming Fix</t>
+        </is>
+      </c>
+      <c r="C658" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D658" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-09_0354_Clock-Net-Naming-Fix.md</t>
+        </is>
+      </c>
+      <c r="E658" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F658" s="2" t="inlineStr"/>
+      <c r="G658" s="3" t="inlineStr">
+        <is>
+          <t>Altium schematic clock net naming, multichannel reuse block and duplicate net errors.</t>
+        </is>
+      </c>
+      <c r="H658" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="B659" s="3" t="inlineStr">
+        <is>
+          <t>Multiple Top-Level Documents</t>
+        </is>
+      </c>
+      <c r="C659" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D659" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-11_1441_Multiple-Top-Level-Documents.md</t>
+        </is>
+      </c>
+      <c r="E659" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F659" s="2" t="inlineStr"/>
+      <c r="G659" s="3" t="inlineStr">
+        <is>
+          <t>Altium compile error about multiple top-level documents in the CCD38x interface design.</t>
+        </is>
+      </c>
+      <c r="H659" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="B660" s="3" t="inlineStr">
+        <is>
+          <t>Negative Feedback Resistors x5</t>
+        </is>
+      </c>
+      <c r="C660" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D660" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-12_0950_Negative-Feedback-Resistors-x5.md</t>
+        </is>
+      </c>
+      <c r="E660" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F660" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G660" s="3" t="inlineStr">
+        <is>
+          <t>Electronics circuit design and Altium multichannel schematic/PCB questions, likely for professional design work.</t>
+        </is>
+      </c>
+      <c r="H660" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="B661" s="3" t="inlineStr">
+        <is>
+          <t>Altium Pin Designator Issue</t>
+        </is>
+      </c>
+      <c r="C661" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D661" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-15_2025_Altium-Pin-Designator-Issue.md</t>
+        </is>
+      </c>
+      <c r="E661" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F661" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G661" s="3" t="inlineStr">
+        <is>
+          <t>Altium symbol/footprint pin designator mapping for a connector part, likely professional design work.</t>
+        </is>
+      </c>
+      <c r="H661" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B662" s="3" t="inlineStr">
+        <is>
+          <t>Comfortable Bike Seat Replacement</t>
+        </is>
+      </c>
+      <c r="C662" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D662" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16_0747_Comfortable-Bike-Seat-Replacement.md</t>
+        </is>
+      </c>
+      <c r="E662" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F662" s="2" t="inlineStr"/>
+      <c r="G662" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H662" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B663" s="3" t="inlineStr">
+        <is>
+          <t>Melatonin Caffeine Creativity Effects</t>
+        </is>
+      </c>
+      <c r="C663" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D663" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16_1406_Melatonin-Caffeine-Creativity-Effects.md</t>
+        </is>
+      </c>
+      <c r="E663" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F663" s="2" t="inlineStr"/>
+      <c r="G663" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H663" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B664" s="3" t="inlineStr">
+        <is>
+          <t>Electronics Sales Strategy</t>
+        </is>
+      </c>
+      <c r="C664" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D664" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16_1739_Electronics-Sales-Strategy.md</t>
+        </is>
+      </c>
+      <c r="E664" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F664" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G664" s="3" t="inlineStr">
+        <is>
+          <t>Commercial and product-compliance strategy for selling a lab electronics system.</t>
+        </is>
+      </c>
+      <c r="H664" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B665" s="3" t="inlineStr">
+        <is>
+          <t>19" Rackmount LCD Console</t>
+        </is>
+      </c>
+      <c r="C665" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D665" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16_1749_19-Rackmount-LCD-Console.md</t>
+        </is>
+      </c>
+      <c r="E665" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F665" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G665" s="3" t="inlineStr">
+        <is>
+          <t>Rackmount console and operator-station options for a lab/test rack.</t>
+        </is>
+      </c>
+      <c r="H665" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B666" s="3" t="inlineStr">
+        <is>
+          <t>What is an EMP</t>
+        </is>
+      </c>
+      <c r="C666" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D666" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16_1808_What-is-an-EMP.md</t>
+        </is>
+      </c>
+      <c r="E666" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F666" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G666" s="3" t="inlineStr">
+        <is>
+          <t>Structure and draft of an Engineering Management Plan including a market-placement and compliance section for a lab electronics platform.</t>
+        </is>
+      </c>
+      <c r="H666" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B667" s="3" t="inlineStr">
+        <is>
+          <t>Boiler Warranty Information</t>
+        </is>
+      </c>
+      <c r="C667" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D667" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16_1858_Boiler-Warranty-Information.md</t>
+        </is>
+      </c>
+      <c r="E667" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F667" s="2" t="inlineStr"/>
+      <c r="G667" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H667" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B668" s="3" t="inlineStr">
+        <is>
+          <t>User inquiry</t>
+        </is>
+      </c>
+      <c r="C668" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D668" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16_2243_User-inquiry.md</t>
+        </is>
+      </c>
+      <c r="E668" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F668" s="2" t="inlineStr"/>
+      <c r="G668" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H668" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B669" s="3" t="inlineStr">
+        <is>
+          <t>ADHD Medication Alternatives</t>
+        </is>
+      </c>
+      <c r="C669" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D669" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17_0927_ADHD-Medication-Alternatives.md</t>
+        </is>
+      </c>
+      <c r="E669" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F669" s="2" t="inlineStr"/>
+      <c r="G669" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H669" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B670" s="3" t="inlineStr">
+        <is>
+          <t>Access to Private Land</t>
+        </is>
+      </c>
+      <c r="C670" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D670" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17_1205_Access-to-Private-Land.md</t>
+        </is>
+      </c>
+      <c r="E670" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F670" s="2" t="inlineStr"/>
+      <c r="G670" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H670" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B671" s="3" t="inlineStr">
+        <is>
+          <t>ASD Assessment Process Clarification</t>
+        </is>
+      </c>
+      <c r="C671" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D671" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17_1354_ASD-Assessment-Process-Clarification.md</t>
+        </is>
+      </c>
+      <c r="E671" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F671" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G671" s="3" t="inlineStr">
+        <is>
+          <t>Mentions occupational health as a source of documentation.</t>
+        </is>
+      </c>
+      <c r="H671" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B672" s="3" t="inlineStr">
+        <is>
+          <t>Pre-show Stage Explanation</t>
+        </is>
+      </c>
+      <c r="C672" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D672" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17_1600_Pre-show-Stage-Explanation.md</t>
+        </is>
+      </c>
+      <c r="E672" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F672" s="2" t="inlineStr"/>
+      <c r="G672" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H672" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B673" s="3" t="inlineStr">
+        <is>
+          <t>Dragon vs Microsoft Dictation</t>
+        </is>
+      </c>
+      <c r="C673" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D673" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17_1711_Dragon-vs-Microsoft-Dictation.md</t>
+        </is>
+      </c>
+      <c r="E673" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F673" s="2" t="inlineStr"/>
+      <c r="G673" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H673" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B674" s="3" t="inlineStr">
+        <is>
+          <t>Next antidepressant after vortioxetine</t>
+        </is>
+      </c>
+      <c r="C674" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D674" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17_2201_Next-antidepressant-after-vortioxetine.md</t>
+        </is>
+      </c>
+      <c r="E674" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F674" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G674" s="3" t="inlineStr">
+        <is>
+          <t>Mentions a period of intense working, sometimes overnight.</t>
+        </is>
+      </c>
+      <c r="H674" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B675" s="3" t="inlineStr">
+        <is>
+          <t>Underworld Dirty Epic Meaning</t>
+        </is>
+      </c>
+      <c r="C675" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D675" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-18_1851_Underworld-Dirty-Epic-Meaning.md</t>
+        </is>
+      </c>
+      <c r="E675" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F675" s="2" t="inlineStr"/>
+      <c r="G675" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H675" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B676" s="3" t="inlineStr">
+        <is>
+          <t>Cimembt Stucjnon Issue</t>
+        </is>
+      </c>
+      <c r="C676" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D676" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-19_1201_Cimembt-Stucjnon-Issue.md</t>
+        </is>
+      </c>
+      <c r="E676" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F676" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G676" s="3" t="inlineStr">
+        <is>
+          <t>Altium schematic library Comment parameter not updating, likely professional design work.</t>
+        </is>
+      </c>
+      <c r="H676" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B677" s="3" t="inlineStr">
+        <is>
+          <t>Removing U_ Prefix in Altium</t>
+        </is>
+      </c>
+      <c r="C677" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D677" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-20_0548_Removing-U-Prefix-in-Altium.md</t>
+        </is>
+      </c>
+      <c r="E677" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F677" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G677" s="3" t="inlineStr">
+        <is>
+          <t>Altium sheet symbol naming, and a workplace discussion with a colleague about component library standards and use of the Comment field.</t>
+        </is>
+      </c>
+      <c r="H677" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B678" s="3" t="inlineStr">
+        <is>
+          <t>Charity Shop Find</t>
+        </is>
+      </c>
+      <c r="C678" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D678" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-20_0749_Charity-Shop-Find.md</t>
+        </is>
+      </c>
+      <c r="E678" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F678" s="2" t="inlineStr"/>
+      <c r="G678" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H678" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B679" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp Timed Images</t>
+        </is>
+      </c>
+      <c r="C679" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D679" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-20_1208_WhatsApp-Timed-Images.md</t>
+        </is>
+      </c>
+      <c r="E679" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F679" s="2" t="inlineStr"/>
+      <c r="G679" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H679" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B680" s="3" t="inlineStr">
+        <is>
+          <t>E-bike storage canopy</t>
+        </is>
+      </c>
+      <c r="C680" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D680" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-21_0641_E-bike-storage-canopy.md</t>
+        </is>
+      </c>
+      <c r="E680" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F680" s="2" t="inlineStr"/>
+      <c r="G680" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H680" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B681" s="3" t="inlineStr">
+        <is>
+          <t>Front Wheel Motor Setup</t>
+        </is>
+      </c>
+      <c r="C681" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D681" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-21_1000_Front-Wheel-Motor-Setup.md</t>
+        </is>
+      </c>
+      <c r="E681" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F681" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G681" s="3" t="inlineStr">
+        <is>
+          <t>Discusses electronics circuit design choices for a CCD signal monitoring board, including component selection, schematic layout and anticipated design review by a colleague.</t>
+        </is>
+      </c>
+      <c r="H681" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B682" s="3" t="inlineStr">
+        <is>
+          <t>Cabin Studio Rental Pricing</t>
+        </is>
+      </c>
+      <c r="C682" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D682" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-21_1542_Cabin-Studio-Rental-Pricing.md</t>
+        </is>
+      </c>
+      <c r="E682" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F682" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G682" s="3" t="inlineStr">
+        <is>
+          <t>Discusses a possible venture renting out a cabin studio, including pricing and planning considerations.</t>
+        </is>
+      </c>
+      <c r="H682" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="B683" s="3" t="inlineStr">
+        <is>
+          <t>Cement board packing uses</t>
+        </is>
+      </c>
+      <c r="C683" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D683" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-21_2101_Cement-board-packing-uses.md</t>
+        </is>
+      </c>
+      <c r="E683" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F683" s="2" t="inlineStr"/>
+      <c r="G683" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H683" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B684" s="3" t="inlineStr">
+        <is>
+          <t>Angle Calculation Assistance</t>
+        </is>
+      </c>
+      <c r="C684" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D684" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22_0730_Angle-Calculation-Assistance.md</t>
+        </is>
+      </c>
+      <c r="E684" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F684" s="2" t="inlineStr"/>
+      <c r="G684" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H684" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B685" s="3" t="inlineStr">
+        <is>
+          <t>Laptop Sluggishness Diagnosis</t>
+        </is>
+      </c>
+      <c r="C685" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D685" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22_0917_Laptop-Sluggishness-Diagnosis.md</t>
+        </is>
+      </c>
+      <c r="E685" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F685" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G685" s="3" t="inlineStr">
+        <is>
+          <t>Performance of the owner's managed work laptop, and Altium PCB/schematic tool settings and CPLD SPI fanout design questions.</t>
+        </is>
+      </c>
+      <c r="H685" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="B686" s="3" t="inlineStr">
+        <is>
+          <t>Text Positioning Issues</t>
+        </is>
+      </c>
+      <c r="C686" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D686" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-22_1545_Text-Positioning-Issues.md</t>
+        </is>
+      </c>
+      <c r="E686" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F686" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G686" s="3" t="inlineStr">
+        <is>
+          <t>Altium schematic library component text positioning and multi-window setup.</t>
+        </is>
+      </c>
+      <c r="H686" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B687" s="3" t="inlineStr">
+        <is>
+          <t>x5 Signal Weighting Differences</t>
+        </is>
+      </c>
+      <c r="C687" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D687" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-23_0026_x5-Signal-Weighting-Differences.md</t>
+        </is>
+      </c>
+      <c r="E687" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F687" s="2" t="inlineStr"/>
+      <c r="G687" s="3" t="inlineStr">
+        <is>
+          <t>Electronics design work on a detector headboard (output buffering, clock slew, designator conventions), a design review meeting, and restructuring of the CDR design report.</t>
+        </is>
+      </c>
+      <c r="H687" s="2" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B688" s="3" t="inlineStr">
+        <is>
+          <t>Graphic Enhancement Request</t>
+        </is>
+      </c>
+      <c r="C688" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D688" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-23_2313_Graphic-Enhancement-Request.md</t>
+        </is>
+      </c>
+      <c r="E688" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F688" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G688" s="3" t="inlineStr">
+        <is>
+          <t>Requests for a CPLD graphic for a technical digital hierarchy block diagram.</t>
+        </is>
+      </c>
+      <c r="H688" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B689" s="3" t="inlineStr">
+        <is>
+          <t>Altium Access Benefits</t>
+        </is>
+      </c>
+      <c r="C689" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D689" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24_1012_Altium-Access-Benefits.md</t>
+        </is>
+      </c>
+      <c r="E689" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F689" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G689" s="3" t="inlineStr">
+        <is>
+          <t>Use of MS Access as a component database backend for Altium PCB design libraries.</t>
+        </is>
+      </c>
+      <c r="H689" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B690" s="3" t="inlineStr">
+        <is>
+          <t>Syncing Function Generators</t>
+        </is>
+      </c>
+      <c r="C690" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D690" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24_1551_Syncing-Function-Generators.md</t>
+        </is>
+      </c>
+      <c r="E690" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F690" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G690" s="3" t="inlineStr">
+        <is>
+          <t>Synchronising function generators in a Multisim circuit design.</t>
+        </is>
+      </c>
+      <c r="H690" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B691" s="3" t="inlineStr">
+        <is>
+          <t>Switching Units in Altium</t>
+        </is>
+      </c>
+      <c r="C691" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D691" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24_1700_Switching-Units-in-Altium.md</t>
+        </is>
+      </c>
+      <c r="E691" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F691" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G691" s="3" t="inlineStr">
+        <is>
+          <t>Switching editor units in Altium design software.</t>
+        </is>
+      </c>
+      <c r="H691" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B692" s="3" t="inlineStr">
+        <is>
+          <t>Relay Position Check</t>
+        </is>
+      </c>
+      <c r="C692" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D692" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24_2128_Relay-Position-Check.md</t>
+        </is>
+      </c>
+      <c r="E692" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F692" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G692" s="3" t="inlineStr">
+        <is>
+          <t>Checking a relay position on a circuit schematic.</t>
+        </is>
+      </c>
+      <c r="H692" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B693" s="3" t="inlineStr">
+        <is>
+          <t>Relay Contact Configuration</t>
+        </is>
+      </c>
+      <c r="C693" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D693" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24_2147_Relay-Contact-Configuration.md</t>
+        </is>
+      </c>
+      <c r="E693" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F693" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G693" s="3" t="inlineStr">
+        <is>
+          <t>Relay contact configuration and sampling path placement on a CCD readout schematic.</t>
+        </is>
+      </c>
+      <c r="H693" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B694" s="3" t="inlineStr">
+        <is>
+          <t>Altium Slew Rate Evaluation</t>
+        </is>
+      </c>
+      <c r="C694" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D694" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25_1255_Altium-Slew-Rate-Evaluation.md</t>
+        </is>
+      </c>
+      <c r="E694" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F694" s="2" t="inlineStr"/>
+      <c r="G694" s="3" t="inlineStr">
+        <is>
+          <t>Evaluating CCD clock driver slew rates using Altium simulation and circuit stage design.</t>
+        </is>
+      </c>
+      <c r="H694" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B695" s="3" t="inlineStr">
+        <is>
+          <t>Power Net Component Report</t>
+        </is>
+      </c>
+      <c r="C695" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D695" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25_1544_Power-Net-Component-Report.md</t>
+        </is>
+      </c>
+      <c r="E695" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F695" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G695" s="3" t="inlineStr">
+        <is>
+          <t>Generating an Altium report of components on a power net.</t>
+        </is>
+      </c>
+      <c r="H695" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B696" s="3" t="inlineStr">
+        <is>
+          <t>Slew Rate and Amplifiers</t>
+        </is>
+      </c>
+      <c r="C696" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D696" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-26_1653_Slew-Rate-and-Amplifiers.md</t>
+        </is>
+      </c>
+      <c r="E696" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F696" s="2" t="inlineStr"/>
+      <c r="G696" s="3" t="inlineStr">
+        <is>
+          <t>CCD clock driver design: slew rate, amplifier selection, gain networks and ringing.</t>
+        </is>
+      </c>
+      <c r="H696" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B697" s="3" t="inlineStr">
+        <is>
+          <t>Sliding Barn Door Gate</t>
+        </is>
+      </c>
+      <c r="C697" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D697" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-27_1607_Sliding-Barn-Door-Gate.md</t>
+        </is>
+      </c>
+      <c r="E697" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F697" s="2" t="inlineStr"/>
+      <c r="G697" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H697" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B698" s="3" t="inlineStr">
+        <is>
+          <t>Downsides of Liquid Membrane</t>
+        </is>
+      </c>
+      <c r="C698" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D698" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-28_1102_Downsides-of-Liquid-Membrane.md</t>
+        </is>
+      </c>
+      <c r="E698" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F698" s="2" t="inlineStr"/>
+      <c r="G698" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H698" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B699" s="3" t="inlineStr">
+        <is>
+          <t>Angle Calculation for Slope</t>
+        </is>
+      </c>
+      <c r="C699" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D699" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-28_1403_Angle-Calculation-for-Slope.md</t>
+        </is>
+      </c>
+      <c r="E699" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F699" s="2" t="inlineStr"/>
+      <c r="G699" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H699" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="B700" s="3" t="inlineStr">
+        <is>
+          <t>Wall Insulation Plan Review</t>
+        </is>
+      </c>
+      <c r="C700" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D700" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-28_1521_Wall-Insulation-Plan-Review.md</t>
+        </is>
+      </c>
+      <c r="E700" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F700" s="2" t="inlineStr"/>
+      <c r="G700" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H700" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B701" s="3" t="inlineStr">
+        <is>
+          <t>68pF Cap and Dip</t>
+        </is>
+      </c>
+      <c r="C701" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-006.json</t>
+        </is>
+      </c>
+      <c r="D701" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-31_1609_68pF-Cap-and-Dip.md</t>
+        </is>
+      </c>
+      <c r="E701" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F701" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G701" s="3" t="inlineStr">
+        <is>
+          <t>Electronics circuit design and bench debugging of an amplifier stage, possibly a professional engineering project.</t>
+        </is>
+      </c>
+      <c r="H701" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="B702" s="3" t="inlineStr">
+        <is>
+          <t>Screw Size Recommendation</t>
+        </is>
+      </c>
+      <c r="C702" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D702" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-31_1854_Screw-Size-Recommendation.md</t>
+        </is>
+      </c>
+      <c r="E702" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F702" s="2" t="inlineStr"/>
+      <c r="G702" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H702" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B703" s="3" t="inlineStr">
+        <is>
+          <t>Schematic Part Alignment Issue</t>
+        </is>
+      </c>
+      <c r="C703" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D703" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-02_0414_Schematic-Part-Alignment-Issue.md</t>
+        </is>
+      </c>
+      <c r="E703" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F703" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G703" s="3" t="inlineStr">
+        <is>
+          <t>Altium schematic issue, possibly part of professional electronics design work.</t>
+        </is>
+      </c>
+      <c r="H703" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B704" s="3" t="inlineStr">
+        <is>
+          <t>Altium Mouse Wheel Issue</t>
+        </is>
+      </c>
+      <c r="C704" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D704" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-02_0641_Altium-Mouse-Wheel-Issue.md</t>
+        </is>
+      </c>
+      <c r="E704" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F704" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G704" s="3" t="inlineStr">
+        <is>
+          <t>Altium software navigation issue, possibly part of professional electronics design work.</t>
+        </is>
+      </c>
+      <c r="H704" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B705" s="3" t="inlineStr">
+        <is>
+          <t>High slew-rate OP amps</t>
+        </is>
+      </c>
+      <c r="C705" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D705" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-02_1133_High-slew-rate-OP-amps.md</t>
+        </is>
+      </c>
+      <c r="E705" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F705" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G705" s="3" t="inlineStr">
+        <is>
+          <t>Component selection of high slew-rate op-amps, possibly for a professional electronics project.</t>
+        </is>
+      </c>
+      <c r="H705" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="B706" s="3" t="inlineStr">
+        <is>
+          <t>Active Low with -5V</t>
+        </is>
+      </c>
+      <c r="C706" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D706" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-02_1305_Active-Low-with-5V.md</t>
+        </is>
+      </c>
+      <c r="E706" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F706" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G706" s="3" t="inlineStr">
+        <is>
+          <t>Op-amp control pin logic levels for a circuit design, possibly a professional electronics project.</t>
+        </is>
+      </c>
+      <c r="H706" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B707" s="3" t="inlineStr">
+        <is>
+          <t>Reordering Rows in Excel</t>
+        </is>
+      </c>
+      <c r="C707" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D707" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-03_1352_Reordering-Rows-in-Excel.md</t>
+        </is>
+      </c>
+      <c r="E707" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F707" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G707" s="3" t="inlineStr">
+        <is>
+          <t>Excel row reordering, with reference to engineering tracker sheets possibly used at work.</t>
+        </is>
+      </c>
+      <c r="H707" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
+        </is>
+      </c>
+      <c r="B708" s="3" t="inlineStr">
+        <is>
+          <t>Lost Undo Button</t>
+        </is>
+      </c>
+      <c r="C708" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D708" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-03_1632_Lost-Undo-Button.md</t>
+        </is>
+      </c>
+      <c r="E708" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F708" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G708" s="3" t="inlineStr">
+        <is>
+          <t>PowerPoint toolbar issue, possibly related to work use of software.</t>
+        </is>
+      </c>
+      <c r="H708" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B709" s="3" t="inlineStr">
+        <is>
+          <t>Log Cabin Modification Advice</t>
+        </is>
+      </c>
+      <c r="C709" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D709" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04_1003_Log-Cabin-Modification-Advice.md</t>
+        </is>
+      </c>
+      <c r="E709" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F709" s="2" t="inlineStr"/>
+      <c r="G709" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H709" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="B710" s="3" t="inlineStr">
+        <is>
+          <t>Keter Store It Out Pro Dimensions</t>
+        </is>
+      </c>
+      <c r="C710" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D710" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04_1328_Keter-Store-It-Out-Pro-Dimensions.md</t>
+        </is>
+      </c>
+      <c r="E710" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F710" s="2" t="inlineStr"/>
+      <c r="G710" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H710" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B711" s="3" t="inlineStr">
+        <is>
+          <t>Tool not working intermittently</t>
+        </is>
+      </c>
+      <c r="C711" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D711" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-05_0825_Tool-not-working-intermittently.md</t>
+        </is>
+      </c>
+      <c r="E711" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F711" s="2" t="inlineStr"/>
+      <c r="G711" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H711" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B712" s="3" t="inlineStr">
+        <is>
+          <t>Mixing sand and cement</t>
+        </is>
+      </c>
+      <c r="C712" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D712" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-05_1723_Mixing-sand-and-cement.md</t>
+        </is>
+      </c>
+      <c r="E712" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F712" s="2" t="inlineStr"/>
+      <c r="G712" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H712" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B713" s="3" t="inlineStr">
+        <is>
+          <t>Excel cross-workbook reference</t>
+        </is>
+      </c>
+      <c r="C713" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D713" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06_0435_Excel-cross-workbook-reference.md</t>
+        </is>
+      </c>
+      <c r="E713" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F713" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G713" s="3" t="inlineStr">
+        <is>
+          <t>Excel cross-workbook references and dropdowns, possibly for a work spreadsheet.</t>
+        </is>
+      </c>
+      <c r="H713" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="B714" s="3" t="inlineStr">
+        <is>
+          <t>IC Footprint Pad Shape</t>
+        </is>
+      </c>
+      <c r="C714" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D714" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06_1020_IC-Footprint-Pad-Shape.md</t>
+        </is>
+      </c>
+      <c r="E714" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F714" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G714" s="3" t="inlineStr">
+        <is>
+          <t>PCB footprint pad shape question in Altium, possibly part of professional electronics design work.</t>
+        </is>
+      </c>
+      <c r="H714" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B715" s="3" t="inlineStr">
+        <is>
+          <t>PIP and Autism Support</t>
+        </is>
+      </c>
+      <c r="C715" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D715" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-13_1622_PIP-and-Autism-Support.md</t>
+        </is>
+      </c>
+      <c r="E715" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F715" s="2" t="inlineStr"/>
+      <c r="G715" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H715" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B716" s="3" t="inlineStr">
+        <is>
+          <t>Repeat syntax issue</t>
+        </is>
+      </c>
+      <c r="C716" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D716" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-14_0816_Repeat-syntax-issue.md</t>
+        </is>
+      </c>
+      <c r="E716" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F716" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G716" s="3" t="inlineStr">
+        <is>
+          <t>Troubleshooting Altium multi-channel schematic net naming, apparently for a professional electronics design project.</t>
+        </is>
+      </c>
+      <c r="H716" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B717" s="3" t="inlineStr">
+        <is>
+          <t>Ethernet connector temp rating</t>
+        </is>
+      </c>
+      <c r="C717" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D717" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17_0828_Ethernet-connector-temp-rating.md</t>
+        </is>
+      </c>
+      <c r="E717" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F717" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G717" s="3" t="inlineStr">
+        <is>
+          <t>Sourcing a high-temperature right-angle PCB-mount Ethernet connector, apparently for a professional engineering project.</t>
+        </is>
+      </c>
+      <c r="H717" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B718" s="3" t="inlineStr">
+        <is>
+          <t>Social Energy and Executive Function</t>
+        </is>
+      </c>
+      <c r="C718" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D718" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17_1450_Social-Energy-and-Executive-Function.md</t>
+        </is>
+      </c>
+      <c r="E718" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F718" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G718" s="3" t="inlineStr">
+        <is>
+          <t>Owner describes work as a source of energy demand and reserving limited functional capacity for work.</t>
+        </is>
+      </c>
+      <c r="H718" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B719" s="3" t="inlineStr">
+        <is>
+          <t>Reviving Rusty Drill Bits</t>
+        </is>
+      </c>
+      <c r="C719" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D719" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17_1610_Reviving-Rusty-Drill-Bits.md</t>
+        </is>
+      </c>
+      <c r="E719" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F719" s="2" t="inlineStr"/>
+      <c r="G719" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H719" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="B720" s="3" t="inlineStr">
+        <is>
+          <t>Lean-to Conservatory Roof Conversion</t>
+        </is>
+      </c>
+      <c r="C720" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D720" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-17_2129_Lean-to-Conservatory-Roof-Conversion.md</t>
+        </is>
+      </c>
+      <c r="E720" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F720" s="2" t="inlineStr"/>
+      <c r="G720" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H720" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H637"/>
+  <autoFilter ref="A1:H720"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24080,7 +27228,7 @@
         </is>
       </c>
       <c r="B1" t="n">
-        <v>636</v>
+        <v>719</v>
       </c>
     </row>
     <row r="2">
@@ -24090,7 +27238,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>154</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3">
@@ -24100,7 +27248,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>68</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4">
@@ -24110,7 +27258,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>222</v>
+        <v>276</v>
       </c>
     </row>
     <row r="5">
@@ -24120,7 +27268,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>414</v>
+        <v>443</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
chat-sift: all 98 batches read; final index.xlsx, extracts.docx and progress
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Aq7txTcfpUgzabiqqnXaKj
</commit_message>
<xml_diff>
--- a/chat-sift/output/index.xlsx
+++ b/chat-sift/output/index.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Counts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$720</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Index'!$A$1:$H$829</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H720"/>
+  <dimension ref="A1:H829"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27203,8 +27203,4060 @@
         <v>0</v>
       </c>
     </row>
+    <row r="721">
+      <c r="A721" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B721" s="3" t="inlineStr">
+        <is>
+          <t>AI Economy Financial Planning</t>
+        </is>
+      </c>
+      <c r="C721" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D721" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-18_0424_AI-Economy-Financial-Planning.md</t>
+        </is>
+      </c>
+      <c r="E721" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F721" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G721" s="3" t="inlineStr">
+        <is>
+          <t>Discusses career and income resilience under AI and the development of the owner's own men's wellbeing venture, including counselling training routes, pricing and a founding proposal.</t>
+        </is>
+      </c>
+      <c r="H721" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B722" s="3" t="inlineStr">
+        <is>
+          <t>Reviving Sofa for Room</t>
+        </is>
+      </c>
+      <c r="C722" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D722" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-18_1234_Reviving-Sofa-for-Room.md</t>
+        </is>
+      </c>
+      <c r="E722" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F722" s="2" t="inlineStr"/>
+      <c r="G722" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H722" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B723" s="3" t="inlineStr">
+        <is>
+          <t>Vacuum Motor Repair Project</t>
+        </is>
+      </c>
+      <c r="C723" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D723" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-18_1348_Vacuum-Motor-Repair-Project.md</t>
+        </is>
+      </c>
+      <c r="E723" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F723" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G723" s="3" t="inlineStr">
+        <is>
+          <t>Discusses an appliance repair as practice for the owner's planned electrical-fixes cabin venture.</t>
+        </is>
+      </c>
+      <c r="H723" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B724" s="3" t="inlineStr">
+        <is>
+          <t>Shark Carpet Cleaner Tips</t>
+        </is>
+      </c>
+      <c r="C724" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D724" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-18_1702_Shark-Carpet-Cleaner-Tips.md</t>
+        </is>
+      </c>
+      <c r="E724" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F724" s="2" t="inlineStr"/>
+      <c r="G724" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H724" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B725" s="3" t="inlineStr">
+        <is>
+          <t>Curved Monitors for Work</t>
+        </is>
+      </c>
+      <c r="C725" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D725" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-18_1953_Curved-Monitors-for-Work.md</t>
+        </is>
+      </c>
+      <c r="E725" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F725" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G725" s="3" t="inlineStr">
+        <is>
+          <t>Suitability of curved monitors for design and document work.</t>
+        </is>
+      </c>
+      <c r="H725" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B726" s="3" t="inlineStr">
+        <is>
+          <t>Folding golf trolley frame</t>
+        </is>
+      </c>
+      <c r="C726" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D726" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-19_1019_Folding-golf-trolley-frame.md</t>
+        </is>
+      </c>
+      <c r="E726" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F726" s="2" t="inlineStr"/>
+      <c r="G726" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H726" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B727" s="3" t="inlineStr">
+        <is>
+          <t>Overhang Stability Concerns</t>
+        </is>
+      </c>
+      <c r="C727" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D727" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-19_1255_Overhang-Stability-Concerns.md</t>
+        </is>
+      </c>
+      <c r="E727" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F727" s="2" t="inlineStr"/>
+      <c r="G727" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H727" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B728" s="3" t="inlineStr">
+        <is>
+          <t>Push to break switch</t>
+        </is>
+      </c>
+      <c r="C728" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D728" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20_0600_Push-to-break-switch.md</t>
+        </is>
+      </c>
+      <c r="E728" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F728" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G728" s="3" t="inlineStr">
+        <is>
+          <t>Electronics design work (switch selection, regulator and ADA4870 clock driver circuit review, calculation table), a slow work laptop, and getting started with the company's Altium Enterprise server.</t>
+        </is>
+      </c>
+      <c r="H728" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B729" s="3" t="inlineStr">
+        <is>
+          <t>Altium Logo Usage Rules</t>
+        </is>
+      </c>
+      <c r="C729" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D729" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20_1409_Altium-Logo-Usage-Rules.md</t>
+        </is>
+      </c>
+      <c r="E729" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F729" s="2" t="inlineStr"/>
+      <c r="G729" s="3" t="inlineStr">
+        <is>
+          <t>Engineering design review checklist: Altium logo use, review gate hover text and workbook image compression.</t>
+        </is>
+      </c>
+      <c r="H729" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B730" s="3" t="inlineStr">
+        <is>
+          <t>10-way version lookup</t>
+        </is>
+      </c>
+      <c r="C730" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D730" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20_2142_10-way-version-lookup.md</t>
+        </is>
+      </c>
+      <c r="E730" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F730" s="2" t="inlineStr"/>
+      <c r="G730" s="3" t="inlineStr">
+        <is>
+          <t>Component library consolidation, part equivalents and Altium library/footprint tasks.</t>
+        </is>
+      </c>
+      <c r="H730" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B731" s="3" t="inlineStr">
+        <is>
+          <t>Altium multi-channel error</t>
+        </is>
+      </c>
+      <c r="C731" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D731" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23_0656_Altium-multi-channel-error.md</t>
+        </is>
+      </c>
+      <c r="E731" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F731" s="2" t="inlineStr"/>
+      <c r="G731" s="3" t="inlineStr">
+        <is>
+          <t>Altium multi-channel hierarchy naming errors in a design.</t>
+        </is>
+      </c>
+      <c r="H731" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B732" s="3" t="inlineStr">
+        <is>
+          <t>Altium comment mismatch</t>
+        </is>
+      </c>
+      <c r="C732" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D732" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24_0023_Altium-comment-mismatch.md</t>
+        </is>
+      </c>
+      <c r="E732" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F732" s="2" t="inlineStr"/>
+      <c r="G732" s="3" t="inlineStr">
+        <is>
+          <t>Altium reuse block component matching, ECO and designator handling in a PCB design.</t>
+        </is>
+      </c>
+      <c r="H732" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24</t>
+        </is>
+      </c>
+      <c r="B733" s="3" t="inlineStr">
+        <is>
+          <t>Formatting Mac Drive HFS</t>
+        </is>
+      </c>
+      <c r="C733" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D733" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24_1329_Formatting-Mac-Drive-HFS.md</t>
+        </is>
+      </c>
+      <c r="E733" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F733" s="2" t="inlineStr"/>
+      <c r="G733" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H733" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B734" s="3" t="inlineStr">
+        <is>
+          <t>Painting Cabin Roof Panels</t>
+        </is>
+      </c>
+      <c r="C734" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D734" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-26_0812_Painting-Cabin-Roof-Panels.md</t>
+        </is>
+      </c>
+      <c r="E734" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F734" s="2" t="inlineStr"/>
+      <c r="G734" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H734" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B735" s="3" t="inlineStr">
+        <is>
+          <t>Wildkraut Energy Sniff Info</t>
+        </is>
+      </c>
+      <c r="C735" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D735" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27_1148_Wildkraut-Energy-Sniff-Info.md</t>
+        </is>
+      </c>
+      <c r="E735" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F735" s="2" t="inlineStr"/>
+      <c r="G735" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H735" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B736" s="3" t="inlineStr">
+        <is>
+          <t>Salary Increase Calculation</t>
+        </is>
+      </c>
+      <c r="C736" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D736" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27_1151_Salary-Increase-Calculation.md</t>
+        </is>
+      </c>
+      <c r="E736" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F736" s="2" t="inlineStr"/>
+      <c r="G736" s="3" t="inlineStr">
+        <is>
+          <t>Calculation of a salary increase in net and gross terms.</t>
+        </is>
+      </c>
+      <c r="H736" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B737" s="3" t="inlineStr">
+        <is>
+          <t>Sonos app discussion</t>
+        </is>
+      </c>
+      <c r="C737" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D737" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27_1253_Sonos-app-discussion.md</t>
+        </is>
+      </c>
+      <c r="E737" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F737" s="2" t="inlineStr"/>
+      <c r="G737" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H737" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B738" s="3" t="inlineStr">
+        <is>
+          <t>Mac Boot Disk Creation</t>
+        </is>
+      </c>
+      <c r="C738" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D738" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27_1450_Mac-Boot-Disk-Creation.md</t>
+        </is>
+      </c>
+      <c r="E738" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F738" s="2" t="inlineStr"/>
+      <c r="G738" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H738" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B739" s="3" t="inlineStr">
+        <is>
+          <t>ADHD Prescription Process Clarification</t>
+        </is>
+      </c>
+      <c r="C739" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D739" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30_0708_ADHD-Prescription-Process-Clarification.md</t>
+        </is>
+      </c>
+      <c r="E739" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F739" s="2" t="inlineStr"/>
+      <c r="G739" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H739" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B740" s="3" t="inlineStr">
+        <is>
+          <t>40-Core Cable Search</t>
+        </is>
+      </c>
+      <c r="C740" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D740" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30_0827_40-Core-Cable-Search.md</t>
+        </is>
+      </c>
+      <c r="E740" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F740" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G740" s="3" t="inlineStr">
+        <is>
+          <t>Sourcing a 40-core 16/0.2 cable and conductor sizing, apparently for engineering work.</t>
+        </is>
+      </c>
+      <c r="H740" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B741" s="3" t="inlineStr">
+        <is>
+          <t>IPC J-STD-001 and IPC-A-610 Compliance</t>
+        </is>
+      </c>
+      <c r="C741" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D741" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30_1359_IPC-J-STD-001-and-IPC-A-610-Compliance.md</t>
+        </is>
+      </c>
+      <c r="E741" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F741" s="2" t="inlineStr"/>
+      <c r="G741" s="3" t="inlineStr">
+        <is>
+          <t>Setting IPC J-STD-001 and IPC-A-610 requirements and ownership with a subcontract assembler.</t>
+        </is>
+      </c>
+      <c r="H741" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B742" s="3" t="inlineStr">
+        <is>
+          <t>Intel i7 Ultra vPro Explained</t>
+        </is>
+      </c>
+      <c r="C742" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D742" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30_2109_Intel-i7-Ultra-vPro-Explained.md</t>
+        </is>
+      </c>
+      <c r="E742" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F742" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G742" s="3" t="inlineStr">
+        <is>
+          <t>Laptop processor specifications possibly for a work/design laptop.</t>
+        </is>
+      </c>
+      <c r="H742" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B743" s="3" t="inlineStr">
+        <is>
+          <t>Altium Enterprise User Guide</t>
+        </is>
+      </c>
+      <c r="C743" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D743" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30_2244_Altium-Enterprise-User-Guide.md</t>
+        </is>
+      </c>
+      <c r="E743" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F743" s="2" t="inlineStr"/>
+      <c r="G743" s="3" t="inlineStr">
+        <is>
+          <t>Locating an earlier chat about the work Altium Enterprise server and user guidance.</t>
+        </is>
+      </c>
+      <c r="H743" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B744" s="3" t="inlineStr">
+        <is>
+          <t>Altium Enterprise Guide</t>
+        </is>
+      </c>
+      <c r="C744" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D744" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30_2245_Altium-Enterprise-Guide.md</t>
+        </is>
+      </c>
+      <c r="E744" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F744" s="2" t="inlineStr"/>
+      <c r="G744" s="3" t="inlineStr">
+        <is>
+          <t>Capability manual and rollout plan for the company's on-premise Altium Enterprise Server.</t>
+        </is>
+      </c>
+      <c r="H744" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B745" s="3" t="inlineStr">
+        <is>
+          <t>Altium user manual chat</t>
+        </is>
+      </c>
+      <c r="C745" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D745" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30_2306_Altium-user-manual-chat.md</t>
+        </is>
+      </c>
+      <c r="E745" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F745" s="2" t="inlineStr"/>
+      <c r="G745" s="3" t="inlineStr">
+        <is>
+          <t>Locating earlier chats about the work Altium Enterprise setup.</t>
+        </is>
+      </c>
+      <c r="H745" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B746" s="3" t="inlineStr">
+        <is>
+          <t>Coach bolt pilot size</t>
+        </is>
+      </c>
+      <c r="C746" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D746" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-03_1348_Coach-bolt-pilot-size.md</t>
+        </is>
+      </c>
+      <c r="E746" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F746" s="2" t="inlineStr"/>
+      <c r="G746" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H746" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B747" s="3" t="inlineStr">
+        <is>
+          <t>Anti-lift Adhesive Tips</t>
+        </is>
+      </c>
+      <c r="C747" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D747" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-03_2105_Anti-lift-Adhesive-Tips.md</t>
+        </is>
+      </c>
+      <c r="E747" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F747" s="2" t="inlineStr"/>
+      <c r="G747" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H747" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B748" s="3" t="inlineStr">
+        <is>
+          <t>Counselling Course Application Help</t>
+        </is>
+      </c>
+      <c r="C748" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D748" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-05_2038_Counselling-Course-Application-Help.md</t>
+        </is>
+      </c>
+      <c r="E748" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F748" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G748" s="3" t="inlineStr">
+        <is>
+          <t>Application for a counselling course, with reference to the owner's technical career.</t>
+        </is>
+      </c>
+      <c r="H748" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="B749" s="3" t="inlineStr">
+        <is>
+          <t>Power Supply Compliance Query</t>
+        </is>
+      </c>
+      <c r="C749" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D749" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-12_2127_Power-Supply-Compliance-Query.md</t>
+        </is>
+      </c>
+      <c r="E749" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F749" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G749" s="3" t="inlineStr">
+        <is>
+          <t>Discussion of a chief engineer's objection to supplying a commercial PSU in a rack, signalling choices, and PXI data-capture hardware for a work system.</t>
+        </is>
+      </c>
+      <c r="H749" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B750" s="3" t="inlineStr">
+        <is>
+          <t>Communication Competency Appraisal</t>
+        </is>
+      </c>
+      <c r="C750" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D750" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13_0613_Communication-Competency-Appraisal.md</t>
+        </is>
+      </c>
+      <c r="E750" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F750" s="2" t="inlineStr"/>
+      <c r="G750" s="3" t="inlineStr">
+        <is>
+          <t>Drafting a response to the communication competency rating in the owner's appraisal.</t>
+        </is>
+      </c>
+      <c r="H750" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B751" s="3" t="inlineStr">
+        <is>
+          <t>Temperature Sensor Cable Length</t>
+        </is>
+      </c>
+      <c r="C751" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D751" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13_0726_Temperature-Sensor-Cable-Length.md</t>
+        </is>
+      </c>
+      <c r="E751" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F751" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G751" s="3" t="inlineStr">
+        <is>
+          <t>Technical question on measuring a temperature sensor over a long cable with a Lake Shore instrument.</t>
+        </is>
+      </c>
+      <c r="H751" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B752" s="3" t="inlineStr">
+        <is>
+          <t>Far Out Radiohead Songs</t>
+        </is>
+      </c>
+      <c r="C752" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D752" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13_1249_Far-Out-Radiohead-Songs.md</t>
+        </is>
+      </c>
+      <c r="E752" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F752" s="2" t="inlineStr"/>
+      <c r="G752" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H752" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B753" s="3" t="inlineStr">
+        <is>
+          <t>Resistor Tolerance Limits</t>
+        </is>
+      </c>
+      <c r="C753" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D753" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13_1653_Resistor-Tolerance-Limits.md</t>
+        </is>
+      </c>
+      <c r="E753" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F753" s="2" t="inlineStr"/>
+      <c r="G753" s="3" t="inlineStr">
+        <is>
+          <t>Tolerance calculations and statistical comparison of manual versus automated test measurement data.</t>
+        </is>
+      </c>
+      <c r="H753" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B754" s="3" t="inlineStr">
+        <is>
+          <t>Green Dot in Altium 365</t>
+        </is>
+      </c>
+      <c r="C754" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D754" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13_1756_Green-Dot-in-Altium-365.md</t>
+        </is>
+      </c>
+      <c r="E754" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F754" s="2" t="inlineStr"/>
+      <c r="G754" s="3" t="inlineStr">
+        <is>
+          <t>Question about Altium 365 presence indicators shown for former colleagues.</t>
+        </is>
+      </c>
+      <c r="H754" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B755" s="3" t="inlineStr">
+        <is>
+          <t>Gamma vs Neutron Testing</t>
+        </is>
+      </c>
+      <c r="C755" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D755" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13_2011_Gamma-vs-Neutron-Testing.md</t>
+        </is>
+      </c>
+      <c r="E755" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F755" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G755" s="3" t="inlineStr">
+        <is>
+          <t>Technical discussion of gamma, X-ray, neutron and heavy-ion radiation testing of electronics and test conditions.</t>
+        </is>
+      </c>
+      <c r="H755" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B756" s="3" t="inlineStr">
+        <is>
+          <t>IEC 61010 Compliance Justification</t>
+        </is>
+      </c>
+      <c r="C756" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D756" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14_0035_IEC-61010-Compliance-Justification.md</t>
+        </is>
+      </c>
+      <c r="E756" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F756" s="2" t="inlineStr"/>
+      <c r="G756" s="3" t="inlineStr">
+        <is>
+          <t>Drafting IEC 61010 and regulatory compliance wording for a work document and a customer email.</t>
+        </is>
+      </c>
+      <c r="H756" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B757" s="3" t="inlineStr">
+        <is>
+          <t>Clarification Request</t>
+        </is>
+      </c>
+      <c r="C757" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D757" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14_1439_Clarification-Request.md</t>
+        </is>
+      </c>
+      <c r="E757" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F757" s="2" t="inlineStr"/>
+      <c r="G757" s="3" t="inlineStr">
+        <is>
+          <t>Shielding and LVDS/fibre-optic signal transmission options for radiation testing of electronic sensors.</t>
+        </is>
+      </c>
+      <c r="H757" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B758" s="3" t="inlineStr">
+        <is>
+          <t>Radiation Effects on Fibres</t>
+        </is>
+      </c>
+      <c r="C758" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D758" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14_1543_Radiation-Effects-on-Fibres.md</t>
+        </is>
+      </c>
+      <c r="E758" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F758" s="2" t="inlineStr"/>
+      <c r="G758" s="3" t="inlineStr">
+        <is>
+          <t>Selection of radiation-tolerant optical transmitters and power options for a radiation test campaign.</t>
+        </is>
+      </c>
+      <c r="H758" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B759" s="3" t="inlineStr">
+        <is>
+          <t>Oxide Controllers Benefits</t>
+        </is>
+      </c>
+      <c r="C759" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D759" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14_1726_Oxide-Controllers-Benefits.md</t>
+        </is>
+      </c>
+      <c r="E759" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F759" s="2" t="inlineStr"/>
+      <c r="G759" s="3" t="inlineStr">
+        <is>
+          <t>Benefits of PXI embedded controllers relative to cost.</t>
+        </is>
+      </c>
+      <c r="H759" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B760" s="3" t="inlineStr">
+        <is>
+          <t>PXI Embedded Controllers Benefits</t>
+        </is>
+      </c>
+      <c r="C760" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D760" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14_1727_PXI-Embedded-Controllers-Benefits.md</t>
+        </is>
+      </c>
+      <c r="E760" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F760" s="2" t="inlineStr"/>
+      <c r="G760" s="3" t="inlineStr">
+        <is>
+          <t>Engineering design discussion for a radiation test system project: PXI controller selection, data logging and storage architecture, firmware fault handling, current sensing and state machine documentation.</t>
+        </is>
+      </c>
+      <c r="H760" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B761" s="3" t="inlineStr">
+        <is>
+          <t>Best Mouse for AI Work</t>
+        </is>
+      </c>
+      <c r="C761" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D761" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14_2103_Best-Mouse-for-AI-Work.md</t>
+        </is>
+      </c>
+      <c r="E761" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F761" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G761" s="3" t="inlineStr">
+        <is>
+          <t>Choice of mouse for AI and engineering work tasks.</t>
+        </is>
+      </c>
+      <c r="H761" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B762" s="3" t="inlineStr">
+        <is>
+          <t>HR Cliques and Dysfunction</t>
+        </is>
+      </c>
+      <c r="C762" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D762" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14_2259_HR-Cliques-and-Dysfunction.md</t>
+        </is>
+      </c>
+      <c r="E762" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F762" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G762" s="3" t="inlineStr">
+        <is>
+          <t>Workplace HR conduct, an employee's resignation after a performance investigation, the owner's appraisal rating during ill health, and changed relations with colleagues.</t>
+        </is>
+      </c>
+      <c r="H762" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B763" s="3" t="inlineStr">
+        <is>
+          <t>PXI 4-Wire Sense Options</t>
+        </is>
+      </c>
+      <c r="C763" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D763" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15_0430_PXI-4-Wire-Sense-Options.md</t>
+        </is>
+      </c>
+      <c r="E763" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F763" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G763" s="3" t="inlineStr">
+        <is>
+          <t>Instrumentation selection, refurbished equipment procurement and IEC 61010 compliance for a sellable rack system used in radiation testing.</t>
+        </is>
+      </c>
+      <c r="H763" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B764" s="3" t="inlineStr">
+        <is>
+          <t>Triz Connector Pinout Configuration</t>
+        </is>
+      </c>
+      <c r="C764" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D764" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15_0613_Triz-Connector-Pinout-Configuration.md</t>
+        </is>
+      </c>
+      <c r="E764" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F764" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G764" s="3" t="inlineStr">
+        <is>
+          <t>Connector, cable and signalling design for clocks, bias rails and LVDS links into a radiation test area.</t>
+        </is>
+      </c>
+      <c r="H764" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B765" s="3" t="inlineStr">
+        <is>
+          <t>Keysight 61010 Compliance Evidence</t>
+        </is>
+      </c>
+      <c r="C765" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D765" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15_0812_Keysight-61010-Compliance-Evidence.md</t>
+        </is>
+      </c>
+      <c r="E765" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F765" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G765" s="3" t="inlineStr">
+        <is>
+          <t>Finding IEC 61010 compliance evidence for chassis and power supply mainframe for a technical file.</t>
+        </is>
+      </c>
+      <c r="H765" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B766" s="3" t="inlineStr">
+        <is>
+          <t>Harwell Radiation Facility Info</t>
+        </is>
+      </c>
+      <c r="C766" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D766" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15_0818_Harwell-Radiation-Facility-Info.md</t>
+        </is>
+      </c>
+      <c r="E766" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F766" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G766" s="3" t="inlineStr">
+        <is>
+          <t>Radiation test facility capabilities and a test plan for irradiating an imaging sensor.</t>
+        </is>
+      </c>
+      <c r="H766" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B767" s="3" t="inlineStr">
+        <is>
+          <t>Rack Layout Design Tips</t>
+        </is>
+      </c>
+      <c r="C767" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D767" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15_0937_Rack-Layout-Design-Tips.md</t>
+        </is>
+      </c>
+      <c r="E767" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F767" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G767" s="3" t="inlineStr">
+        <is>
+          <t>Layout and airflow design of an instrumentation rack containing customer electronics and PXI.</t>
+        </is>
+      </c>
+      <c r="H767" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B768" s="3" t="inlineStr">
+        <is>
+          <t>Escort Ad Sites Alternatives</t>
+        </is>
+      </c>
+      <c r="C768" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D768" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15_1906_Escort-Ad-Sites-Alternatives.md</t>
+        </is>
+      </c>
+      <c r="E768" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F768" s="2" t="inlineStr"/>
+      <c r="G768" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H768" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B769" s="3" t="inlineStr">
+        <is>
+          <t>Mermaid Diagram in Draw.io</t>
+        </is>
+      </c>
+      <c r="C769" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D769" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16_1906_Mermaid-Diagram-in-Draw-io.md</t>
+        </is>
+      </c>
+      <c r="E769" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F769" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G769" s="3" t="inlineStr">
+        <is>
+          <t>Diagramming an irradiation test system state machine for design review using Mermaid, Visio and Excel.</t>
+        </is>
+      </c>
+      <c r="H769" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B770" s="3" t="inlineStr">
+        <is>
+          <t>Sensor Current Monitoring</t>
+        </is>
+      </c>
+      <c r="C770" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D770" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20_1549_Sensor-Current-Monitoring.md</t>
+        </is>
+      </c>
+      <c r="E770" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F770" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G770" s="3" t="inlineStr">
+        <is>
+          <t>Current monitoring ranges and gain for sensor supply rails during heavy ion testing.</t>
+        </is>
+      </c>
+      <c r="H770" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B771" s="3" t="inlineStr">
+        <is>
+          <t>Certification Comparison 61010 FCC</t>
+        </is>
+      </c>
+      <c r="C771" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D771" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20_1726_Certification-Comparison-61010-FCC.md</t>
+        </is>
+      </c>
+      <c r="E771" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F771" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G771" s="3" t="inlineStr">
+        <is>
+          <t>Comparison of IEC 61010 and FCC certification routes for selling lab electronics to US customers.</t>
+        </is>
+      </c>
+      <c r="H771" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B772" s="3" t="inlineStr">
+        <is>
+          <t>Xilinx KX7 RS232 Ports</t>
+        </is>
+      </c>
+      <c r="C772" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D772" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21_1554_Xilinx-KX7-RS232-Ports.md</t>
+        </is>
+      </c>
+      <c r="E772" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F772" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G772" s="3" t="inlineStr">
+        <is>
+          <t>Technical question on the number of RS-232 ports supported by a Kintex-7 FPGA card.</t>
+        </is>
+      </c>
+      <c r="H772" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B773" s="3" t="inlineStr">
+        <is>
+          <t>Concrete screw drill size</t>
+        </is>
+      </c>
+      <c r="C773" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D773" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-23_1047_Concrete-screw-drill-size.md</t>
+        </is>
+      </c>
+      <c r="E773" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F773" s="2" t="inlineStr"/>
+      <c r="G773" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H773" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="B774" s="3" t="inlineStr">
+        <is>
+          <t>MS Polymer vs Silicone</t>
+        </is>
+      </c>
+      <c r="C774" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D774" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-23_1230_MS-Polymer-vs-Silicone.md</t>
+        </is>
+      </c>
+      <c r="E774" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F774" s="2" t="inlineStr"/>
+      <c r="G774" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H774" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B775" s="3" t="inlineStr">
+        <is>
+          <t>Window Module Installation Advice</t>
+        </is>
+      </c>
+      <c r="C775" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D775" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24_1105_Window-Module-Installation-Advice.md</t>
+        </is>
+      </c>
+      <c r="E775" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F775" s="2" t="inlineStr"/>
+      <c r="G775" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H775" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B776" s="3" t="inlineStr">
+        <is>
+          <t>Mirrored Configuration Request</t>
+        </is>
+      </c>
+      <c r="C776" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D776" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24_1139_Mirrored-Configuration-Request.md</t>
+        </is>
+      </c>
+      <c r="E776" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F776" s="2" t="inlineStr"/>
+      <c r="G776" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H776" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B777" s="3" t="inlineStr">
+        <is>
+          <t>Remove wood from glass</t>
+        </is>
+      </c>
+      <c r="C777" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D777" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24_1150_Remove-wood-from-glass.md</t>
+        </is>
+      </c>
+      <c r="E777" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F777" s="2" t="inlineStr"/>
+      <c r="G777" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H777" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B778" s="3" t="inlineStr">
+        <is>
+          <t>Sage Cleaning Cycle Steps</t>
+        </is>
+      </c>
+      <c r="C778" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D778" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-24_1303_Sage-Cleaning-Cycle-Steps.md</t>
+        </is>
+      </c>
+      <c r="E778" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F778" s="2" t="inlineStr"/>
+      <c r="G778" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H778" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B779" s="3" t="inlineStr">
+        <is>
+          <t>Carb Fuel Line Explanation</t>
+        </is>
+      </c>
+      <c r="C779" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D779" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-25_0543_Carb-Fuel-Line-Explanation.md</t>
+        </is>
+      </c>
+      <c r="E779" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F779" s="2" t="inlineStr"/>
+      <c r="G779" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H779" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="B780" s="3" t="inlineStr">
+        <is>
+          <t>Clarification Request</t>
+        </is>
+      </c>
+      <c r="C780" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D780" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26_1459_Clarification-Request.md</t>
+        </is>
+      </c>
+      <c r="E780" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F780" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G780" s="3" t="inlineStr">
+        <is>
+          <t>Income protection and redundancy cover in relation to the owner's employment and length of service.</t>
+        </is>
+      </c>
+      <c r="H780" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B781" s="3" t="inlineStr">
+        <is>
+          <t>Log cabin work summary</t>
+        </is>
+      </c>
+      <c r="C781" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D781" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28_1009_Log-cabin-work-summary.md</t>
+        </is>
+      </c>
+      <c r="E781" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F781" s="2" t="inlineStr"/>
+      <c r="G781" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H781" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B782" s="3" t="inlineStr">
+        <is>
+          <t>Plumbing Crash Courses</t>
+        </is>
+      </c>
+      <c r="C782" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D782" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28_1739_Plumbing-Crash-Courses.md</t>
+        </is>
+      </c>
+      <c r="E782" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F782" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G782" s="3" t="inlineStr">
+        <is>
+          <t>Enquiry about fast-track training routes to retrain as a plumber (possible career change).</t>
+        </is>
+      </c>
+      <c r="H782" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B783" s="3" t="inlineStr">
+        <is>
+          <t>Gym Contract Dispute</t>
+        </is>
+      </c>
+      <c r="C783" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D783" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30_2029_Gym-Contract-Dispute.md</t>
+        </is>
+      </c>
+      <c r="E783" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F783" s="2" t="inlineStr"/>
+      <c r="G783" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H783" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B784" s="3" t="inlineStr">
+        <is>
+          <t>Saab 9-5 Idle Issue</t>
+        </is>
+      </c>
+      <c r="C784" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D784" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31_1250_Saab-9-5-Idle-Issue.md</t>
+        </is>
+      </c>
+      <c r="E784" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F784" s="2" t="inlineStr"/>
+      <c r="G784" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H784" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B785" s="3" t="inlineStr">
+        <is>
+          <t>19" Rack Controllers</t>
+        </is>
+      </c>
+      <c r="C785" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D785" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02_0822_19-Rack-Controllers.md</t>
+        </is>
+      </c>
+      <c r="E785" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F785" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G785" s="3" t="inlineStr">
+        <is>
+          <t>Technical enquiry about 19-inch rack-format controllers for a test-equipment rack, apparently for professional engineering work.</t>
+        </is>
+      </c>
+      <c r="H785" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B786" s="3" t="inlineStr">
+        <is>
+          <t>Telephone wire vs twisted pair</t>
+        </is>
+      </c>
+      <c r="C786" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D786" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04_1055_Telephone-wire-vs-twisted-pair.md</t>
+        </is>
+      </c>
+      <c r="E786" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F786" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G786" s="3" t="inlineStr">
+        <is>
+          <t>Technical question on using telephone wire as differential signal cable, possibly for professional engineering work.</t>
+        </is>
+      </c>
+      <c r="H786" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B787" s="3" t="inlineStr">
+        <is>
+          <t>Obesity and Alcoholism as Diseases</t>
+        </is>
+      </c>
+      <c r="C787" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D787" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08_1711_Obesity-and-Alcoholism-as-Diseases.md</t>
+        </is>
+      </c>
+      <c r="E787" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F787" s="2" t="inlineStr"/>
+      <c r="G787" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H787" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B788" s="3" t="inlineStr">
+        <is>
+          <t>AGI/ASI and Money Value</t>
+        </is>
+      </c>
+      <c r="C788" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D788" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08_1915_AGI-ASI-and-Money-Value.md</t>
+        </is>
+      </c>
+      <c r="E788" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F788" s="2" t="inlineStr"/>
+      <c r="G788" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H788" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B789" s="3" t="inlineStr">
+        <is>
+          <t>LVDS Twisted Ribbon Shielding</t>
+        </is>
+      </c>
+      <c r="C789" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D789" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09_1240_LVDS-Twisted-Ribbon-Shielding.md</t>
+        </is>
+      </c>
+      <c r="E789" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F789" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G789" s="3" t="inlineStr">
+        <is>
+          <t>Technical discussion of a 25 m LVDS cable prototype test, apparently for a professional engineering project.</t>
+        </is>
+      </c>
+      <c r="H789" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B790" s="3" t="inlineStr">
+        <is>
+          <t>SMBJ15A Transient Protection</t>
+        </is>
+      </c>
+      <c r="C790" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D790" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09_1603_SMBJ15A-Transient-Protection.md</t>
+        </is>
+      </c>
+      <c r="E790" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F790" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G790" s="3" t="inlineStr">
+        <is>
+          <t>Fault-finding repeated capacitor failures on a 15 V rail board in an established system, apparently professional engineering work.</t>
+        </is>
+      </c>
+      <c r="H790" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B791" s="3" t="inlineStr">
+        <is>
+          <t>Vinted Fraud Scheme Inquiry</t>
+        </is>
+      </c>
+      <c r="C791" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D791" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11_1809_Vinted-Fraud-Scheme-Inquiry.md</t>
+        </is>
+      </c>
+      <c r="E791" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F791" s="2" t="inlineStr"/>
+      <c r="G791" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H791" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B792" s="3" t="inlineStr">
+        <is>
+          <t>Cocaine Ingestion Effects</t>
+        </is>
+      </c>
+      <c r="C792" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D792" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12_1124_Cocaine-Ingestion-Effects.md</t>
+        </is>
+      </c>
+      <c r="E792" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F792" s="2" t="inlineStr"/>
+      <c r="G792" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H792" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B793" s="3" t="inlineStr">
+        <is>
+          <t>Saab 9-5 ABS Issue</t>
+        </is>
+      </c>
+      <c r="C793" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D793" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12_1515_Saab-9-5-ABS-Issue.md</t>
+        </is>
+      </c>
+      <c r="E793" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F793" s="2" t="inlineStr"/>
+      <c r="G793" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H793" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B794" s="3" t="inlineStr">
+        <is>
+          <t>Wet kiln sand fix</t>
+        </is>
+      </c>
+      <c r="C794" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D794" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12_2105_Wet-kiln-sand-fix.md</t>
+        </is>
+      </c>
+      <c r="E794" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F794" s="2" t="inlineStr"/>
+      <c r="G794" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H794" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B795" s="3" t="inlineStr">
+        <is>
+          <t>Hinge Profile Setup Tips</t>
+        </is>
+      </c>
+      <c r="C795" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D795" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12_2303_Hinge-Profile-Setup-Tips.md</t>
+        </is>
+      </c>
+      <c r="E795" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="F795" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G795" s="3" t="inlineStr">
+        <is>
+          <t>Brief discussion of how to describe job title and workplace.</t>
+        </is>
+      </c>
+      <c r="H795" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B796" s="3" t="inlineStr">
+        <is>
+          <t>Joining Tyvek Super Pro</t>
+        </is>
+      </c>
+      <c r="C796" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D796" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-13_1751_Joining-Tyvek-Super-Pro.md</t>
+        </is>
+      </c>
+      <c r="E796" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F796" s="2" t="inlineStr"/>
+      <c r="G796" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H796" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B797" s="3" t="inlineStr">
+        <is>
+          <t>David Byrne 2026 Tour</t>
+        </is>
+      </c>
+      <c r="C797" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D797" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-13_2107_David-Byrne-2026-Tour.md</t>
+        </is>
+      </c>
+      <c r="E797" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F797" s="2" t="inlineStr"/>
+      <c r="G797" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H797" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B798" s="3" t="inlineStr">
+        <is>
+          <t>Infrared Heating Panels Benefits</t>
+        </is>
+      </c>
+      <c r="C798" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D798" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14_0907_Infrared-Heating-Panels-Benefits.md</t>
+        </is>
+      </c>
+      <c r="E798" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F798" s="2" t="inlineStr"/>
+      <c r="G798" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H798" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B799" s="3" t="inlineStr">
+        <is>
+          <t>Swollen Eyelid Diagnosis</t>
+        </is>
+      </c>
+      <c r="C799" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D799" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14_0916_Swollen-Eyelid-Diagnosis.md</t>
+        </is>
+      </c>
+      <c r="E799" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F799" s="2" t="inlineStr"/>
+      <c r="G799" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H799" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B800" s="3" t="inlineStr">
+        <is>
+          <t>Hole drill assembly guide</t>
+        </is>
+      </c>
+      <c r="C800" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D800" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14_1600_Hole-drill-assembly-guide.md</t>
+        </is>
+      </c>
+      <c r="E800" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F800" s="2" t="inlineStr"/>
+      <c r="G800" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H800" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B801" s="3" t="inlineStr">
+        <is>
+          <t>Insurance after drug driving</t>
+        </is>
+      </c>
+      <c r="C801" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-007.json</t>
+        </is>
+      </c>
+      <c r="D801" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15_1357_Insurance-after-drug-driving.md</t>
+        </is>
+      </c>
+      <c r="E801" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F801" s="2" t="inlineStr"/>
+      <c r="G801" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H801" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B802" s="3" t="inlineStr">
+        <is>
+          <t>Duck tape on cement board</t>
+        </is>
+      </c>
+      <c r="C802" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D802" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15_1717_Duck-tape-on-cement-board.md</t>
+        </is>
+      </c>
+      <c r="E802" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F802" s="2" t="inlineStr"/>
+      <c r="G802" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H802" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B803" s="3" t="inlineStr">
+        <is>
+          <t>IKOpro Stickall Use</t>
+        </is>
+      </c>
+      <c r="C803" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D803" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15_2200_IKOpro-Stickall-Use.md</t>
+        </is>
+      </c>
+      <c r="E803" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F803" s="2" t="inlineStr"/>
+      <c r="G803" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H803" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B804" s="3" t="inlineStr">
+        <is>
+          <t>Stage 1 Tuning Plan</t>
+        </is>
+      </c>
+      <c r="C804" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D804" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16_1524_Stage-1-Tuning-Plan.md</t>
+        </is>
+      </c>
+      <c r="E804" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F804" s="2" t="inlineStr"/>
+      <c r="G804" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H804" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B805" s="3" t="inlineStr">
+        <is>
+          <t>Mattress Stain Removal Advice</t>
+        </is>
+      </c>
+      <c r="C805" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D805" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19_1018_Mattress-Stain-Removal-Advice.md</t>
+        </is>
+      </c>
+      <c r="E805" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F805" s="2" t="inlineStr"/>
+      <c r="G805" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H805" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B806" s="3" t="inlineStr">
+        <is>
+          <t>Learning Windows Speech Prompts</t>
+        </is>
+      </c>
+      <c r="C806" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D806" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19_1324_Learning-Windows-Speech-Prompts.md</t>
+        </is>
+      </c>
+      <c r="E806" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F806" s="2" t="inlineStr"/>
+      <c r="G806" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H806" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B807" s="3" t="inlineStr">
+        <is>
+          <t>Tyvek Branding Orientation</t>
+        </is>
+      </c>
+      <c r="C807" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D807" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20_1146_Tyvek-Branding-Orientation.md</t>
+        </is>
+      </c>
+      <c r="E807" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F807" s="2" t="inlineStr"/>
+      <c r="G807" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H807" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B808" s="3" t="inlineStr">
+        <is>
+          <t>Membrane Securing Advice</t>
+        </is>
+      </c>
+      <c r="C808" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D808" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21_1354_Membrane-Securing-Advice.md</t>
+        </is>
+      </c>
+      <c r="E808" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F808" s="2" t="inlineStr"/>
+      <c r="G808" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H808" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B809" s="3" t="inlineStr">
+        <is>
+          <t>DPM Sand Topcoat Tips</t>
+        </is>
+      </c>
+      <c r="C809" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D809" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22_1139_DPM-Sand-Topcoat-Tips.md</t>
+        </is>
+      </c>
+      <c r="E809" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F809" s="2" t="inlineStr"/>
+      <c r="G809" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H809" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B810" s="3" t="inlineStr">
+        <is>
+          <t>Radiation Suited Cables</t>
+        </is>
+      </c>
+      <c r="C810" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D810" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22_1703_Radiation-Suited-Cables.md</t>
+        </is>
+      </c>
+      <c r="E810" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F810" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G810" s="3" t="inlineStr">
+        <is>
+          <t>Looking up earlier findings on radiation-tolerant Ethernet and LVDS cabling, apparently for professional engineering work.</t>
+        </is>
+      </c>
+      <c r="H810" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B811" s="3" t="inlineStr">
+        <is>
+          <t>Voltage at Load Current at Source</t>
+        </is>
+      </c>
+      <c r="C811" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D811" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23_1546_Voltage-at-Load-Current-at-Source.md</t>
+        </is>
+      </c>
+      <c r="E811" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F811" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G811" s="3" t="inlineStr">
+        <is>
+          <t>Technical question on measuring voltage at the load and current at the source under system constraints, likely for test-system work.</t>
+        </is>
+      </c>
+      <c r="H811" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B812" s="3" t="inlineStr">
+        <is>
+          <t>External Trigger for Timestamps</t>
+        </is>
+      </c>
+      <c r="C812" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D812" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23_1758_External-Trigger-for-Timestamps.md</t>
+        </is>
+      </c>
+      <c r="E812" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F812" s="2" t="inlineStr"/>
+      <c r="G812" s="3" t="inlineStr">
+        <is>
+          <t>Design discussion and one-page proposal for sub-second timestamping and metadata improvements on a PXI/FPGA radiation test system.</t>
+        </is>
+      </c>
+      <c r="H812" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B813" s="3" t="inlineStr">
+        <is>
+          <t>Radiation System State Machine</t>
+        </is>
+      </c>
+      <c r="C813" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D813" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23_1955_Radiation-System-State-Machine.md</t>
+        </is>
+      </c>
+      <c r="E813" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F813" s="2" t="inlineStr"/>
+      <c r="G813" s="3" t="inlineStr">
+        <is>
+          <t>Radiation test rig architecture: state-machine synopsis, timestamping subsystem development, physical block diagrams, PXI-6683H timing and circular-buffer event capture.</t>
+        </is>
+      </c>
+      <c r="H813" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B814" s="3" t="inlineStr">
+        <is>
+          <t>Radiation Effects on Sensors</t>
+        </is>
+      </c>
+      <c r="C814" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D814" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25_1128_Radiation-Effects-on-Sensors.md</t>
+        </is>
+      </c>
+      <c r="E814" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F814" s="2" t="inlineStr"/>
+      <c r="G814" s="3" t="inlineStr">
+        <is>
+          <t>Justifying a requirement for supply monitoring during radiation testing of sensors, responding to a colleague's query, and voltage/current measurement bandwidth.</t>
+        </is>
+      </c>
+      <c r="H814" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B815" s="3" t="inlineStr">
+        <is>
+          <t>Op-amp Circuit Schematic</t>
+        </is>
+      </c>
+      <c r="C815" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D815" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25_1528_Op-amp-Circuit-Schematic.md</t>
+        </is>
+      </c>
+      <c r="E815" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F815" s="2" t="inlineStr"/>
+      <c r="G815" s="3" t="inlineStr">
+        <is>
+          <t>Clock-driver amplifier chain slew-rate analysis and report section on meeting an adjustable slew requirement (REQ-ELE-007).</t>
+        </is>
+      </c>
+      <c r="H815" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B816" s="3" t="inlineStr">
+        <is>
+          <t>Multiplying factor calculation</t>
+        </is>
+      </c>
+      <c r="C816" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D816" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26_0637_Multiplying-factor-calculation.md</t>
+        </is>
+      </c>
+      <c r="E816" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F816" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G816" s="3" t="inlineStr">
+        <is>
+          <t>Frequency ratio calculation between 50 kHz and 250 MHz, likely relating to measurement bandwidths in test work.</t>
+        </is>
+      </c>
+      <c r="H816" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B817" s="3" t="inlineStr">
+        <is>
+          <t>Dyson V11 Cuts Out</t>
+        </is>
+      </c>
+      <c r="C817" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D817" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28_0824_Dyson-V11-Cuts-Out.md</t>
+        </is>
+      </c>
+      <c r="E817" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F817" s="2" t="inlineStr"/>
+      <c r="G817" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H817" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B818" s="3" t="inlineStr">
+        <is>
+          <t>Rise time measurement tweak</t>
+        </is>
+      </c>
+      <c r="C818" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D818" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29_1135_Rise-time-measurement-tweak.md</t>
+        </is>
+      </c>
+      <c r="E818" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F818" s="2" t="inlineStr"/>
+      <c r="G818" s="3" t="inlineStr">
+        <is>
+          <t>Bench measurement of clock edge rise time and slew, termination setup, report evidence, and comparator/buffer options to validate a 3 ns requirement.</t>
+        </is>
+      </c>
+      <c r="H818" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B819" s="3" t="inlineStr">
+        <is>
+          <t>Retrospective IEC 61010 Uplift</t>
+        </is>
+      </c>
+      <c r="C819" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D819" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03_0922_Retrospective-IEC-61010-Uplift.md</t>
+        </is>
+      </c>
+      <c r="E819" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F819" s="2" t="inlineStr"/>
+      <c r="G819" s="3" t="inlineStr">
+        <is>
+          <t>Planning a retrospective IEC 61010 technical file uplift for a radiation image-sensor test system, including document templates.</t>
+        </is>
+      </c>
+      <c r="H819" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B820" s="3" t="inlineStr">
+        <is>
+          <t>Document Tree Analysis</t>
+        </is>
+      </c>
+      <c r="C820" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D820" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06_1944_Document-Tree-Analysis.md</t>
+        </is>
+      </c>
+      <c r="E820" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F820" s="2" t="inlineStr"/>
+      <c r="G820" s="3" t="inlineStr">
+        <is>
+          <t>Restructuring the IEC 61010 compliance uplift job specification and combined source material into an execution manual.</t>
+        </is>
+      </c>
+      <c r="H820" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B821" s="3" t="inlineStr">
+        <is>
+          <t>Best App for Disk Images</t>
+        </is>
+      </c>
+      <c r="C821" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D821" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11_1931_Best-App-for-Disk-Images.md</t>
+        </is>
+      </c>
+      <c r="E821" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F821" s="2" t="inlineStr">
+        <is>
+          <t>borderline</t>
+        </is>
+      </c>
+      <c r="G821" s="3" t="inlineStr">
+        <is>
+          <t>Restoring software on a Tektronix oscilloscope from boot disk images; unclear whether this is work equipment.</t>
+        </is>
+      </c>
+      <c r="H821" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B822" s="3" t="inlineStr">
+        <is>
+          <t>Mitre Saw Blade Size</t>
+        </is>
+      </c>
+      <c r="C822" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D822" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-19_1209_Mitre-Saw-Blade-Size.md</t>
+        </is>
+      </c>
+      <c r="E822" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F822" s="2" t="inlineStr"/>
+      <c r="G822" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H822" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B823" s="3" t="inlineStr">
+        <is>
+          <t>Cement over Bostik Aquaprufe</t>
+        </is>
+      </c>
+      <c r="C823" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D823" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05_0616_Cement-over-Bostik-Aquaprufe.md</t>
+        </is>
+      </c>
+      <c r="E823" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F823" s="2" t="inlineStr"/>
+      <c r="G823" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H823" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B824" s="3" t="inlineStr">
+        <is>
+          <t>Broadfix Shim Feature</t>
+        </is>
+      </c>
+      <c r="C824" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D824" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06_0719_Broadfix-Shim-Feature.md</t>
+        </is>
+      </c>
+      <c r="E824" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F824" s="2" t="inlineStr"/>
+      <c r="G824" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H824" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B825" s="3" t="inlineStr">
+        <is>
+          <t>djay Pro 2 Crash</t>
+        </is>
+      </c>
+      <c r="C825" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D825" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06_1641_djay-Pro-2-Crash.md</t>
+        </is>
+      </c>
+      <c r="E825" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F825" s="2" t="inlineStr"/>
+      <c r="G825" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H825" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B826" s="3" t="inlineStr">
+        <is>
+          <t>Expanding Tape Recommendation</t>
+        </is>
+      </c>
+      <c r="C826" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D826" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13_0507_Expanding-Tape-Recommendation.md</t>
+        </is>
+      </c>
+      <c r="E826" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F826" s="2" t="inlineStr"/>
+      <c r="G826" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H826" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B827" s="3" t="inlineStr">
+        <is>
+          <t>Project Reflection Strategy</t>
+        </is>
+      </c>
+      <c r="C827" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D827" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13_2226_Project-Reflection-Strategy.md</t>
+        </is>
+      </c>
+      <c r="E827" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F827" s="2" t="inlineStr"/>
+      <c r="G827" s="3" t="inlineStr">
+        <is>
+          <t>Planning a structured reflection and evidence record of the owner's workplace history and concern about being pushed out at work.</t>
+        </is>
+      </c>
+      <c r="H827" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B828" s="3" t="inlineStr">
+        <is>
+          <t>Work History Recovery</t>
+        </is>
+      </c>
+      <c r="C828" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D828" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13_2233_Work-History-Recovery.md</t>
+        </is>
+      </c>
+      <c r="E828" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F828" s="2" t="inlineStr"/>
+      <c r="G828" s="3" t="inlineStr">
+        <is>
+          <t>Planning recovery of earlier chats about the owner's work situation to build a consolidated work-history and professional contribution record.</t>
+        </is>
+      </c>
+      <c r="H828" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B829" s="3" t="inlineStr">
+        <is>
+          <t>Max Voltage Inputs LM1086 MAX604</t>
+        </is>
+      </c>
+      <c r="C829" s="2" t="inlineStr">
+        <is>
+          <t>Conversations__7c20a96482f3aa11fccee3586429b7a503a5350734f19c55cb3e538cc195527e-chatgpt-0001-part-0001/conversations-008.json</t>
+        </is>
+      </c>
+      <c r="D829" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-17_1510_Max-Voltage-Inputs-LM1086-MAX604.md</t>
+        </is>
+      </c>
+      <c r="E829" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F829" s="2" t="inlineStr"/>
+      <c r="G829" s="3" t="inlineStr">
+        <is>
+          <t>No work-related content.</t>
+        </is>
+      </c>
+      <c r="H829" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H720"/>
+  <autoFilter ref="A1:H829"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -27228,7 +31280,7 @@
         </is>
       </c>
       <c r="B1" t="n">
-        <v>719</v>
+        <v>828</v>
       </c>
     </row>
     <row r="2">
@@ -27238,7 +31290,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>199</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3">
@@ -27248,7 +31300,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4">
@@ -27258,7 +31310,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>276</v>
+        <v>334</v>
       </c>
     </row>
     <row r="5">
@@ -27268,7 +31320,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>443</v>
+        <v>494</v>
       </c>
     </row>
     <row r="6">

</xml_diff>